<commit_message>
Update NURUL HIDAYATI, S.Pd., M.Psi Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H53"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,19 +442,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>NURUL HIDAYATI, S.Pd., M.Psi</v>
+        <v>Drs. MOEHAIMIN</v>
       </c>
       <c r="C2" t="str">
-        <v>197004301998022004</v>
+        <v>196709041997031005</v>
       </c>
       <c r="D2" t="str">
-        <v>X TEI 1</v>
+        <v>X TEI 2</v>
       </c>
       <c r="E2" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/UttCqb2kxt4LevCA8</v>
+        <v>https://forms.gle/ekQJWbDbi72DSNHX9</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,19 +468,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Drs. MOEHAIMIN</v>
+        <v>MUNASRI, S.Pd.</v>
       </c>
       <c r="C3" t="str">
-        <v>196709041997031005</v>
+        <v>197003282008012013</v>
       </c>
       <c r="D3" t="str">
-        <v>X TEI 2</v>
+        <v>X TPM 1</v>
       </c>
       <c r="E3" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/ekQJWbDbi72DSNHX9</v>
+        <v>https://forms.gle/FzjMqjr2bhYB4mFGA</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,19 +494,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>MUNASRI, S.Pd.</v>
+        <v>DWI RETNO TUGAS ERNAWATI, S.Pd</v>
       </c>
       <c r="C4" t="str">
-        <v>197003282008012013</v>
+        <v>196702142008012009</v>
       </c>
       <c r="D4" t="str">
-        <v>X TPM 1</v>
+        <v>X TKR1</v>
       </c>
       <c r="E4" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/FzjMqjr2bhYB4mFGA</v>
+        <v>https://forms.gle/hpaJmjc4TSuY21187</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,19 +520,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>DWI RETNO TUGAS ERNAWATI, S.Pd</v>
+        <v>KASIATIN, S.Pd</v>
       </c>
       <c r="C5" t="str">
-        <v>196702142008012009</v>
+        <v>196908112007012019</v>
       </c>
       <c r="D5" t="str">
-        <v>X TKR1</v>
+        <v>X TKR2</v>
       </c>
       <c r="E5" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/hpaJmjc4TSuY21187</v>
+        <v>https://forms.gle/zCXw2UY7hgtbguuc6</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,19 +546,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>KASIATIN, S.Pd</v>
+        <v>SUHARTO DWI SUHERNOWO, ST</v>
       </c>
       <c r="C6" t="str">
-        <v>196908112007012019</v>
+        <v>197803262009011007</v>
       </c>
       <c r="D6" t="str">
-        <v>X TKR2</v>
+        <v>X TBKR</v>
       </c>
       <c r="E6" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/zCXw2UY7hgtbguuc6</v>
+        <v>https://forms.gle/8SMDhw8YpsNPPHPK7</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,19 +572,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>SUHARTO DWI SUHERNOWO, ST</v>
+        <v>ARSYL NOVA ARIRI, ST, M.Pd.</v>
       </c>
       <c r="C7" t="str">
-        <v>197803262009011007</v>
+        <v>197811142009012007</v>
       </c>
       <c r="D7" t="str">
-        <v>X TBKR</v>
+        <v>X TSM 1</v>
       </c>
       <c r="E7" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/8SMDhw8YpsNPPHPK7</v>
+        <v>https://forms.gle/sZ2Rff4sL9N4FTrh9</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,19 +598,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>ARSYL NOVA ARIRI, ST, M.Pd.</v>
+        <v>WAWAN SISWANTO, SS</v>
       </c>
       <c r="C8" t="str">
-        <v>197811142009012007</v>
+        <v>196904012007011025</v>
       </c>
       <c r="D8" t="str">
-        <v>X TSM 1</v>
+        <v>XI TAV</v>
       </c>
       <c r="E8" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/sZ2Rff4sL9N4FTrh9</v>
+        <v>https://forms.gle/ghNaoJYp7o2SbkjS8</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,19 +624,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>WAWAN SISWANTO, SS</v>
+        <v>R.A. RATNA KARTIKAWATI, S.Pd</v>
       </c>
       <c r="C9" t="str">
-        <v>196904012007011025</v>
+        <v>196905132008012023</v>
       </c>
       <c r="D9" t="str">
-        <v>XI TAV</v>
+        <v>XI TEI 1</v>
       </c>
       <c r="E9" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/ghNaoJYp7o2SbkjS8</v>
+        <v>https://forms.gle/bPxWzjgFDES2StGo6</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,19 +650,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>R.A. RATNA KARTIKAWATI, S.Pd</v>
+        <v>NURUL HUDA, ST, M.Si.</v>
       </c>
       <c r="C10" t="str">
-        <v>196905132008012023</v>
+        <v>197102162008011009</v>
       </c>
       <c r="D10" t="str">
-        <v>XI TEI 1</v>
+        <v>XI TPL 1</v>
       </c>
       <c r="E10" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/bPxWzjgFDES2StGo6</v>
+        <v>https://forms.gle/aaS7YNQQ97713C18A</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,19 +676,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>NURUL HUDA, ST, M.Si.</v>
+        <v>NUR 'AFIIFAH, M.Pd.</v>
       </c>
       <c r="C11" t="str">
-        <v>197102162008011009</v>
+        <v>197208052007012020</v>
       </c>
       <c r="D11" t="str">
-        <v>XI TPL 1</v>
+        <v>XI TPL 2</v>
       </c>
       <c r="E11" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/aaS7YNQQ97713C18A</v>
+        <v>https://forms.gle/6YPzECievjrGJZBnA</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,19 +702,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>NUR 'AFIIFAH, M.Pd.</v>
+        <v>TRIBUDI HARTONO, S.Pd</v>
       </c>
       <c r="C12" t="str">
-        <v>197208052007012020</v>
+        <v>197511052003121004</v>
       </c>
       <c r="D12" t="str">
-        <v>XI TPL 2</v>
+        <v>XI TPM 1</v>
       </c>
       <c r="E12" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/6YPzECievjrGJZBnA</v>
+        <v>https://forms.gle/2mog9vghqCw6TSTw7</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,19 +728,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>TRIBUDI HARTONO, S.Pd</v>
+        <v>SAMSUL HADI, M.Pd.</v>
       </c>
       <c r="C13" t="str">
-        <v>197511052003121004</v>
+        <v>197509262008011011</v>
       </c>
       <c r="D13" t="str">
-        <v>XI TPM 1</v>
+        <v>XI TKR2</v>
       </c>
       <c r="E13" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/2mog9vghqCw6TSTw7</v>
+        <v>https://forms.gle/DSDoMKgI8XxbcPr78</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,19 +754,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>SAMSUL HADI, M.Pd.</v>
+        <v>HISBULLOH HUDA, M.Pd.</v>
       </c>
       <c r="C14" t="str">
-        <v>197509262008011011</v>
+        <v>197602072010011006</v>
       </c>
       <c r="D14" t="str">
-        <v>XI TKR2</v>
+        <v>XI TBKR</v>
       </c>
       <c r="E14" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/DSDoMKgI8XxbcPr78</v>
+        <v>https://forms.gle/jVwhLYXebas1GSZQJ6</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,19 +780,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>HISBULLOH HUDA, M.Pd.</v>
+        <v>AGUS HARIYANTO, ST. M.Pd</v>
       </c>
       <c r="C15" t="str">
-        <v>197602072010011006</v>
+        <v>198010032010011010</v>
       </c>
       <c r="D15" t="str">
-        <v>XI TBKR</v>
+        <v>XI TSM 2</v>
       </c>
       <c r="E15" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/jVwhLYXebas1GSZQJ6</v>
+        <v>https://forms.gle/r3mekFxufrTcJjgRA</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,19 +806,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>AGUS HARIYANTO, ST. M.Pd</v>
+        <v>SIGIT EKO PRAMONO, S.Pd</v>
       </c>
       <c r="C16" t="str">
-        <v>198010032010011010</v>
+        <v>198301122009011006</v>
       </c>
       <c r="D16" t="str">
-        <v>XI TSM 2</v>
+        <v>XII TAV</v>
       </c>
       <c r="E16" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/r3mekFxufrTcJjgRA</v>
+        <v>https://forms.gle/PSXtPwi7yQN3Mfi8</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,19 +832,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>SIGIT EKO PRAMONO, S.Pd</v>
+        <v>MOHAMAD ARIEF PRIYO UTOMO, S.Pd</v>
       </c>
       <c r="C17" t="str">
-        <v>198301122009011006</v>
+        <v>198209292010011011</v>
       </c>
       <c r="D17" t="str">
-        <v>XII TAV</v>
+        <v>XII TPL 1</v>
       </c>
       <c r="E17" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/PSXtPwi7yQN3Mfi8</v>
+        <v>https://forms.gle/ESlazXu6aQ3PklsD9</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,19 +858,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>MOHAMAD ARIEF PRIYO UTOMO, S.Pd</v>
+        <v>Dr. RIRIN DIYANNITA SASANTI, M.Pd.</v>
       </c>
       <c r="C18" t="str">
-        <v>198209292010011011</v>
+        <v>198212022014062003</v>
       </c>
       <c r="D18" t="str">
-        <v>XII TPL 1</v>
+        <v>XII TPL 2</v>
       </c>
       <c r="E18" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/ESlazXu6aQ3PklsD9</v>
+        <v>https://forms.gle/KwfitQjMYbtsnr4UZV6</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,19 +884,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>Dr. RIRIN DIYANNITA SASANTI, M.Pd.</v>
+        <v>SULIADI, S.Pd</v>
       </c>
       <c r="C19" t="str">
-        <v>198212022014062003</v>
+        <v>198403262010011008</v>
       </c>
       <c r="D19" t="str">
-        <v>XII TPL 2</v>
+        <v>XII TPM 1</v>
       </c>
       <c r="E19" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/KwfitQjMYbtsnr4UZV6</v>
+        <v>https://forms.gle/DStwfQQGe3W3gc73A</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,19 +910,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>SULIADI, S.Pd</v>
+        <v>TUTIK QOMARIYAH, S.Si</v>
       </c>
       <c r="C20" t="str">
-        <v>198403262010011008</v>
+        <v>198504032010012014</v>
       </c>
       <c r="D20" t="str">
-        <v>XII TPM 1</v>
+        <v>XII TPM 2</v>
       </c>
       <c r="E20" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/DStwfQQGe3W3gc73A</v>
+        <v>https://forms.gle/8Z33XXUnWmhZCY9S9</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,19 +936,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>TUTIK QOMARIYAH, S.Si</v>
+        <v>FIRMAN ARDIANSYAH, S.Pd.</v>
       </c>
       <c r="C21" t="str">
-        <v>198504032010012014</v>
+        <v>198706172011011010</v>
       </c>
       <c r="D21" t="str">
-        <v>XII TPM 2</v>
+        <v>XII TKR2</v>
       </c>
       <c r="E21" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/8Z33XXUnWmhZCY9S9</v>
+        <v>https://forms.gle/iGQNqJij1huPUYbk8</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,19 +962,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>FIRMAN ARDIANSYAH, S.Pd.</v>
+        <v>AZIZ CAHYA PRADANA, S.Pd.</v>
       </c>
       <c r="C22" t="str">
-        <v>198706172011011010</v>
+        <v>199103072019031014</v>
       </c>
       <c r="D22" t="str">
-        <v>XII TKR2</v>
+        <v>XII TBKR</v>
       </c>
       <c r="E22" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/iGQNqJij1huPUYbk8</v>
+        <v>https://forms.gle/RvBNnww2vjNe3gNo76</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -988,19 +988,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>AZIZ CAHYA PRADANA, S.Pd.</v>
+        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
       </c>
       <c r="C23" t="str">
-        <v>199103072019031014</v>
+        <v>199311072019031004</v>
       </c>
       <c r="D23" t="str">
-        <v>XII TBKR</v>
+        <v>XII TSM 1</v>
       </c>
       <c r="E23" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F23" t="str">
-        <v>https://forms.gle/RvBNnww2vjNe3gNo76</v>
+        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
       </c>
       <c r="G23" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1014,19 +1014,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
+        <v>EFRIDA ISBANDRIYAH, S.T.</v>
       </c>
       <c r="C24" t="str">
-        <v>199311072019031004</v>
+        <v>199511062019032010</v>
       </c>
       <c r="D24" t="str">
-        <v>XII TSM 1</v>
+        <v>XII DKV 1</v>
       </c>
       <c r="E24" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F24" t="str">
-        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
+        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
       </c>
       <c r="G24" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1040,19 +1040,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>EFRIDA ISBANDRIYAH, S.T.</v>
+        <v>ETIK SULISTYOWATI, S.Pd.</v>
       </c>
       <c r="C25" t="str">
-        <v>199511062019032010</v>
+        <v>198304282022212026</v>
       </c>
       <c r="D25" t="str">
-        <v>XII DKV 1</v>
+        <v>-</v>
       </c>
       <c r="E25" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F25" t="str">
-        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
+        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
       </c>
       <c r="G25" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1066,10 +1066,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>ETIK SULISTYOWATI, S.Pd.</v>
+        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
       </c>
       <c r="C26" t="str">
-        <v>198304282022212026</v>
+        <v>198404192022211018</v>
       </c>
       <c r="D26" t="str">
         <v>-</v>
@@ -1078,7 +1078,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F26" t="str">
-        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
+        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
       </c>
       <c r="G26" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1092,10 +1092,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
+        <v>YAYUK NURNANINGSIH, S.Pd</v>
       </c>
       <c r="C27" t="str">
-        <v>198404192022211018</v>
+        <v>198607052022212052</v>
       </c>
       <c r="D27" t="str">
         <v>-</v>
@@ -1104,7 +1104,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F27" t="str">
-        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
+        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
       </c>
       <c r="G27" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1118,10 +1118,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>YAYUK NURNANINGSIH, S.Pd</v>
+        <v>KHOIRUZEN, ST</v>
       </c>
       <c r="C28" t="str">
-        <v>198607052022212052</v>
+        <v>197107222023211002</v>
       </c>
       <c r="D28" t="str">
         <v>-</v>
@@ -1130,7 +1130,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F28" t="str">
-        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
+        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
       </c>
       <c r="G28" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1144,10 +1144,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>KHOIRUZEN, ST</v>
+        <v>DARIS UMAMI, S.Pd.</v>
       </c>
       <c r="C29" t="str">
-        <v>197107222023211002</v>
+        <v>198205042023212026</v>
       </c>
       <c r="D29" t="str">
         <v>-</v>
@@ -1156,7 +1156,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F29" t="str">
-        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
+        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
       </c>
       <c r="G29" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1170,10 +1170,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>DARIS UMAMI, S.Pd.</v>
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
       </c>
       <c r="C30" t="str">
-        <v>198205042023212026</v>
+        <v>198808072023211018</v>
       </c>
       <c r="D30" t="str">
         <v>-</v>
@@ -1182,7 +1182,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F30" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
       </c>
       <c r="G30" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1196,10 +1196,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
       </c>
       <c r="C31" t="str">
-        <v>198808072023211018</v>
+        <v>199606142023212026</v>
       </c>
       <c r="D31" t="str">
         <v>-</v>
@@ -1208,7 +1208,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F31" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
       </c>
       <c r="G31" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1222,10 +1222,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C32" t="str">
-        <v>199606142023212026</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D32" t="str">
         <v>-</v>
@@ -1234,7 +1234,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F32" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="G32" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1248,10 +1248,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C33" t="str">
-        <v>197206202024211005</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D33" t="str">
         <v>-</v>
@@ -1260,7 +1260,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F33" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G33" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1274,10 +1274,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C34" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D34" t="str">
         <v>-</v>
@@ -1286,7 +1286,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F34" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G34" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1300,10 +1300,10 @@
         <v>34</v>
       </c>
       <c r="B35" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C35" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D35" t="str">
         <v>-</v>
@@ -1312,7 +1312,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F35" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G35" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1326,10 +1326,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C36" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D36" t="str">
         <v>-</v>
@@ -1338,7 +1338,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F36" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G36" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1352,10 +1352,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C37" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D37" t="str">
         <v>-</v>
@@ -1364,7 +1364,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F37" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G37" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1378,10 +1378,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C38" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D38" t="str">
         <v>-</v>
@@ -1390,7 +1390,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F38" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G38" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1404,10 +1404,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C39" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D39" t="str">
         <v>-</v>
@@ -1416,7 +1416,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F39" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G39" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1430,10 +1430,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C40" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D40" t="str">
         <v>-</v>
@@ -1442,7 +1442,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F40" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G40" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1456,10 +1456,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C41" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D41" t="str">
         <v>-</v>
@@ -1468,7 +1468,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F41" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G41" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1482,7 +1482,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C42" t="str">
         <v>-</v>
@@ -1494,7 +1494,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F42" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G42" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1508,7 +1508,7 @@
         <v>42</v>
       </c>
       <c r="B43" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C43" t="str">
         <v>-</v>
@@ -1520,7 +1520,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F43" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G43" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1534,7 +1534,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C44" t="str">
         <v>-</v>
@@ -1546,7 +1546,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F44" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G44" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1560,7 +1560,7 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C45" t="str">
         <v>-</v>
@@ -1572,7 +1572,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F45" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G45" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1586,7 +1586,7 @@
         <v>45</v>
       </c>
       <c r="B46" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C46" t="str">
         <v>-</v>
@@ -1598,7 +1598,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F46" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G46" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1612,7 +1612,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C47" t="str">
         <v>-</v>
@@ -1624,7 +1624,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F47" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G47" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1638,7 +1638,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C48" t="str">
         <v>-</v>
@@ -1650,7 +1650,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F48" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G48" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1664,7 +1664,7 @@
         <v>48</v>
       </c>
       <c r="B49" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C49" t="str">
         <v>-</v>
@@ -1676,7 +1676,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F49" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G49" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1690,7 +1690,7 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C50" t="str">
         <v>-</v>
@@ -1702,7 +1702,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F50" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G50" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1716,7 +1716,7 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C51" t="str">
         <v>-</v>
@@ -1728,7 +1728,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F51" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G51" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1742,7 +1742,7 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C52" t="str">
         <v>-</v>
@@ -1754,7 +1754,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F52" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G52" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1768,7 +1768,7 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C53" t="str">
         <v>-</v>
@@ -1780,7 +1780,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F53" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G53" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1789,42 +1789,16 @@
         <v/>
       </c>
     </row>
-    <row r="54">
-      <c r="A54">
-        <v>53</v>
-      </c>
-      <c r="B54" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C54" t="str">
-        <v>-</v>
-      </c>
-      <c r="D54" t="str">
-        <v>-</v>
-      </c>
-      <c r="E54" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F54" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G54" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H54" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H53"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -1886,19 +1860,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>DHURROTUL FARIDAH, S.Pd</v>
+        <v>NURUL HIDAYATI, S.Pd., M.Psi</v>
       </c>
       <c r="C3" t="str">
-        <v>196707142006042005</v>
+        <v>197004301998022004</v>
       </c>
       <c r="D3" t="str">
-        <v>X TPL 1</v>
+        <v>X TEI 1</v>
       </c>
       <c r="E3" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F3" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeMVWzzDZ53AHLlhGUhchbGtjSPh774mpA2M0nanLr8yfuENQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeN20MexbrBL34C2Q686_fkiIwRRd1p8MlfQmirZxcd7z32gA/viewform</v>
       </c>
       <c r="G3" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1909,19 +1883,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>SRI WINARTI, S.Pd</v>
+        <v>DHURROTUL FARIDAH, S.Pd</v>
       </c>
       <c r="C4" t="str">
-        <v>197307112007012008</v>
+        <v>196707142006042005</v>
       </c>
       <c r="D4" t="str">
-        <v>X TPL 2</v>
+        <v>X TPL 1</v>
       </c>
       <c r="E4" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F4" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeDax_Aw_bF0ozmHf2395mK0_9K9QaIgPxKL3Msw8FyZrsKJw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeMVWzzDZ53AHLlhGUhchbGtjSPh774mpA2M0nanLr8yfuENQ/viewform</v>
       </c>
       <c r="G4" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1932,19 +1906,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>NUR HAYATI, S.Psi, M.Pd.</v>
+        <v>SRI WINARTI, S.Pd</v>
       </c>
       <c r="C5" t="str">
-        <v>197310152009012003</v>
+        <v>197307112007012008</v>
       </c>
       <c r="D5" t="str">
-        <v>X TPM 2</v>
+        <v>X TPL 2</v>
       </c>
       <c r="E5" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F5" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeD8S_m6otgqVphxM7Ux4fGC0wrPh7aPQIKMKg_uaW5tKl42w/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeDax_Aw_bF0ozmHf2395mK0_9K9QaIgPxKL3Msw8FyZrsKJw/viewform</v>
       </c>
       <c r="G5" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1955,19 +1929,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>LAILA FITRIYA, S.Pd.I</v>
+        <v>NUR HAYATI, S.Psi, M.Pd.</v>
       </c>
       <c r="C6" t="str">
-        <v>198506172009012006</v>
+        <v>197310152009012003</v>
       </c>
       <c r="D6" t="str">
-        <v>X TSM 2</v>
+        <v>X TPM 2</v>
       </c>
       <c r="E6" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F6" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfLY_MCLONnsdcq8EWaQayXJZ8_9cAWE7IYKvdeEhm2S0GL9A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeD8S_m6otgqVphxM7Ux4fGC0wrPh7aPQIKMKg_uaW5tKl42w/viewform</v>
       </c>
       <c r="G6" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1978,19 +1952,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>EKA PRAMITASARI, S.Pd. M.Pd.</v>
+        <v>LAILA FITRIYA, S.Pd.I</v>
       </c>
       <c r="C7" t="str">
-        <v>198710302010012005</v>
+        <v>198506172009012006</v>
       </c>
       <c r="D7" t="str">
-        <v>X DKV 1</v>
+        <v>X TSM 2</v>
       </c>
       <c r="E7" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F7" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFNOjWRONIbFscUAVy_gPYaD8c1ehSpS2dTykzwJAn_RUDGw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfLY_MCLONnsdcq8EWaQayXJZ8_9cAWE7IYKvdeEhm2S0GL9A/viewform</v>
       </c>
       <c r="G7" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2001,19 +1975,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>MISBAHUR ROSYIDIN, S.Pd.</v>
+        <v>EKA PRAMITASARI, S.Pd. M.Pd.</v>
       </c>
       <c r="C8" t="str">
-        <v>196802112008011008</v>
+        <v>198710302010012005</v>
       </c>
       <c r="D8" t="str">
-        <v>X DKV 2</v>
+        <v>X DKV 1</v>
       </c>
       <c r="E8" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F8" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe7MHsr1k2S6apY2TP7L_VulJ7MaQqcKaEsASfOrFV2WfDKSw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFNOjWRONIbFscUAVy_gPYaD8c1ehSpS2dTykzwJAn_RUDGw/viewform</v>
       </c>
       <c r="G8" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2024,19 +1998,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>Dra. DYAH CHUSNUL CHOTIMAH</v>
+        <v>MISBAHUR ROSYIDIN, S.Pd.</v>
       </c>
       <c r="C9" t="str">
-        <v>196802142007012016</v>
+        <v>196802112008011008</v>
       </c>
       <c r="D9" t="str">
-        <v>X DKV 3</v>
+        <v>X DKV 2</v>
       </c>
       <c r="E9" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F9" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScl7wa5Pd4jitd3sxqnpqk8tlBpTw-Bx1jl50JwfjGXK_v6ZQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe7MHsr1k2S6apY2TP7L_VulJ7MaQqcKaEsASfOrFV2WfDKSw/viewform</v>
       </c>
       <c r="G9" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2047,19 +2021,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>HERI SUBYANTORO, ST, M.Pd.</v>
+        <v>Dra. DYAH CHUSNUL CHOTIMAH</v>
       </c>
       <c r="C10" t="str">
-        <v>196910102008011021</v>
+        <v>196802142007012016</v>
       </c>
       <c r="D10" t="str">
-        <v>XI TEI 2</v>
+        <v>X DKV 3</v>
       </c>
       <c r="E10" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F10" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdHmC5tO01PGYfeU-it6vioHYot6MO4Enq9Nbw1oA8DLgGJog/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScl7wa5Pd4jitd3sxqnpqk8tlBpTw-Bx1jl50JwfjGXK_v6ZQ/viewform</v>
       </c>
       <c r="G10" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2070,19 +2044,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>DEDY HENDRIANA, S.Pd. M.Pd.</v>
+        <v>HERI SUBYANTORO, ST, M.Pd.</v>
       </c>
       <c r="C11" t="str">
-        <v>197904072010011002</v>
+        <v>196910102008011021</v>
       </c>
       <c r="D11" t="str">
-        <v>XI TPM 2</v>
+        <v>XI TEI 2</v>
       </c>
       <c r="E11" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F11" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSecBLlEDfTwutpIfoRhoxlk9TykVgqtywzFBczl8dG7w3nLgg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdHmC5tO01PGYfeU-it6vioHYot6MO4Enq9Nbw1oA8DLgGJog/viewform</v>
       </c>
       <c r="G11" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2093,19 +2067,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>AGUS HIDAYAT, S.Pd</v>
+        <v>DEDY HENDRIANA, S.Pd. M.Pd.</v>
       </c>
       <c r="C12" t="str">
-        <v>196907272007011018</v>
+        <v>197904072010011002</v>
       </c>
       <c r="D12" t="str">
-        <v>XI TKR1</v>
+        <v>XI TPM 2</v>
       </c>
       <c r="E12" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F12" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4cLrLtqJrSQCZlTZvjVDTqCqwr0Ezvo9jj1xlEEVIA1TgLQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSecBLlEDfTwutpIfoRhoxlk9TykVgqtywzFBczl8dG7w3nLgg/viewform</v>
       </c>
       <c r="G12" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2116,19 +2090,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>DWI SANTOSO, S.Pd</v>
+        <v>AGUS HIDAYAT, S.Pd</v>
       </c>
       <c r="C13" t="str">
-        <v>197908082006041019</v>
+        <v>196907272007011018</v>
       </c>
       <c r="D13" t="str">
-        <v>XI TSM 1</v>
+        <v>XI TKR1</v>
       </c>
       <c r="E13" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F13" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc3pPlG2fg8z9mrKutplhHQxr-oLEDr0OrG2tbckE403avEiw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4cLrLtqJrSQCZlTZvjVDTqCqwr0Ezvo9jj1xlEEVIA1TgLQ/viewform</v>
       </c>
       <c r="G13" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2139,19 +2113,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>ZAINUL ARIFIN, M.Pd.</v>
+        <v>DWI SANTOSO, S.Pd</v>
       </c>
       <c r="C14" t="str">
-        <v>198210112010011009</v>
+        <v>197908082006041019</v>
       </c>
       <c r="D14" t="str">
-        <v>XI DKV 1</v>
+        <v>XI TSM 1</v>
       </c>
       <c r="E14" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F14" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc1knrp09uNEhFpIHg2HnTVcw1HE0-aoR7bacYb4cXIsHAleQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc3pPlG2fg8z9mrKutplhHQxr-oLEDr0OrG2tbckE403avEiw/viewform</v>
       </c>
       <c r="G14" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2162,19 +2136,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>BAMBANG SUJATMIKO, S.Pd</v>
+        <v>ZAINUL ARIFIN, M.Pd.</v>
       </c>
       <c r="C15" t="str">
-        <v>198211222006041009</v>
+        <v>198210112010011009</v>
       </c>
       <c r="D15" t="str">
-        <v>XI DKV 2</v>
+        <v>XI DKV 1</v>
       </c>
       <c r="E15" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F15" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYyOzS9TUnTH79m-niYDGHWqxmhbtWyxFehMM6Td06hqBh1A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc1knrp09uNEhFpIHg2HnTVcw1HE0-aoR7bacYb4cXIsHAleQ/viewform</v>
       </c>
       <c r="G15" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2185,19 +2159,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>HARTONO, S.Pd</v>
+        <v>BAMBANG SUJATMIKO, S.Pd</v>
       </c>
       <c r="C16" t="str">
-        <v>198205122009011009</v>
+        <v>198211222006041009</v>
       </c>
       <c r="D16" t="str">
-        <v>XI DKV 3</v>
+        <v>XI DKV 2</v>
       </c>
       <c r="E16" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F16" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSczcB1-HoNbq4XLNVL6d22ps_sHXrr_yAMrTdi-SXUI9dyDiA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYyOzS9TUnTH79m-niYDGHWqxmhbtWyxFehMM6Td06hqBh1A/viewform</v>
       </c>
       <c r="G16" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2208,19 +2182,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>AGUNG RAKHMANDA, S.Kom.</v>
+        <v>HARTONO, S.Pd</v>
       </c>
       <c r="C17" t="str">
-        <v>198303272009031002</v>
+        <v>198205122009011009</v>
       </c>
       <c r="D17" t="str">
-        <v>XII TEI 1</v>
+        <v>XI DKV 3</v>
       </c>
       <c r="E17" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F17" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe3WNA-vHAA16POkCpcvBUl2Kc57HtjVXCkAQEm_mMB69NPow/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSczcB1-HoNbq4XLNVL6d22ps_sHXrr_yAMrTdi-SXUI9dyDiA/viewform</v>
       </c>
       <c r="G17" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2231,19 +2205,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>IMAM SUFERI, ST.</v>
+        <v>AGUNG RAKHMANDA, S.Kom.</v>
       </c>
       <c r="C18" t="str">
-        <v>197712302008011013</v>
+        <v>198303272009031002</v>
       </c>
       <c r="D18" t="str">
-        <v>XII TKR1</v>
+        <v>XII TEI 1</v>
       </c>
       <c r="E18" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F18" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe8sSOVeefXvVkHVMUzrTdYO8RrfqdFwT5AQRWWlJ3ZzJAluQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe3WNA-vHAA16POkCpcvBUl2Kc57HtjVXCkAQEm_mMB69NPow/viewform</v>
       </c>
       <c r="G18" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2254,19 +2228,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
+        <v>IMAM SUFERI, ST.</v>
       </c>
       <c r="C19" t="str">
-        <v>199410092019032012</v>
+        <v>197712302008011013</v>
       </c>
       <c r="D19" t="str">
-        <v>XII TSM 2</v>
+        <v>XII TKR1</v>
       </c>
       <c r="E19" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F19" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe8sSOVeefXvVkHVMUzrTdYO8RrfqdFwT5AQRWWlJ3ZzJAluQ/viewform</v>
       </c>
       <c r="G19" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2277,19 +2251,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>SOTYA BAYUNTARA, S.Pd.</v>
+        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
       </c>
       <c r="C20" t="str">
-        <v>196906252022211004</v>
+        <v>199410092019032012</v>
       </c>
       <c r="D20" t="str">
-        <v>XII DKV 2</v>
+        <v>XII TSM 2</v>
       </c>
       <c r="E20" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F20" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
       </c>
       <c r="G20" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2300,19 +2274,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>SRIGATI, SE</v>
+        <v>SOTYA BAYUNTARA, S.Pd.</v>
       </c>
       <c r="C21" t="str">
-        <v>197505052022212013</v>
+        <v>196906252022211004</v>
       </c>
       <c r="D21" t="str">
-        <v>XII DKV 3</v>
+        <v>XII DKV 2</v>
       </c>
       <c r="E21" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F21" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
       </c>
       <c r="G21" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2323,19 +2297,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>HARI PURWANTO, ST</v>
+        <v>SRIGATI, SE</v>
       </c>
       <c r="C22" t="str">
-        <v>197711242022211006</v>
+        <v>197505052022212013</v>
       </c>
       <c r="D22" t="str">
-        <v>-</v>
+        <v>XII DKV 3</v>
       </c>
       <c r="E22" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F22" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
       </c>
       <c r="G22" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2346,10 +2320,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>ESTI WIDHIARNI, S.T</v>
+        <v>HARI PURWANTO, ST</v>
       </c>
       <c r="C23" t="str">
-        <v>197906032022212022</v>
+        <v>197711242022211006</v>
       </c>
       <c r="D23" t="str">
         <v>-</v>
@@ -2358,7 +2332,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F23" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
       </c>
       <c r="G23" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2369,19 +2343,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
+        <v>ESTI WIDHIARNI, S.T</v>
       </c>
       <c r="C24" t="str">
-        <v>198109092022211004</v>
+        <v>197906032022212022</v>
       </c>
       <c r="D24" t="str">
-        <v>XII TEI 2</v>
+        <v>-</v>
       </c>
       <c r="E24" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F24" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
       </c>
       <c r="G24" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2392,19 +2366,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
+        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
       </c>
       <c r="C25" t="str">
-        <v>198212102022211017</v>
+        <v>198109092022211004</v>
       </c>
       <c r="D25" t="str">
-        <v>-</v>
+        <v>XII TEI 2</v>
       </c>
       <c r="E25" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F25" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
       </c>
       <c r="G25" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2415,10 +2389,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>KHOIRUL AMIN, S.Pd</v>
+        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
       </c>
       <c r="C26" t="str">
-        <v>198701192022211009</v>
+        <v>198212102022211017</v>
       </c>
       <c r="D26" t="str">
         <v>-</v>
@@ -2427,7 +2401,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F26" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
       </c>
       <c r="G26" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2438,10 +2412,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
+        <v>KHOIRUL AMIN, S.Pd</v>
       </c>
       <c r="C27" t="str">
-        <v>198712072022211015</v>
+        <v>198701192022211009</v>
       </c>
       <c r="D27" t="str">
         <v>-</v>
@@ -2450,7 +2424,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F27" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
       </c>
       <c r="G27" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2461,10 +2435,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>HEPPY LUCKITO, SST</v>
+        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
       </c>
       <c r="C28" t="str">
-        <v>198110272023211008</v>
+        <v>198712072022211015</v>
       </c>
       <c r="D28" t="str">
         <v>-</v>
@@ -2473,7 +2447,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F28" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
       </c>
       <c r="G28" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2484,10 +2458,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>SRI PURWANINGSIH, S.Pd</v>
+        <v>HEPPY LUCKITO, SST</v>
       </c>
       <c r="C29" t="str">
-        <v>198203022023212020</v>
+        <v>198110272023211008</v>
       </c>
       <c r="D29" t="str">
         <v>-</v>
@@ -2496,7 +2470,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F29" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
       </c>
       <c r="G29" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2507,10 +2481,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+        <v>SRI PURWANINGSIH, S.Pd</v>
       </c>
       <c r="C30" t="str">
-        <v>199410282023211012</v>
+        <v>198203022023212020</v>
       </c>
       <c r="D30" t="str">
         <v>-</v>
@@ -2519,7 +2493,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F30" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
       </c>
       <c r="G30" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2530,10 +2504,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
       </c>
       <c r="C31" t="str">
-        <v>197509042024211002</v>
+        <v>199410282023211012</v>
       </c>
       <c r="D31" t="str">
         <v>-</v>
@@ -2542,7 +2516,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F31" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
       </c>
       <c r="G31" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2553,10 +2527,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="C32" t="str">
-        <v>198103052024211008</v>
+        <v>197509042024211002</v>
       </c>
       <c r="D32" t="str">
         <v>-</v>
@@ -2565,7 +2539,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F32" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="G32" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2576,10 +2550,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C33" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D33" t="str">
         <v>-</v>
@@ -2588,7 +2562,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F33" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G33" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2599,10 +2573,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C34" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D34" t="str">
         <v>-</v>
@@ -2611,7 +2585,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F34" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G34" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2622,10 +2596,10 @@
         <v>34</v>
       </c>
       <c r="B35" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C35" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D35" t="str">
         <v>-</v>
@@ -2634,7 +2608,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F35" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G35" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2645,10 +2619,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C36" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D36" t="str">
         <v>-</v>
@@ -2657,7 +2631,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F36" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G36" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2668,7 +2642,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C37" t="str">
         <v>-</v>
@@ -2680,7 +2654,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F37" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G37" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2691,7 +2665,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C38" t="str">
         <v>-</v>
@@ -2703,7 +2677,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F38" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G38" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2714,7 +2688,7 @@
         <v>38</v>
       </c>
       <c r="B39" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C39" t="str">
         <v>-</v>
@@ -2726,7 +2700,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F39" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G39" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2737,7 +2711,7 @@
         <v>39</v>
       </c>
       <c r="B40" t="str">
-        <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
+        <v>NUR KHOLIFAH, S.Pd.</v>
       </c>
       <c r="C40" t="str">
         <v>-</v>
@@ -2749,15 +2723,38 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F40" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
       </c>
       <c r="G40" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="str">
+        <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
+      </c>
+      <c r="C41" t="str">
+        <v>-</v>
+      </c>
+      <c r="D41" t="str">
+        <v>-</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F41" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
+      </c>
+      <c r="G41" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G41"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2845,13 +2842,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/UttCqb2kxt4LevCA8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeN20MexbrBL34C2Q686_fkiIwRRd1p8MlfQmirZxcd7z32gA/viewform</v>
       </c>
       <c r="G3" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H3" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Update TUTIK QOMARIYAH, S.Si Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="54 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="38 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="33 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="59 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H34"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,19 +442,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Drs. MOEHAIMIN</v>
+        <v>FIRMAN ARDIANSYAH, S.Pd.</v>
       </c>
       <c r="C2" t="str">
-        <v>196709041997031005</v>
+        <v>198706172011011010</v>
       </c>
       <c r="D2" t="str">
-        <v>X TEI 2</v>
+        <v>XII TKR2</v>
       </c>
       <c r="E2" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/ekQJWbDbi72DSNHX9</v>
+        <v>https://forms.gle/iGQNqJij1huPUYbk8</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,19 +468,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>MUNASRI, S.Pd.</v>
+        <v>AZIZ CAHYA PRADANA, S.Pd.</v>
       </c>
       <c r="C3" t="str">
-        <v>197003282008012013</v>
+        <v>199103072019031014</v>
       </c>
       <c r="D3" t="str">
-        <v>X TPM 1</v>
+        <v>XII TBKR</v>
       </c>
       <c r="E3" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/FzjMqjr2bhYB4mFGA</v>
+        <v>https://forms.gle/RvBNnww2vjNe3gNo76</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,19 +494,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>DWI RETNO TUGAS ERNAWATI, S.Pd</v>
+        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
       </c>
       <c r="C4" t="str">
-        <v>196702142008012009</v>
+        <v>199311072019031004</v>
       </c>
       <c r="D4" t="str">
-        <v>X TKR1</v>
+        <v>XII TSM 1</v>
       </c>
       <c r="E4" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/hpaJmjc4TSuY21187</v>
+        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,19 +520,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>KASIATIN, S.Pd</v>
+        <v>EFRIDA ISBANDRIYAH, S.T.</v>
       </c>
       <c r="C5" t="str">
-        <v>196908112007012019</v>
+        <v>199511062019032010</v>
       </c>
       <c r="D5" t="str">
-        <v>X TKR2</v>
+        <v>XII DKV 1</v>
       </c>
       <c r="E5" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/zCXw2UY7hgtbguuc6</v>
+        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,19 +546,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>SUHARTO DWI SUHERNOWO, ST</v>
+        <v>ETIK SULISTYOWATI, S.Pd.</v>
       </c>
       <c r="C6" t="str">
-        <v>197803262009011007</v>
+        <v>198304282022212026</v>
       </c>
       <c r="D6" t="str">
-        <v>X TBKR</v>
+        <v>-</v>
       </c>
       <c r="E6" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/8SMDhw8YpsNPPHPK7</v>
+        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,19 +572,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>ARSYL NOVA ARIRI, ST, M.Pd.</v>
+        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
       </c>
       <c r="C7" t="str">
-        <v>197811142009012007</v>
+        <v>198404192022211018</v>
       </c>
       <c r="D7" t="str">
-        <v>X TSM 1</v>
+        <v>-</v>
       </c>
       <c r="E7" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/sZ2Rff4sL9N4FTrh9</v>
+        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,19 +598,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>WAWAN SISWANTO, SS</v>
+        <v>YAYUK NURNANINGSIH, S.Pd</v>
       </c>
       <c r="C8" t="str">
-        <v>196904012007011025</v>
+        <v>198607052022212052</v>
       </c>
       <c r="D8" t="str">
-        <v>XI TAV</v>
+        <v>-</v>
       </c>
       <c r="E8" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/ghNaoJYp7o2SbkjS8</v>
+        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,19 +624,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>R.A. RATNA KARTIKAWATI, S.Pd</v>
+        <v>KHOIRUZEN, ST</v>
       </c>
       <c r="C9" t="str">
-        <v>196905132008012023</v>
+        <v>197107222023211002</v>
       </c>
       <c r="D9" t="str">
-        <v>XI TEI 1</v>
+        <v>-</v>
       </c>
       <c r="E9" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/bPxWzjgFDES2StGo6</v>
+        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,19 +650,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>NURUL HUDA, ST, M.Si.</v>
+        <v>DARIS UMAMI, S.Pd.</v>
       </c>
       <c r="C10" t="str">
-        <v>197102162008011009</v>
+        <v>198205042023212026</v>
       </c>
       <c r="D10" t="str">
-        <v>XI TPL 1</v>
+        <v>-</v>
       </c>
       <c r="E10" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/aaS7YNQQ97713C18A</v>
+        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,19 +676,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>NUR 'AFIIFAH, M.Pd.</v>
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
       </c>
       <c r="C11" t="str">
-        <v>197208052007012020</v>
+        <v>198808072023211018</v>
       </c>
       <c r="D11" t="str">
-        <v>XI TPL 2</v>
+        <v>-</v>
       </c>
       <c r="E11" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/6YPzECievjrGJZBnA</v>
+        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,19 +702,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>TRIBUDI HARTONO, S.Pd</v>
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
       </c>
       <c r="C12" t="str">
-        <v>197511052003121004</v>
+        <v>199606142023212026</v>
       </c>
       <c r="D12" t="str">
-        <v>XI TPM 1</v>
+        <v>-</v>
       </c>
       <c r="E12" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/2mog9vghqCw6TSTw7</v>
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,19 +728,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>SAMSUL HADI, M.Pd.</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C13" t="str">
-        <v>197509262008011011</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D13" t="str">
-        <v>XI TKR2</v>
+        <v>-</v>
       </c>
       <c r="E13" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/DSDoMKgI8XxbcPr78</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,19 +754,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>HISBULLOH HUDA, M.Pd.</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C14" t="str">
-        <v>197602072010011006</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D14" t="str">
-        <v>XI TBKR</v>
+        <v>-</v>
       </c>
       <c r="E14" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/jVwhLYXebas1GSZQJ6</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,19 +780,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>AGUS HARIYANTO, ST. M.Pd</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C15" t="str">
-        <v>198010032010011010</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D15" t="str">
-        <v>XI TSM 2</v>
+        <v>-</v>
       </c>
       <c r="E15" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/r3mekFxufrTcJjgRA</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,19 +806,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>SIGIT EKO PRAMONO, S.Pd</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C16" t="str">
-        <v>198301122009011006</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D16" t="str">
-        <v>XII TAV</v>
+        <v>-</v>
       </c>
       <c r="E16" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/PSXtPwi7yQN3Mfi8</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,19 +832,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>MOHAMAD ARIEF PRIYO UTOMO, S.Pd</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C17" t="str">
-        <v>198209292010011011</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D17" t="str">
-        <v>XII TPL 1</v>
+        <v>-</v>
       </c>
       <c r="E17" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/ESlazXu6aQ3PklsD9</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,19 +858,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>Dr. RIRIN DIYANNITA SASANTI, M.Pd.</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C18" t="str">
-        <v>198212022014062003</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D18" t="str">
-        <v>XII TPL 2</v>
+        <v>-</v>
       </c>
       <c r="E18" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/KwfitQjMYbtsnr4UZV6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,19 +884,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>SULIADI, S.Pd</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C19" t="str">
-        <v>198403262010011008</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D19" t="str">
-        <v>XII TPM 1</v>
+        <v>-</v>
       </c>
       <c r="E19" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/DStwfQQGe3W3gc73A</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,19 +910,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>TUTIK QOMARIYAH, S.Si</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C20" t="str">
-        <v>198504032010012014</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D20" t="str">
-        <v>XII TPM 2</v>
+        <v>-</v>
       </c>
       <c r="E20" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/8Z33XXUnWmhZCY9S9</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,19 +936,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>FIRMAN ARDIANSYAH, S.Pd.</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C21" t="str">
-        <v>198706172011011010</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D21" t="str">
-        <v>XII TKR2</v>
+        <v>-</v>
       </c>
       <c r="E21" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/iGQNqJij1huPUYbk8</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,19 +962,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>AZIZ CAHYA PRADANA, S.Pd.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C22" t="str">
-        <v>199103072019031014</v>
+        <v>-</v>
       </c>
       <c r="D22" t="str">
-        <v>XII TBKR</v>
+        <v>-</v>
       </c>
       <c r="E22" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/RvBNnww2vjNe3gNo76</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -988,19 +988,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C23" t="str">
-        <v>199311072019031004</v>
+        <v>-</v>
       </c>
       <c r="D23" t="str">
-        <v>XII TSM 1</v>
+        <v>-</v>
       </c>
       <c r="E23" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F23" t="str">
-        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G23" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1014,19 +1014,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>EFRIDA ISBANDRIYAH, S.T.</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C24" t="str">
-        <v>199511062019032010</v>
+        <v>-</v>
       </c>
       <c r="D24" t="str">
-        <v>XII DKV 1</v>
+        <v>-</v>
       </c>
       <c r="E24" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F24" t="str">
-        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G24" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1040,10 +1040,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>ETIK SULISTYOWATI, S.Pd.</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C25" t="str">
-        <v>198304282022212026</v>
+        <v>-</v>
       </c>
       <c r="D25" t="str">
         <v>-</v>
@@ -1052,7 +1052,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F25" t="str">
-        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G25" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1066,10 +1066,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C26" t="str">
-        <v>198404192022211018</v>
+        <v>-</v>
       </c>
       <c r="D26" t="str">
         <v>-</v>
@@ -1078,7 +1078,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F26" t="str">
-        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G26" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1092,10 +1092,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>YAYUK NURNANINGSIH, S.Pd</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C27" t="str">
-        <v>198607052022212052</v>
+        <v>-</v>
       </c>
       <c r="D27" t="str">
         <v>-</v>
@@ -1104,7 +1104,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F27" t="str">
-        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G27" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1118,10 +1118,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>KHOIRUZEN, ST</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C28" t="str">
-        <v>197107222023211002</v>
+        <v>-</v>
       </c>
       <c r="D28" t="str">
         <v>-</v>
@@ -1130,7 +1130,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F28" t="str">
-        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G28" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1144,10 +1144,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>DARIS UMAMI, S.Pd.</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C29" t="str">
-        <v>198205042023212026</v>
+        <v>-</v>
       </c>
       <c r="D29" t="str">
         <v>-</v>
@@ -1156,7 +1156,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F29" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G29" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1170,10 +1170,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C30" t="str">
-        <v>198808072023211018</v>
+        <v>-</v>
       </c>
       <c r="D30" t="str">
         <v>-</v>
@@ -1182,7 +1182,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F30" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G30" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1196,10 +1196,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C31" t="str">
-        <v>199606142023212026</v>
+        <v>-</v>
       </c>
       <c r="D31" t="str">
         <v>-</v>
@@ -1208,7 +1208,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F31" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G31" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1222,10 +1222,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C32" t="str">
-        <v>197206202024211005</v>
+        <v>-</v>
       </c>
       <c r="D32" t="str">
         <v>-</v>
@@ -1234,7 +1234,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F32" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G32" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1248,10 +1248,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C33" t="str">
-        <v>197907232024211002</v>
+        <v>-</v>
       </c>
       <c r="D33" t="str">
         <v>-</v>
@@ -1260,7 +1260,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F33" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G33" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1274,10 +1274,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C34" t="str">
-        <v>198005222024211005</v>
+        <v>-</v>
       </c>
       <c r="D34" t="str">
         <v>-</v>
@@ -1286,7 +1286,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F34" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G34" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1295,510 +1295,16 @@
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="A35">
-        <v>34</v>
-      </c>
-      <c r="B35" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
-      </c>
-      <c r="C35" t="str">
-        <v>198112142024212008</v>
-      </c>
-      <c r="D35" t="str">
-        <v>-</v>
-      </c>
-      <c r="E35" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F35" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
-      </c>
-      <c r="G35" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H35" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36">
-        <v>35</v>
-      </c>
-      <c r="B36" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
-      </c>
-      <c r="C36" t="str">
-        <v>198201062024212001</v>
-      </c>
-      <c r="D36" t="str">
-        <v>-</v>
-      </c>
-      <c r="E36" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F36" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
-      </c>
-      <c r="G36" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H36" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37">
-        <v>36</v>
-      </c>
-      <c r="B37" t="str">
-        <v>YEFI WULANDARI, SE</v>
-      </c>
-      <c r="C37" t="str">
-        <v>198204272024212014</v>
-      </c>
-      <c r="D37" t="str">
-        <v>-</v>
-      </c>
-      <c r="E37" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F37" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
-      </c>
-      <c r="G37" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H37" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38">
-        <v>37</v>
-      </c>
-      <c r="B38" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
-      </c>
-      <c r="C38" t="str">
-        <v>198209202024212008</v>
-      </c>
-      <c r="D38" t="str">
-        <v>-</v>
-      </c>
-      <c r="E38" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F38" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
-      </c>
-      <c r="G38" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H38" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39">
-        <v>38</v>
-      </c>
-      <c r="B39" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
-      </c>
-      <c r="C39" t="str">
-        <v>198606052024212013</v>
-      </c>
-      <c r="D39" t="str">
-        <v>-</v>
-      </c>
-      <c r="E39" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F39" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
-      </c>
-      <c r="G39" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H39" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40">
-        <v>39</v>
-      </c>
-      <c r="B40" t="str">
-        <v>SUYANTI, S.Kom.</v>
-      </c>
-      <c r="C40" t="str">
-        <v>198206012025212027</v>
-      </c>
-      <c r="D40" t="str">
-        <v>-</v>
-      </c>
-      <c r="E40" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F40" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
-      </c>
-      <c r="G40" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H40" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41">
-        <v>40</v>
-      </c>
-      <c r="B41" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
-      </c>
-      <c r="C41" t="str">
-        <v>-</v>
-      </c>
-      <c r="D41" t="str">
-        <v>-</v>
-      </c>
-      <c r="E41" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F41" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
-      </c>
-      <c r="G41" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H41" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42">
-        <v>41</v>
-      </c>
-      <c r="B42" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
-      </c>
-      <c r="C42" t="str">
-        <v>-</v>
-      </c>
-      <c r="D42" t="str">
-        <v>-</v>
-      </c>
-      <c r="E42" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F42" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
-      </c>
-      <c r="G42" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H42" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43">
-        <v>42</v>
-      </c>
-      <c r="B43" t="str">
-        <v>BENY WIJAYANTO, SS</v>
-      </c>
-      <c r="C43" t="str">
-        <v>-</v>
-      </c>
-      <c r="D43" t="str">
-        <v>-</v>
-      </c>
-      <c r="E43" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F43" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
-      </c>
-      <c r="G43" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H43" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44">
-        <v>43</v>
-      </c>
-      <c r="B44" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
-      </c>
-      <c r="C44" t="str">
-        <v>-</v>
-      </c>
-      <c r="D44" t="str">
-        <v>-</v>
-      </c>
-      <c r="E44" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F44" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
-      </c>
-      <c r="G44" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H44" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45">
-        <v>44</v>
-      </c>
-      <c r="B45" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
-      </c>
-      <c r="C45" t="str">
-        <v>-</v>
-      </c>
-      <c r="D45" t="str">
-        <v>-</v>
-      </c>
-      <c r="E45" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F45" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
-      </c>
-      <c r="G45" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H45" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46">
-        <v>45</v>
-      </c>
-      <c r="B46" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
-      </c>
-      <c r="C46" t="str">
-        <v>-</v>
-      </c>
-      <c r="D46" t="str">
-        <v>-</v>
-      </c>
-      <c r="E46" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F46" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
-      </c>
-      <c r="G46" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H46" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47">
-        <v>46</v>
-      </c>
-      <c r="B47" t="str">
-        <v>SAMUJI, S.Ag</v>
-      </c>
-      <c r="C47" t="str">
-        <v>-</v>
-      </c>
-      <c r="D47" t="str">
-        <v>-</v>
-      </c>
-      <c r="E47" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F47" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
-      </c>
-      <c r="G47" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H47" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48">
-        <v>47</v>
-      </c>
-      <c r="B48" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
-      </c>
-      <c r="C48" t="str">
-        <v>-</v>
-      </c>
-      <c r="D48" t="str">
-        <v>-</v>
-      </c>
-      <c r="E48" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F48" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
-      </c>
-      <c r="G48" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H48" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49">
-        <v>48</v>
-      </c>
-      <c r="B49" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
-      </c>
-      <c r="C49" t="str">
-        <v>-</v>
-      </c>
-      <c r="D49" t="str">
-        <v>-</v>
-      </c>
-      <c r="E49" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F49" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
-      </c>
-      <c r="G49" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H49" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50">
-        <v>49</v>
-      </c>
-      <c r="B50" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
-      </c>
-      <c r="C50" t="str">
-        <v>-</v>
-      </c>
-      <c r="D50" t="str">
-        <v>-</v>
-      </c>
-      <c r="E50" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F50" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
-      </c>
-      <c r="G50" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H50" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51">
-        <v>50</v>
-      </c>
-      <c r="B51" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
-      </c>
-      <c r="C51" t="str">
-        <v>-</v>
-      </c>
-      <c r="D51" t="str">
-        <v>-</v>
-      </c>
-      <c r="E51" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F51" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
-      </c>
-      <c r="G51" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H51" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52">
-        <v>51</v>
-      </c>
-      <c r="B52" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
-      </c>
-      <c r="C52" t="str">
-        <v>-</v>
-      </c>
-      <c r="D52" t="str">
-        <v>-</v>
-      </c>
-      <c r="E52" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F52" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
-      </c>
-      <c r="G52" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H52" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53">
-        <v>52</v>
-      </c>
-      <c r="B53" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C53" t="str">
-        <v>-</v>
-      </c>
-      <c r="D53" t="str">
-        <v>-</v>
-      </c>
-      <c r="E53" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F53" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G53" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H53" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H34"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G60"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -1883,19 +1389,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>DHURROTUL FARIDAH, S.Pd</v>
+        <v>Drs. MOEHAIMIN</v>
       </c>
       <c r="C4" t="str">
-        <v>196707142006042005</v>
+        <v>196709041997031005</v>
       </c>
       <c r="D4" t="str">
-        <v>X TPL 1</v>
+        <v>X TEI 2</v>
       </c>
       <c r="E4" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F4" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeMVWzzDZ53AHLlhGUhchbGtjSPh774mpA2M0nanLr8yfuENQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSez4gjTar2bPbopGm6ErVaBlugek0rGtLocS5azfCCp0MDSIA/viewform</v>
       </c>
       <c r="G4" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1906,19 +1412,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>SRI WINARTI, S.Pd</v>
+        <v>DHURROTUL FARIDAH, S.Pd</v>
       </c>
       <c r="C5" t="str">
-        <v>197307112007012008</v>
+        <v>196707142006042005</v>
       </c>
       <c r="D5" t="str">
-        <v>X TPL 2</v>
+        <v>X TPL 1</v>
       </c>
       <c r="E5" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F5" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeDax_Aw_bF0ozmHf2395mK0_9K9QaIgPxKL3Msw8FyZrsKJw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeMVWzzDZ53AHLlhGUhchbGtjSPh774mpA2M0nanLr8yfuENQ/viewform</v>
       </c>
       <c r="G5" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1929,19 +1435,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>NUR HAYATI, S.Psi, M.Pd.</v>
+        <v>SRI WINARTI, S.Pd</v>
       </c>
       <c r="C6" t="str">
-        <v>197310152009012003</v>
+        <v>197307112007012008</v>
       </c>
       <c r="D6" t="str">
-        <v>X TPM 2</v>
+        <v>X TPL 2</v>
       </c>
       <c r="E6" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F6" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeD8S_m6otgqVphxM7Ux4fGC0wrPh7aPQIKMKg_uaW5tKl42w/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeDax_Aw_bF0ozmHf2395mK0_9K9QaIgPxKL3Msw8FyZrsKJw/viewform</v>
       </c>
       <c r="G6" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1952,19 +1458,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>LAILA FITRIYA, S.Pd.I</v>
+        <v>MUNASRI, S.Pd.</v>
       </c>
       <c r="C7" t="str">
-        <v>198506172009012006</v>
+        <v>197003282008012013</v>
       </c>
       <c r="D7" t="str">
-        <v>X TSM 2</v>
+        <v>X TPM 1</v>
       </c>
       <c r="E7" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F7" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfLY_MCLONnsdcq8EWaQayXJZ8_9cAWE7IYKvdeEhm2S0GL9A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfb21fBd9nBHkgM2MBTbSNxfeTgWiXbFL43E9QIZX-zGLzq0g/viewform</v>
       </c>
       <c r="G7" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1975,19 +1481,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>EKA PRAMITASARI, S.Pd. M.Pd.</v>
+        <v>NUR HAYATI, S.Psi, M.Pd.</v>
       </c>
       <c r="C8" t="str">
-        <v>198710302010012005</v>
+        <v>197310152009012003</v>
       </c>
       <c r="D8" t="str">
-        <v>X DKV 1</v>
+        <v>X TPM 2</v>
       </c>
       <c r="E8" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F8" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFNOjWRONIbFscUAVy_gPYaD8c1ehSpS2dTykzwJAn_RUDGw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeD8S_m6otgqVphxM7Ux4fGC0wrPh7aPQIKMKg_uaW5tKl42w/viewform</v>
       </c>
       <c r="G8" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1998,19 +1504,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>MISBAHUR ROSYIDIN, S.Pd.</v>
+        <v>DWI RETNO TUGAS ERNAWATI, S.Pd</v>
       </c>
       <c r="C9" t="str">
-        <v>196802112008011008</v>
+        <v>196702142008012009</v>
       </c>
       <c r="D9" t="str">
-        <v>X DKV 2</v>
+        <v>X TKR1</v>
       </c>
       <c r="E9" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F9" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe7MHsr1k2S6apY2TP7L_VulJ7MaQqcKaEsASfOrFV2WfDKSw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe-IzLFr71Gdhgd06mjpg2ToTRv1yEa_u8WYc9JsSpikG-NuA/viewform</v>
       </c>
       <c r="G9" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2021,19 +1527,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>Dra. DYAH CHUSNUL CHOTIMAH</v>
+        <v>KASIATIN, S.Pd</v>
       </c>
       <c r="C10" t="str">
-        <v>196802142007012016</v>
+        <v>196908112007012019</v>
       </c>
       <c r="D10" t="str">
-        <v>X DKV 3</v>
+        <v>X TKR2</v>
       </c>
       <c r="E10" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F10" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScl7wa5Pd4jitd3sxqnpqk8tlBpTw-Bx1jl50JwfjGXK_v6ZQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf3zl2VpfYKhir9CPBloLYg_xU95VEOzo28tGm9RxY8hWf_8Q/viewform</v>
       </c>
       <c r="G10" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2044,19 +1550,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>HERI SUBYANTORO, ST, M.Pd.</v>
+        <v>SUHARTO DWI SUHERNOWO, ST</v>
       </c>
       <c r="C11" t="str">
-        <v>196910102008011021</v>
+        <v>197803262009011007</v>
       </c>
       <c r="D11" t="str">
-        <v>XI TEI 2</v>
+        <v>X TBKR</v>
       </c>
       <c r="E11" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F11" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdHmC5tO01PGYfeU-it6vioHYot6MO4Enq9Nbw1oA8DLgGJog/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdEgJQrGVluy9utuyyeyZ7psIgxX5H9-OTYUG63if-14TLXNg/viewform</v>
       </c>
       <c r="G11" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2067,19 +1573,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>DEDY HENDRIANA, S.Pd. M.Pd.</v>
+        <v>ARSYL NOVA ARIRI, ST, M.Pd.</v>
       </c>
       <c r="C12" t="str">
-        <v>197904072010011002</v>
+        <v>197811142009012007</v>
       </c>
       <c r="D12" t="str">
-        <v>XI TPM 2</v>
+        <v>X TSM 1</v>
       </c>
       <c r="E12" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F12" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSecBLlEDfTwutpIfoRhoxlk9TykVgqtywzFBczl8dG7w3nLgg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeYIRHhpNjh1FmGBMMlPQPwu6jnRfYLe__qCNtcIES7ZefQvQ/viewform</v>
       </c>
       <c r="G12" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2090,19 +1596,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>AGUS HIDAYAT, S.Pd</v>
+        <v>LAILA FITRIYA, S.Pd.I</v>
       </c>
       <c r="C13" t="str">
-        <v>196907272007011018</v>
+        <v>198506172009012006</v>
       </c>
       <c r="D13" t="str">
-        <v>XI TKR1</v>
+        <v>X TSM 2</v>
       </c>
       <c r="E13" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F13" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4cLrLtqJrSQCZlTZvjVDTqCqwr0Ezvo9jj1xlEEVIA1TgLQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfLY_MCLONnsdcq8EWaQayXJZ8_9cAWE7IYKvdeEhm2S0GL9A/viewform</v>
       </c>
       <c r="G13" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2113,19 +1619,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>DWI SANTOSO, S.Pd</v>
+        <v>EKA PRAMITASARI, S.Pd. M.Pd.</v>
       </c>
       <c r="C14" t="str">
-        <v>197908082006041019</v>
+        <v>198710302010012005</v>
       </c>
       <c r="D14" t="str">
-        <v>XI TSM 1</v>
+        <v>X DKV 1</v>
       </c>
       <c r="E14" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F14" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc3pPlG2fg8z9mrKutplhHQxr-oLEDr0OrG2tbckE403avEiw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFNOjWRONIbFscUAVy_gPYaD8c1ehSpS2dTykzwJAn_RUDGw/viewform</v>
       </c>
       <c r="G14" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2136,19 +1642,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>ZAINUL ARIFIN, M.Pd.</v>
+        <v>MISBAHUR ROSYIDIN, S.Pd.</v>
       </c>
       <c r="C15" t="str">
-        <v>198210112010011009</v>
+        <v>196802112008011008</v>
       </c>
       <c r="D15" t="str">
-        <v>XI DKV 1</v>
+        <v>X DKV 2</v>
       </c>
       <c r="E15" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F15" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc1knrp09uNEhFpIHg2HnTVcw1HE0-aoR7bacYb4cXIsHAleQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe7MHsr1k2S6apY2TP7L_VulJ7MaQqcKaEsASfOrFV2WfDKSw/viewform</v>
       </c>
       <c r="G15" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2159,19 +1665,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>BAMBANG SUJATMIKO, S.Pd</v>
+        <v>Dra. DYAH CHUSNUL CHOTIMAH</v>
       </c>
       <c r="C16" t="str">
-        <v>198211222006041009</v>
+        <v>196802142007012016</v>
       </c>
       <c r="D16" t="str">
-        <v>XI DKV 2</v>
+        <v>X DKV 3</v>
       </c>
       <c r="E16" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F16" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYyOzS9TUnTH79m-niYDGHWqxmhbtWyxFehMM6Td06hqBh1A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScl7wa5Pd4jitd3sxqnpqk8tlBpTw-Bx1jl50JwfjGXK_v6ZQ/viewform</v>
       </c>
       <c r="G16" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2182,19 +1688,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>HARTONO, S.Pd</v>
+        <v>WAWAN SISWANTO, SS</v>
       </c>
       <c r="C17" t="str">
-        <v>198205122009011009</v>
+        <v>196904012007011025</v>
       </c>
       <c r="D17" t="str">
-        <v>XI DKV 3</v>
+        <v>XI TAV</v>
       </c>
       <c r="E17" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F17" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSczcB1-HoNbq4XLNVL6d22ps_sHXrr_yAMrTdi-SXUI9dyDiA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYaU-G7gAyHPvwtYTw67xI_BcR43imBjiP3RB58jOjnU1XeQ/viewform</v>
       </c>
       <c r="G17" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2205,19 +1711,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>AGUNG RAKHMANDA, S.Kom.</v>
+        <v>R.A. RATNA KARTIKAWATI, S.Pd</v>
       </c>
       <c r="C18" t="str">
-        <v>198303272009031002</v>
+        <v>196905132008012023</v>
       </c>
       <c r="D18" t="str">
-        <v>XII TEI 1</v>
+        <v>XI TEI 1</v>
       </c>
       <c r="E18" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F18" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe3WNA-vHAA16POkCpcvBUl2Kc57HtjVXCkAQEm_mMB69NPow/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSd2bLbWa9Pca9QT7JTzZAnSSDZOakUabHJxB_JnNT3CQEv4gA/viewform</v>
       </c>
       <c r="G18" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2228,19 +1734,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>IMAM SUFERI, ST.</v>
+        <v>HERI SUBYANTORO, ST, M.Pd.</v>
       </c>
       <c r="C19" t="str">
-        <v>197712302008011013</v>
+        <v>196910102008011021</v>
       </c>
       <c r="D19" t="str">
-        <v>XII TKR1</v>
+        <v>XI TEI 2</v>
       </c>
       <c r="E19" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F19" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe8sSOVeefXvVkHVMUzrTdYO8RrfqdFwT5AQRWWlJ3ZzJAluQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdHmC5tO01PGYfeU-it6vioHYot6MO4Enq9Nbw1oA8DLgGJog/viewform</v>
       </c>
       <c r="G19" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2251,19 +1757,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
+        <v>NURUL HUDA, ST, M.Si.</v>
       </c>
       <c r="C20" t="str">
-        <v>199410092019032012</v>
+        <v>197102162008011009</v>
       </c>
       <c r="D20" t="str">
-        <v>XII TSM 2</v>
+        <v>XI TPL 1</v>
       </c>
       <c r="E20" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F20" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSd4Etrlv7kK9gUfKVu1OwwyBhjLAn4-l3PArWhzLxF13MmmVw/viewform</v>
       </c>
       <c r="G20" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2274,19 +1780,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>SOTYA BAYUNTARA, S.Pd.</v>
+        <v>NUR 'AFIIFAH, M.Pd.</v>
       </c>
       <c r="C21" t="str">
-        <v>196906252022211004</v>
+        <v>197208052007012020</v>
       </c>
       <c r="D21" t="str">
-        <v>XII DKV 2</v>
+        <v>XI TPL 2</v>
       </c>
       <c r="E21" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F21" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScZ2l8R4TTNeJdfXVZvYAgc3WGgT9QtEVz0-ANUsebuRgsWsQ/viewform</v>
       </c>
       <c r="G21" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2297,19 +1803,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>SRIGATI, SE</v>
+        <v>TRIBUDI HARTONO, S.Pd</v>
       </c>
       <c r="C22" t="str">
-        <v>197505052022212013</v>
+        <v>197511052003121004</v>
       </c>
       <c r="D22" t="str">
-        <v>XII DKV 3</v>
+        <v>XI TPM 1</v>
       </c>
       <c r="E22" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F22" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdcvHzA1p4OhUC9iXA97o8okqRsjziPMeWoPw6g-Nvt7Pr9jg/viewform</v>
       </c>
       <c r="G22" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2320,19 +1826,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>HARI PURWANTO, ST</v>
+        <v>DEDY HENDRIANA, S.Pd. M.Pd.</v>
       </c>
       <c r="C23" t="str">
-        <v>197711242022211006</v>
+        <v>197904072010011002</v>
       </c>
       <c r="D23" t="str">
-        <v>-</v>
+        <v>XI TPM 2</v>
       </c>
       <c r="E23" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F23" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSecBLlEDfTwutpIfoRhoxlk9TykVgqtywzFBczl8dG7w3nLgg/viewform</v>
       </c>
       <c r="G23" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2343,19 +1849,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>ESTI WIDHIARNI, S.T</v>
+        <v>AGUS HIDAYAT, S.Pd</v>
       </c>
       <c r="C24" t="str">
-        <v>197906032022212022</v>
+        <v>196907272007011018</v>
       </c>
       <c r="D24" t="str">
-        <v>-</v>
+        <v>XI TKR1</v>
       </c>
       <c r="E24" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F24" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4cLrLtqJrSQCZlTZvjVDTqCqwr0Ezvo9jj1xlEEVIA1TgLQ/viewform</v>
       </c>
       <c r="G24" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2366,19 +1872,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
+        <v>SAMSUL HADI, M.Pd.</v>
       </c>
       <c r="C25" t="str">
-        <v>198109092022211004</v>
+        <v>197509262008011011</v>
       </c>
       <c r="D25" t="str">
-        <v>XII TEI 2</v>
+        <v>XI TKR2</v>
       </c>
       <c r="E25" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F25" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdoHRTHs-yCXOAaQukleNcx5jWI79dOK6qbeeCW4p45bJ9CLg/viewform</v>
       </c>
       <c r="G25" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2389,19 +1895,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
+        <v>HISBULLOH HUDA, M.Pd.</v>
       </c>
       <c r="C26" t="str">
-        <v>198212102022211017</v>
+        <v>197602072010011006</v>
       </c>
       <c r="D26" t="str">
-        <v>-</v>
+        <v>XI TBKR</v>
       </c>
       <c r="E26" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F26" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSftHQdc5-VZ5uwLLimFvRnkwycT7Ys50sjgRzMN-ALHGSjCqA/viewform</v>
       </c>
       <c r="G26" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2412,19 +1918,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>KHOIRUL AMIN, S.Pd</v>
+        <v>DWI SANTOSO, S.Pd</v>
       </c>
       <c r="C27" t="str">
-        <v>198701192022211009</v>
+        <v>197908082006041019</v>
       </c>
       <c r="D27" t="str">
-        <v>-</v>
+        <v>XI TSM 1</v>
       </c>
       <c r="E27" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F27" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc3pPlG2fg8z9mrKutplhHQxr-oLEDr0OrG2tbckE403avEiw/viewform</v>
       </c>
       <c r="G27" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2435,19 +1941,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
+        <v>AGUS HARIYANTO, ST. M.Pd</v>
       </c>
       <c r="C28" t="str">
-        <v>198712072022211015</v>
+        <v>198010032010011010</v>
       </c>
       <c r="D28" t="str">
-        <v>-</v>
+        <v>XI TSM 2</v>
       </c>
       <c r="E28" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F28" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNEYg6DAPuUemLNfKalqh5_nN6m2oxlOxSvPG1Fu55a4gqNA/viewform</v>
       </c>
       <c r="G28" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2458,19 +1964,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>HEPPY LUCKITO, SST</v>
+        <v>ZAINUL ARIFIN, M.Pd.</v>
       </c>
       <c r="C29" t="str">
-        <v>198110272023211008</v>
+        <v>198210112010011009</v>
       </c>
       <c r="D29" t="str">
-        <v>-</v>
+        <v>XI DKV 1</v>
       </c>
       <c r="E29" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F29" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc1knrp09uNEhFpIHg2HnTVcw1HE0-aoR7bacYb4cXIsHAleQ/viewform</v>
       </c>
       <c r="G29" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2481,19 +1987,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>SRI PURWANINGSIH, S.Pd</v>
+        <v>BAMBANG SUJATMIKO, S.Pd</v>
       </c>
       <c r="C30" t="str">
-        <v>198203022023212020</v>
+        <v>198211222006041009</v>
       </c>
       <c r="D30" t="str">
-        <v>-</v>
+        <v>XI DKV 2</v>
       </c>
       <c r="E30" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F30" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYyOzS9TUnTH79m-niYDGHWqxmhbtWyxFehMM6Td06hqBh1A/viewform</v>
       </c>
       <c r="G30" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2504,19 +2010,19 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+        <v>HARTONO, S.Pd</v>
       </c>
       <c r="C31" t="str">
-        <v>199410282023211012</v>
+        <v>198205122009011009</v>
       </c>
       <c r="D31" t="str">
-        <v>-</v>
+        <v>XI DKV 3</v>
       </c>
       <c r="E31" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F31" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSczcB1-HoNbq4XLNVL6d22ps_sHXrr_yAMrTdi-SXUI9dyDiA/viewform</v>
       </c>
       <c r="G31" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2527,19 +2033,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SIGIT EKO PRAMONO, S.Pd</v>
       </c>
       <c r="C32" t="str">
-        <v>197509042024211002</v>
+        <v>198301122009011006</v>
       </c>
       <c r="D32" t="str">
-        <v>-</v>
+        <v>XII TAV</v>
       </c>
       <c r="E32" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F32" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdRlmK9kl1qIAOcGpf1Uu18upIQ0GWK8VkTv12k_6AEAERRMQ/viewform</v>
       </c>
       <c r="G32" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2550,19 +2056,19 @@
         <v>32</v>
       </c>
       <c r="B33" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>AGUNG RAKHMANDA, S.Kom.</v>
       </c>
       <c r="C33" t="str">
-        <v>198103052024211008</v>
+        <v>198303272009031002</v>
       </c>
       <c r="D33" t="str">
-        <v>-</v>
+        <v>XII TEI 1</v>
       </c>
       <c r="E33" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F33" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe3WNA-vHAA16POkCpcvBUl2Kc57HtjVXCkAQEm_mMB69NPow/viewform</v>
       </c>
       <c r="G33" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2573,19 +2079,19 @@
         <v>33</v>
       </c>
       <c r="B34" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>MOHAMAD ARIEF PRIYO UTOMO, S.Pd</v>
       </c>
       <c r="C34" t="str">
-        <v>198403072024211011</v>
+        <v>198209292010011011</v>
       </c>
       <c r="D34" t="str">
-        <v>-</v>
+        <v>XII TPL 1</v>
       </c>
       <c r="E34" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F34" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdPW1l4LaclpGdRqS2jqaCtnP9mivQff9TM2a9if71auoCj6g/viewform</v>
       </c>
       <c r="G34" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2596,19 +2102,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>Dr. RIRIN DIYANNITA SASANTI, M.Pd.</v>
       </c>
       <c r="C35" t="str">
-        <v>198410082024211016</v>
+        <v>198212022014062003</v>
       </c>
       <c r="D35" t="str">
-        <v>-</v>
+        <v>XII TPL 2</v>
       </c>
       <c r="E35" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F35" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSejtfmzSD3f24E8Z4AXVPgC0RTs8brRuZ_KCxV9-lmsq4C5iQ/viewform</v>
       </c>
       <c r="G35" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2619,19 +2125,19 @@
         <v>35</v>
       </c>
       <c r="B36" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>SULIADI, S.Pd</v>
       </c>
       <c r="C36" t="str">
-        <v>197411202025212006</v>
+        <v>198403262010011008</v>
       </c>
       <c r="D36" t="str">
-        <v>-</v>
+        <v>XII TPM 1</v>
       </c>
       <c r="E36" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F36" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdaT-LhGEwSzPtm9G3LL6KRs-gFmbNF2uiIykR7J7HDmdC2uQ/viewform</v>
       </c>
       <c r="G36" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2642,19 +2148,19 @@
         <v>36</v>
       </c>
       <c r="B37" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>TUTIK QOMARIYAH, S.Si</v>
       </c>
       <c r="C37" t="str">
-        <v>-</v>
+        <v>198504032010012014</v>
       </c>
       <c r="D37" t="str">
-        <v>-</v>
+        <v>XII TPM 2</v>
       </c>
       <c r="E37" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F37" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFjcTg73409mYsq9RTVwH8IBBBz5ya0_y6K1t74WjfpPWMhA/viewform</v>
       </c>
       <c r="G37" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2665,19 +2171,19 @@
         <v>37</v>
       </c>
       <c r="B38" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>IMAM SUFERI, ST.</v>
       </c>
       <c r="C38" t="str">
-        <v>-</v>
+        <v>197712302008011013</v>
       </c>
       <c r="D38" t="str">
-        <v>-</v>
+        <v>XII TKR1</v>
       </c>
       <c r="E38" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F38" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe8sSOVeefXvVkHVMUzrTdYO8RrfqdFwT5AQRWWlJ3ZzJAluQ/viewform</v>
       </c>
       <c r="G38" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2688,19 +2194,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
       </c>
       <c r="C39" t="str">
-        <v>-</v>
+        <v>199410092019032012</v>
       </c>
       <c r="D39" t="str">
-        <v>-</v>
+        <v>XII TSM 2</v>
       </c>
       <c r="E39" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F39" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
       </c>
       <c r="G39" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2711,19 +2217,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>SOTYA BAYUNTARA, S.Pd.</v>
       </c>
       <c r="C40" t="str">
-        <v>-</v>
+        <v>196906252022211004</v>
       </c>
       <c r="D40" t="str">
-        <v>-</v>
+        <v>XII DKV 2</v>
       </c>
       <c r="E40" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F40" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
       </c>
       <c r="G40" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2734,27 +2240,464 @@
         <v>40</v>
       </c>
       <c r="B41" t="str">
+        <v>SRIGATI, SE</v>
+      </c>
+      <c r="C41" t="str">
+        <v>197505052022212013</v>
+      </c>
+      <c r="D41" t="str">
+        <v>XII DKV 3</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="F41" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
+      </c>
+      <c r="G41" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="str">
+        <v>HARI PURWANTO, ST</v>
+      </c>
+      <c r="C42" t="str">
+        <v>197711242022211006</v>
+      </c>
+      <c r="D42" t="str">
+        <v>-</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F42" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
+      </c>
+      <c r="G42" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="str">
+        <v>ESTI WIDHIARNI, S.T</v>
+      </c>
+      <c r="C43" t="str">
+        <v>197906032022212022</v>
+      </c>
+      <c r="D43" t="str">
+        <v>-</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F43" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
+      </c>
+      <c r="G43" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="str">
+        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
+      </c>
+      <c r="C44" t="str">
+        <v>198109092022211004</v>
+      </c>
+      <c r="D44" t="str">
+        <v>XII TEI 2</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="F44" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
+      </c>
+      <c r="G44" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="str">
+        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
+      </c>
+      <c r="C45" t="str">
+        <v>198212102022211017</v>
+      </c>
+      <c r="D45" t="str">
+        <v>-</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F45" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
+      </c>
+      <c r="G45" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="str">
+        <v>KHOIRUL AMIN, S.Pd</v>
+      </c>
+      <c r="C46" t="str">
+        <v>198701192022211009</v>
+      </c>
+      <c r="D46" t="str">
+        <v>-</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F46" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
+      </c>
+      <c r="G46" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="str">
+        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
+      </c>
+      <c r="C47" t="str">
+        <v>198712072022211015</v>
+      </c>
+      <c r="D47" t="str">
+        <v>-</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F47" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
+      </c>
+      <c r="G47" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="str">
+        <v>HEPPY LUCKITO, SST</v>
+      </c>
+      <c r="C48" t="str">
+        <v>198110272023211008</v>
+      </c>
+      <c r="D48" t="str">
+        <v>-</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F48" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
+      </c>
+      <c r="G48" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="str">
+        <v>SRI PURWANINGSIH, S.Pd</v>
+      </c>
+      <c r="C49" t="str">
+        <v>198203022023212020</v>
+      </c>
+      <c r="D49" t="str">
+        <v>-</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F49" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
+      </c>
+      <c r="G49" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="str">
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+      </c>
+      <c r="C50" t="str">
+        <v>199410282023211012</v>
+      </c>
+      <c r="D50" t="str">
+        <v>-</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F50" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+      </c>
+      <c r="G50" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="str">
+        <v>ROHMAN, S.T.</v>
+      </c>
+      <c r="C51" t="str">
+        <v>197509042024211002</v>
+      </c>
+      <c r="D51" t="str">
+        <v>-</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F51" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+      </c>
+      <c r="G51" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="str">
+        <v>HARIS ALI MUHYIDIN, S.T</v>
+      </c>
+      <c r="C52" t="str">
+        <v>198103052024211008</v>
+      </c>
+      <c r="D52" t="str">
+        <v>-</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F52" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+      </c>
+      <c r="G52" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="str">
+        <v>SUWOYO, S.Kom</v>
+      </c>
+      <c r="C53" t="str">
+        <v>198403072024211011</v>
+      </c>
+      <c r="D53" t="str">
+        <v>-</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F53" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+      </c>
+      <c r="G53" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="str">
+        <v>AAN SUSANTO, S.Pd.</v>
+      </c>
+      <c r="C54" t="str">
+        <v>198410082024211016</v>
+      </c>
+      <c r="D54" t="str">
+        <v>-</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F54" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+      </c>
+      <c r="G54" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="str">
+        <v>NUR FAUZIYAH, S.Ag.</v>
+      </c>
+      <c r="C55" t="str">
+        <v>197411202025212006</v>
+      </c>
+      <c r="D55" t="str">
+        <v>-</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F55" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+      </c>
+      <c r="G55" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="str">
+        <v>CAHYA ISKANDAR, S.T</v>
+      </c>
+      <c r="C56" t="str">
+        <v>-</v>
+      </c>
+      <c r="D56" t="str">
+        <v>-</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F56" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+      </c>
+      <c r="G56" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="str">
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+      </c>
+      <c r="C57" t="str">
+        <v>-</v>
+      </c>
+      <c r="D57" t="str">
+        <v>-</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F57" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+      </c>
+      <c r="G57" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="str">
+        <v>YUNIAR DWI LISTYANTO, ST</v>
+      </c>
+      <c r="C58" t="str">
+        <v>-</v>
+      </c>
+      <c r="D58" t="str">
+        <v>-</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F58" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+      </c>
+      <c r="G58" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C59" t="str">
+        <v>-</v>
+      </c>
+      <c r="D59" t="str">
+        <v>-</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F59" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G59" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C41" t="str">
-        <v>-</v>
-      </c>
-      <c r="D41" t="str">
-        <v>-</v>
-      </c>
-      <c r="E41" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F41" t="str">
+      <c r="C60" t="str">
+        <v>-</v>
+      </c>
+      <c r="D60" t="str">
+        <v>-</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F60" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G41" t="str">
+      <c r="G60" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G60"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2868,13 +2811,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/ekQJWbDbi72DSNHX9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSez4gjTar2bPbopGm6ErVaBlugek0rGtLocS5azfCCp0MDSIA/viewform</v>
       </c>
       <c r="G4" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H4" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="5">
@@ -2946,13 +2889,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/FzjMqjr2bhYB4mFGA</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfb21fBd9nBHkgM2MBTbSNxfeTgWiXbFL43E9QIZX-zGLzq0g/viewform</v>
       </c>
       <c r="G7" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H7" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="8">
@@ -2998,13 +2941,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/hpaJmjc4TSuY21187</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe-IzLFr71Gdhgd06mjpg2ToTRv1yEa_u8WYc9JsSpikG-NuA/viewform</v>
       </c>
       <c r="G9" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H9" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="10">
@@ -3024,13 +2967,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/zCXw2UY7hgtbguuc6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf3zl2VpfYKhir9CPBloLYg_xU95VEOzo28tGm9RxY8hWf_8Q/viewform</v>
       </c>
       <c r="G10" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H10" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="11">
@@ -3050,13 +2993,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/8SMDhw8YpsNPPHPK7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdEgJQrGVluy9utuyyeyZ7psIgxX5H9-OTYUG63if-14TLXNg/viewform</v>
       </c>
       <c r="G11" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H11" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="12">
@@ -3076,13 +3019,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/sZ2Rff4sL9N4FTrh9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeYIRHhpNjh1FmGBMMlPQPwu6jnRfYLe__qCNtcIES7ZefQvQ/viewform</v>
       </c>
       <c r="G12" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H12" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="13">
@@ -3206,13 +3149,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/ghNaoJYp7o2SbkjS8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYaU-G7gAyHPvwtYTw67xI_BcR43imBjiP3RB58jOjnU1XeQ/viewform</v>
       </c>
       <c r="G17" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H17" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="18">
@@ -3232,13 +3175,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/bPxWzjgFDES2StGo6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSd2bLbWa9Pca9QT7JTzZAnSSDZOakUabHJxB_JnNT3CQEv4gA/viewform</v>
       </c>
       <c r="G18" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H18" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="19">
@@ -3284,13 +3227,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/aaS7YNQQ97713C18A</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSd4Etrlv7kK9gUfKVu1OwwyBhjLAn4-l3PArWhzLxF13MmmVw/viewform</v>
       </c>
       <c r="G20" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H20" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="21">
@@ -3310,13 +3253,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/6YPzECievjrGJZBnA</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScZ2l8R4TTNeJdfXVZvYAgc3WGgT9QtEVz0-ANUsebuRgsWsQ/viewform</v>
       </c>
       <c r="G21" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H21" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="22">
@@ -3336,13 +3279,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/2mog9vghqCw6TSTw7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdcvHzA1p4OhUC9iXA97o8okqRsjziPMeWoPw6g-Nvt7Pr9jg/viewform</v>
       </c>
       <c r="G22" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H22" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="23">
@@ -3414,13 +3357,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F25" t="str">
-        <v>https://forms.gle/DSDoMKgI8XxbcPr78</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdoHRTHs-yCXOAaQukleNcx5jWI79dOK6qbeeCW4p45bJ9CLg/viewform</v>
       </c>
       <c r="G25" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H25" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="26">
@@ -3440,13 +3383,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F26" t="str">
-        <v>https://forms.gle/jVwhLYXebas1GSZQJ6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSftHQdc5-VZ5uwLLimFvRnkwycT7Ys50sjgRzMN-ALHGSjCqA/viewform</v>
       </c>
       <c r="G26" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H26" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="27">
@@ -3492,13 +3435,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F28" t="str">
-        <v>https://forms.gle/r3mekFxufrTcJjgRA</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNEYg6DAPuUemLNfKalqh5_nN6m2oxlOxSvPG1Fu55a4gqNA/viewform</v>
       </c>
       <c r="G28" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H28" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="29">
@@ -3596,13 +3539,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F32" t="str">
-        <v>https://forms.gle/PSXtPwi7yQN3Mfi8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdRlmK9kl1qIAOcGpf1Uu18upIQ0GWK8VkTv12k_6AEAERRMQ/viewform</v>
       </c>
       <c r="G32" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H32" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="33">
@@ -3648,13 +3591,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F34" t="str">
-        <v>https://forms.gle/ESlazXu6aQ3PklsD9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdPW1l4LaclpGdRqS2jqaCtnP9mivQff9TM2a9if71auoCj6g/viewform</v>
       </c>
       <c r="G34" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H34" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="35">
@@ -3674,13 +3617,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F35" t="str">
-        <v>https://forms.gle/KwfitQjMYbtsnr4UZV6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSejtfmzSD3f24E8Z4AXVPgC0RTs8brRuZ_KCxV9-lmsq4C5iQ/viewform</v>
       </c>
       <c r="G35" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H35" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="36">
@@ -3700,13 +3643,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F36" t="str">
-        <v>https://forms.gle/DStwfQQGe3W3gc73A</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdaT-LhGEwSzPtm9G3LL6KRs-gFmbNF2uiIykR7J7HDmdC2uQ/viewform</v>
       </c>
       <c r="G36" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H36" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="37">
@@ -3726,13 +3669,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F37" t="str">
-        <v>https://forms.gle/8Z33XXUnWmhZCY9S9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFjcTg73409mYsq9RTVwH8IBBBz5ya0_y6K1t74WjfpPWMhA/viewform</v>
       </c>
       <c r="G37" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H37" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="38">

</xml_diff>

<commit_message>
Update FIRMAN ARDIANSYAH, S.Pd. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="33 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="59 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="32 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="60 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H33"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,19 +442,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>FIRMAN ARDIANSYAH, S.Pd.</v>
+        <v>AZIZ CAHYA PRADANA, S.Pd.</v>
       </c>
       <c r="C2" t="str">
-        <v>198706172011011010</v>
+        <v>199103072019031014</v>
       </c>
       <c r="D2" t="str">
-        <v>XII TKR2</v>
+        <v>XII TBKR</v>
       </c>
       <c r="E2" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/iGQNqJij1huPUYbk8</v>
+        <v>https://forms.gle/RvBNnww2vjNe3gNo76</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,19 +468,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>AZIZ CAHYA PRADANA, S.Pd.</v>
+        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
       </c>
       <c r="C3" t="str">
-        <v>199103072019031014</v>
+        <v>199311072019031004</v>
       </c>
       <c r="D3" t="str">
-        <v>XII TBKR</v>
+        <v>XII TSM 1</v>
       </c>
       <c r="E3" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/RvBNnww2vjNe3gNo76</v>
+        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,19 +494,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
+        <v>EFRIDA ISBANDRIYAH, S.T.</v>
       </c>
       <c r="C4" t="str">
-        <v>199311072019031004</v>
+        <v>199511062019032010</v>
       </c>
       <c r="D4" t="str">
-        <v>XII TSM 1</v>
+        <v>XII DKV 1</v>
       </c>
       <c r="E4" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
+        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,19 +520,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>EFRIDA ISBANDRIYAH, S.T.</v>
+        <v>ETIK SULISTYOWATI, S.Pd.</v>
       </c>
       <c r="C5" t="str">
-        <v>199511062019032010</v>
+        <v>198304282022212026</v>
       </c>
       <c r="D5" t="str">
-        <v>XII DKV 1</v>
+        <v>-</v>
       </c>
       <c r="E5" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
+        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>ETIK SULISTYOWATI, S.Pd.</v>
+        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
       </c>
       <c r="C6" t="str">
-        <v>198304282022212026</v>
+        <v>198404192022211018</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
+        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
+        <v>YAYUK NURNANINGSIH, S.Pd</v>
       </c>
       <c r="C7" t="str">
-        <v>198404192022211018</v>
+        <v>198607052022212052</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
+        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>YAYUK NURNANINGSIH, S.Pd</v>
+        <v>KHOIRUZEN, ST</v>
       </c>
       <c r="C8" t="str">
-        <v>198607052022212052</v>
+        <v>197107222023211002</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
+        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,10 +624,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>KHOIRUZEN, ST</v>
+        <v>DARIS UMAMI, S.Pd.</v>
       </c>
       <c r="C9" t="str">
-        <v>197107222023211002</v>
+        <v>198205042023212026</v>
       </c>
       <c r="D9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
+        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,10 +650,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>DARIS UMAMI, S.Pd.</v>
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
       </c>
       <c r="C10" t="str">
-        <v>198205042023212026</v>
+        <v>198808072023211018</v>
       </c>
       <c r="D10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,10 +676,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
       </c>
       <c r="C11" t="str">
-        <v>198808072023211018</v>
+        <v>199606142023212026</v>
       </c>
       <c r="D11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,10 +702,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C12" t="str">
-        <v>199606142023212026</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,10 +728,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C13" t="str">
-        <v>197206202024211005</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,10 +754,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C14" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,10 +780,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C15" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,10 +806,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C16" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,10 +832,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C17" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,10 +858,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C18" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,10 +884,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C19" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,10 +910,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C20" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,10 +936,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C21" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D21" t="str">
         <v>-</v>
@@ -948,7 +948,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,7 +962,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C22" t="str">
         <v>-</v>
@@ -974,7 +974,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -988,7 +988,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C23" t="str">
         <v>-</v>
@@ -1000,7 +1000,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F23" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G23" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1014,7 +1014,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C24" t="str">
         <v>-</v>
@@ -1026,7 +1026,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F24" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G24" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1040,7 +1040,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C25" t="str">
         <v>-</v>
@@ -1052,7 +1052,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F25" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G25" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1066,7 +1066,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C26" t="str">
         <v>-</v>
@@ -1078,7 +1078,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F26" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G26" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1092,7 +1092,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C27" t="str">
         <v>-</v>
@@ -1104,7 +1104,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F27" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G27" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1118,7 +1118,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C28" t="str">
         <v>-</v>
@@ -1130,7 +1130,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F28" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G28" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1144,7 +1144,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C29" t="str">
         <v>-</v>
@@ -1156,7 +1156,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F29" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G29" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1170,7 +1170,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C30" t="str">
         <v>-</v>
@@ -1182,7 +1182,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F30" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G30" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1196,7 +1196,7 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C31" t="str">
         <v>-</v>
@@ -1208,7 +1208,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F31" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G31" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1222,7 +1222,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C32" t="str">
         <v>-</v>
@@ -1234,7 +1234,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F32" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G32" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1248,7 +1248,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C33" t="str">
         <v>-</v>
@@ -1260,7 +1260,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F33" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G33" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1269,42 +1269,16 @@
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="A34">
-        <v>33</v>
-      </c>
-      <c r="B34" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C34" t="str">
-        <v>-</v>
-      </c>
-      <c r="D34" t="str">
-        <v>-</v>
-      </c>
-      <c r="E34" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F34" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G34" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H34" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H33"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G61"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2194,19 +2168,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="str">
-        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
+        <v>FIRMAN ARDIANSYAH, S.Pd.</v>
       </c>
       <c r="C39" t="str">
-        <v>199410092019032012</v>
+        <v>198706172011011010</v>
       </c>
       <c r="D39" t="str">
-        <v>XII TSM 2</v>
+        <v>XII TKR2</v>
       </c>
       <c r="E39" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F39" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScUo8DXP3Tp38IveX-Bq5eu4aD3aJBRVAjTA8896rGx1WUsNQ/viewform</v>
       </c>
       <c r="G39" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2217,19 +2191,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="str">
-        <v>SOTYA BAYUNTARA, S.Pd.</v>
+        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
       </c>
       <c r="C40" t="str">
-        <v>196906252022211004</v>
+        <v>199410092019032012</v>
       </c>
       <c r="D40" t="str">
-        <v>XII DKV 2</v>
+        <v>XII TSM 2</v>
       </c>
       <c r="E40" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F40" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
       </c>
       <c r="G40" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2240,19 +2214,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="str">
-        <v>SRIGATI, SE</v>
+        <v>SOTYA BAYUNTARA, S.Pd.</v>
       </c>
       <c r="C41" t="str">
-        <v>197505052022212013</v>
+        <v>196906252022211004</v>
       </c>
       <c r="D41" t="str">
-        <v>XII DKV 3</v>
+        <v>XII DKV 2</v>
       </c>
       <c r="E41" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F41" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
       </c>
       <c r="G41" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2263,19 +2237,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="str">
-        <v>HARI PURWANTO, ST</v>
+        <v>SRIGATI, SE</v>
       </c>
       <c r="C42" t="str">
-        <v>197711242022211006</v>
+        <v>197505052022212013</v>
       </c>
       <c r="D42" t="str">
-        <v>-</v>
+        <v>XII DKV 3</v>
       </c>
       <c r="E42" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F42" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
       </c>
       <c r="G42" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2286,10 +2260,10 @@
         <v>42</v>
       </c>
       <c r="B43" t="str">
-        <v>ESTI WIDHIARNI, S.T</v>
+        <v>HARI PURWANTO, ST</v>
       </c>
       <c r="C43" t="str">
-        <v>197906032022212022</v>
+        <v>197711242022211006</v>
       </c>
       <c r="D43" t="str">
         <v>-</v>
@@ -2298,7 +2272,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F43" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
       </c>
       <c r="G43" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2309,19 +2283,19 @@
         <v>43</v>
       </c>
       <c r="B44" t="str">
-        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
+        <v>ESTI WIDHIARNI, S.T</v>
       </c>
       <c r="C44" t="str">
-        <v>198109092022211004</v>
+        <v>197906032022212022</v>
       </c>
       <c r="D44" t="str">
-        <v>XII TEI 2</v>
+        <v>-</v>
       </c>
       <c r="E44" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F44" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
       </c>
       <c r="G44" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2332,19 +2306,19 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
+        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
       </c>
       <c r="C45" t="str">
-        <v>198212102022211017</v>
+        <v>198109092022211004</v>
       </c>
       <c r="D45" t="str">
-        <v>-</v>
+        <v>XII TEI 2</v>
       </c>
       <c r="E45" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F45" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
       </c>
       <c r="G45" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2355,10 +2329,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="str">
-        <v>KHOIRUL AMIN, S.Pd</v>
+        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
       </c>
       <c r="C46" t="str">
-        <v>198701192022211009</v>
+        <v>198212102022211017</v>
       </c>
       <c r="D46" t="str">
         <v>-</v>
@@ -2367,7 +2341,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F46" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
       </c>
       <c r="G46" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2378,10 +2352,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="str">
-        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
+        <v>KHOIRUL AMIN, S.Pd</v>
       </c>
       <c r="C47" t="str">
-        <v>198712072022211015</v>
+        <v>198701192022211009</v>
       </c>
       <c r="D47" t="str">
         <v>-</v>
@@ -2390,7 +2364,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F47" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
       </c>
       <c r="G47" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2401,10 +2375,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>HEPPY LUCKITO, SST</v>
+        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
       </c>
       <c r="C48" t="str">
-        <v>198110272023211008</v>
+        <v>198712072022211015</v>
       </c>
       <c r="D48" t="str">
         <v>-</v>
@@ -2413,7 +2387,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F48" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
       </c>
       <c r="G48" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2424,10 +2398,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="str">
-        <v>SRI PURWANINGSIH, S.Pd</v>
+        <v>HEPPY LUCKITO, SST</v>
       </c>
       <c r="C49" t="str">
-        <v>198203022023212020</v>
+        <v>198110272023211008</v>
       </c>
       <c r="D49" t="str">
         <v>-</v>
@@ -2436,7 +2410,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F49" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
       </c>
       <c r="G49" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2447,10 +2421,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+        <v>SRI PURWANINGSIH, S.Pd</v>
       </c>
       <c r="C50" t="str">
-        <v>199410282023211012</v>
+        <v>198203022023212020</v>
       </c>
       <c r="D50" t="str">
         <v>-</v>
@@ -2459,7 +2433,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F50" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
       </c>
       <c r="G50" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2470,10 +2444,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
       </c>
       <c r="C51" t="str">
-        <v>197509042024211002</v>
+        <v>199410282023211012</v>
       </c>
       <c r="D51" t="str">
         <v>-</v>
@@ -2482,7 +2456,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F51" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
       </c>
       <c r="G51" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2493,10 +2467,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="C52" t="str">
-        <v>198103052024211008</v>
+        <v>197509042024211002</v>
       </c>
       <c r="D52" t="str">
         <v>-</v>
@@ -2505,7 +2479,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F52" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="G52" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2516,10 +2490,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C53" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D53" t="str">
         <v>-</v>
@@ -2528,7 +2502,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F53" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G53" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2539,10 +2513,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C54" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D54" t="str">
         <v>-</v>
@@ -2551,7 +2525,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F54" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G54" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2562,10 +2536,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C55" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D55" t="str">
         <v>-</v>
@@ -2574,7 +2548,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F55" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G55" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2585,10 +2559,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C56" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D56" t="str">
         <v>-</v>
@@ -2597,7 +2571,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F56" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G56" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2608,7 +2582,7 @@
         <v>56</v>
       </c>
       <c r="B57" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C57" t="str">
         <v>-</v>
@@ -2620,7 +2594,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F57" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G57" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2631,7 +2605,7 @@
         <v>57</v>
       </c>
       <c r="B58" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C58" t="str">
         <v>-</v>
@@ -2643,7 +2617,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F58" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G58" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2654,7 +2628,7 @@
         <v>58</v>
       </c>
       <c r="B59" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C59" t="str">
         <v>-</v>
@@ -2666,7 +2640,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F59" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G59" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2677,27 +2651,50 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C60" t="str">
+        <v>-</v>
+      </c>
+      <c r="D60" t="str">
+        <v>-</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F60" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G60" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C60" t="str">
-        <v>-</v>
-      </c>
-      <c r="D60" t="str">
-        <v>-</v>
-      </c>
-      <c r="E60" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F60" t="str">
+      <c r="C61" t="str">
+        <v>-</v>
+      </c>
+      <c r="D61" t="str">
+        <v>-</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F61" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G60" t="str">
+      <c r="G61" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G60"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G61"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3721,13 +3718,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F39" t="str">
-        <v>https://forms.gle/iGQNqJij1huPUYbk8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScUo8DXP3Tp38IveX-Bq5eu4aD3aJBRVAjTA8896rGx1WUsNQ/viewform</v>
       </c>
       <c r="G39" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H39" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="40">

</xml_diff>

<commit_message>
Update AZIZ CAHYA PRADANA, S.Pd. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="32 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="60 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="31 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="61 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H32"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,19 +442,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>AZIZ CAHYA PRADANA, S.Pd.</v>
+        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
       </c>
       <c r="C2" t="str">
-        <v>199103072019031014</v>
+        <v>199311072019031004</v>
       </c>
       <c r="D2" t="str">
-        <v>XII TBKR</v>
+        <v>XII TSM 1</v>
       </c>
       <c r="E2" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/RvBNnww2vjNe3gNo76</v>
+        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,19 +468,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
+        <v>EFRIDA ISBANDRIYAH, S.T.</v>
       </c>
       <c r="C3" t="str">
-        <v>199311072019031004</v>
+        <v>199511062019032010</v>
       </c>
       <c r="D3" t="str">
-        <v>XII TSM 1</v>
+        <v>XII DKV 1</v>
       </c>
       <c r="E3" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
+        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,19 +494,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>EFRIDA ISBANDRIYAH, S.T.</v>
+        <v>ETIK SULISTYOWATI, S.Pd.</v>
       </c>
       <c r="C4" t="str">
-        <v>199511062019032010</v>
+        <v>198304282022212026</v>
       </c>
       <c r="D4" t="str">
-        <v>XII DKV 1</v>
+        <v>-</v>
       </c>
       <c r="E4" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
+        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>ETIK SULISTYOWATI, S.Pd.</v>
+        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
       </c>
       <c r="C5" t="str">
-        <v>198304282022212026</v>
+        <v>198404192022211018</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
+        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
+        <v>YAYUK NURNANINGSIH, S.Pd</v>
       </c>
       <c r="C6" t="str">
-        <v>198404192022211018</v>
+        <v>198607052022212052</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
+        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>YAYUK NURNANINGSIH, S.Pd</v>
+        <v>KHOIRUZEN, ST</v>
       </c>
       <c r="C7" t="str">
-        <v>198607052022212052</v>
+        <v>197107222023211002</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
+        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>KHOIRUZEN, ST</v>
+        <v>DARIS UMAMI, S.Pd.</v>
       </c>
       <c r="C8" t="str">
-        <v>197107222023211002</v>
+        <v>198205042023212026</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
+        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,10 +624,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>DARIS UMAMI, S.Pd.</v>
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
       </c>
       <c r="C9" t="str">
-        <v>198205042023212026</v>
+        <v>198808072023211018</v>
       </c>
       <c r="D9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,10 +650,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
       </c>
       <c r="C10" t="str">
-        <v>198808072023211018</v>
+        <v>199606142023212026</v>
       </c>
       <c r="D10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,10 +676,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C11" t="str">
-        <v>199606142023212026</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,10 +702,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C12" t="str">
-        <v>197206202024211005</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,10 +728,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C13" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,10 +754,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C14" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,10 +780,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C15" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,10 +806,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C16" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,10 +832,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C17" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,10 +858,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C18" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,10 +884,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C19" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,10 +910,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C20" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,7 +936,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C21" t="str">
         <v>-</v>
@@ -948,7 +948,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,7 +962,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C22" t="str">
         <v>-</v>
@@ -974,7 +974,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -988,7 +988,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C23" t="str">
         <v>-</v>
@@ -1000,7 +1000,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F23" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G23" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1014,7 +1014,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C24" t="str">
         <v>-</v>
@@ -1026,7 +1026,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F24" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G24" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1040,7 +1040,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C25" t="str">
         <v>-</v>
@@ -1052,7 +1052,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F25" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G25" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1066,7 +1066,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C26" t="str">
         <v>-</v>
@@ -1078,7 +1078,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F26" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G26" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1092,7 +1092,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C27" t="str">
         <v>-</v>
@@ -1104,7 +1104,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F27" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G27" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1118,7 +1118,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C28" t="str">
         <v>-</v>
@@ -1130,7 +1130,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F28" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G28" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1144,7 +1144,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C29" t="str">
         <v>-</v>
@@ -1156,7 +1156,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F29" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G29" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1170,7 +1170,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C30" t="str">
         <v>-</v>
@@ -1182,7 +1182,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F30" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G30" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1196,7 +1196,7 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C31" t="str">
         <v>-</v>
@@ -1208,7 +1208,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F31" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G31" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1222,7 +1222,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C32" t="str">
         <v>-</v>
@@ -1234,7 +1234,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F32" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G32" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1243,42 +1243,16 @@
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33">
-        <v>32</v>
-      </c>
-      <c r="B33" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C33" t="str">
-        <v>-</v>
-      </c>
-      <c r="D33" t="str">
-        <v>-</v>
-      </c>
-      <c r="E33" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F33" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G33" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H33" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H32"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G62"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2191,19 +2165,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="str">
-        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
+        <v>AZIZ CAHYA PRADANA, S.Pd.</v>
       </c>
       <c r="C40" t="str">
-        <v>199410092019032012</v>
+        <v>199103072019031014</v>
       </c>
       <c r="D40" t="str">
-        <v>XII TSM 2</v>
+        <v>XII TBKR</v>
       </c>
       <c r="E40" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F40" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScKk6RYj6qkwSYwir5SH2zma20b5qhM4boLx8UqeQ19DUTIfA/viewform</v>
       </c>
       <c r="G40" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2214,19 +2188,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="str">
-        <v>SOTYA BAYUNTARA, S.Pd.</v>
+        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
       </c>
       <c r="C41" t="str">
-        <v>196906252022211004</v>
+        <v>199410092019032012</v>
       </c>
       <c r="D41" t="str">
-        <v>XII DKV 2</v>
+        <v>XII TSM 2</v>
       </c>
       <c r="E41" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F41" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
       </c>
       <c r="G41" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2237,19 +2211,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="str">
-        <v>SRIGATI, SE</v>
+        <v>SOTYA BAYUNTARA, S.Pd.</v>
       </c>
       <c r="C42" t="str">
-        <v>197505052022212013</v>
+        <v>196906252022211004</v>
       </c>
       <c r="D42" t="str">
-        <v>XII DKV 3</v>
+        <v>XII DKV 2</v>
       </c>
       <c r="E42" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F42" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
       </c>
       <c r="G42" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2260,19 +2234,19 @@
         <v>42</v>
       </c>
       <c r="B43" t="str">
-        <v>HARI PURWANTO, ST</v>
+        <v>SRIGATI, SE</v>
       </c>
       <c r="C43" t="str">
-        <v>197711242022211006</v>
+        <v>197505052022212013</v>
       </c>
       <c r="D43" t="str">
-        <v>-</v>
+        <v>XII DKV 3</v>
       </c>
       <c r="E43" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F43" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
       </c>
       <c r="G43" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2283,10 +2257,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="str">
-        <v>ESTI WIDHIARNI, S.T</v>
+        <v>HARI PURWANTO, ST</v>
       </c>
       <c r="C44" t="str">
-        <v>197906032022212022</v>
+        <v>197711242022211006</v>
       </c>
       <c r="D44" t="str">
         <v>-</v>
@@ -2295,7 +2269,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F44" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
       </c>
       <c r="G44" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2306,19 +2280,19 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
+        <v>ESTI WIDHIARNI, S.T</v>
       </c>
       <c r="C45" t="str">
-        <v>198109092022211004</v>
+        <v>197906032022212022</v>
       </c>
       <c r="D45" t="str">
-        <v>XII TEI 2</v>
+        <v>-</v>
       </c>
       <c r="E45" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F45" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
       </c>
       <c r="G45" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2329,19 +2303,19 @@
         <v>45</v>
       </c>
       <c r="B46" t="str">
-        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
+        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
       </c>
       <c r="C46" t="str">
-        <v>198212102022211017</v>
+        <v>198109092022211004</v>
       </c>
       <c r="D46" t="str">
-        <v>-</v>
+        <v>XII TEI 2</v>
       </c>
       <c r="E46" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F46" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
       </c>
       <c r="G46" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2352,10 +2326,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="str">
-        <v>KHOIRUL AMIN, S.Pd</v>
+        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
       </c>
       <c r="C47" t="str">
-        <v>198701192022211009</v>
+        <v>198212102022211017</v>
       </c>
       <c r="D47" t="str">
         <v>-</v>
@@ -2364,7 +2338,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F47" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
       </c>
       <c r="G47" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2375,10 +2349,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
+        <v>KHOIRUL AMIN, S.Pd</v>
       </c>
       <c r="C48" t="str">
-        <v>198712072022211015</v>
+        <v>198701192022211009</v>
       </c>
       <c r="D48" t="str">
         <v>-</v>
@@ -2387,7 +2361,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F48" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
       </c>
       <c r="G48" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2398,10 +2372,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="str">
-        <v>HEPPY LUCKITO, SST</v>
+        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
       </c>
       <c r="C49" t="str">
-        <v>198110272023211008</v>
+        <v>198712072022211015</v>
       </c>
       <c r="D49" t="str">
         <v>-</v>
@@ -2410,7 +2384,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F49" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
       </c>
       <c r="G49" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2421,10 +2395,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>SRI PURWANINGSIH, S.Pd</v>
+        <v>HEPPY LUCKITO, SST</v>
       </c>
       <c r="C50" t="str">
-        <v>198203022023212020</v>
+        <v>198110272023211008</v>
       </c>
       <c r="D50" t="str">
         <v>-</v>
@@ -2433,7 +2407,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F50" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
       </c>
       <c r="G50" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2444,10 +2418,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+        <v>SRI PURWANINGSIH, S.Pd</v>
       </c>
       <c r="C51" t="str">
-        <v>199410282023211012</v>
+        <v>198203022023212020</v>
       </c>
       <c r="D51" t="str">
         <v>-</v>
@@ -2456,7 +2430,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F51" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
       </c>
       <c r="G51" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2467,10 +2441,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
       </c>
       <c r="C52" t="str">
-        <v>197509042024211002</v>
+        <v>199410282023211012</v>
       </c>
       <c r="D52" t="str">
         <v>-</v>
@@ -2479,7 +2453,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F52" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
       </c>
       <c r="G52" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2490,10 +2464,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="C53" t="str">
-        <v>198103052024211008</v>
+        <v>197509042024211002</v>
       </c>
       <c r="D53" t="str">
         <v>-</v>
@@ -2502,7 +2476,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F53" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="G53" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2513,10 +2487,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C54" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D54" t="str">
         <v>-</v>
@@ -2525,7 +2499,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F54" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G54" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2536,10 +2510,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C55" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D55" t="str">
         <v>-</v>
@@ -2548,7 +2522,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F55" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G55" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2559,10 +2533,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C56" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D56" t="str">
         <v>-</v>
@@ -2571,7 +2545,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F56" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G56" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2582,10 +2556,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C57" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D57" t="str">
         <v>-</v>
@@ -2594,7 +2568,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F57" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G57" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2605,7 +2579,7 @@
         <v>57</v>
       </c>
       <c r="B58" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C58" t="str">
         <v>-</v>
@@ -2617,7 +2591,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F58" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G58" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2628,7 +2602,7 @@
         <v>58</v>
       </c>
       <c r="B59" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C59" t="str">
         <v>-</v>
@@ -2640,7 +2614,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F59" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G59" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2651,7 +2625,7 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C60" t="str">
         <v>-</v>
@@ -2663,7 +2637,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F60" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G60" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2674,27 +2648,50 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C61" t="str">
+        <v>-</v>
+      </c>
+      <c r="D61" t="str">
+        <v>-</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F61" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G61" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C61" t="str">
-        <v>-</v>
-      </c>
-      <c r="D61" t="str">
-        <v>-</v>
-      </c>
-      <c r="E61" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F61" t="str">
+      <c r="C62" t="str">
+        <v>-</v>
+      </c>
+      <c r="D62" t="str">
+        <v>-</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F62" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G61" t="str">
+      <c r="G62" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G62"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3744,13 +3741,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F40" t="str">
-        <v>https://forms.gle/RvBNnww2vjNe3gNo76</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScKk6RYj6qkwSYwir5SH2zma20b5qhM4boLx8UqeQ19DUTIfA/viewform</v>
       </c>
       <c r="G40" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H40" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="41">

</xml_diff>

<commit_message>
Update KHOIRUZEN, ST Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="31 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="61 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="30 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="62 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H31"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>KHOIRUZEN, ST</v>
+        <v>DARIS UMAMI, S.Pd.</v>
       </c>
       <c r="C7" t="str">
-        <v>197107222023211002</v>
+        <v>198205042023212026</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
+        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>DARIS UMAMI, S.Pd.</v>
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
       </c>
       <c r="C8" t="str">
-        <v>198205042023212026</v>
+        <v>198808072023211018</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,10 +624,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
       </c>
       <c r="C9" t="str">
-        <v>198808072023211018</v>
+        <v>199606142023212026</v>
       </c>
       <c r="D9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,10 +650,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C10" t="str">
-        <v>199606142023212026</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,10 +676,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C11" t="str">
-        <v>197206202024211005</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,10 +702,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C12" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,10 +728,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C13" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,10 +754,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C14" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,10 +780,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C15" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,10 +806,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C16" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,10 +832,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C17" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,10 +858,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C18" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,10 +884,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C19" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,7 +936,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C21" t="str">
         <v>-</v>
@@ -948,7 +948,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,7 +962,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C22" t="str">
         <v>-</v>
@@ -974,7 +974,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -988,7 +988,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C23" t="str">
         <v>-</v>
@@ -1000,7 +1000,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F23" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G23" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1014,7 +1014,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C24" t="str">
         <v>-</v>
@@ -1026,7 +1026,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F24" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G24" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1040,7 +1040,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C25" t="str">
         <v>-</v>
@@ -1052,7 +1052,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F25" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G25" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1066,7 +1066,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C26" t="str">
         <v>-</v>
@@ -1078,7 +1078,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F26" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G26" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1092,7 +1092,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C27" t="str">
         <v>-</v>
@@ -1104,7 +1104,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F27" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G27" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1118,7 +1118,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C28" t="str">
         <v>-</v>
@@ -1130,7 +1130,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F28" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G28" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1144,7 +1144,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C29" t="str">
         <v>-</v>
@@ -1156,7 +1156,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F29" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G29" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1170,7 +1170,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C30" t="str">
         <v>-</v>
@@ -1182,7 +1182,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F30" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G30" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1196,7 +1196,7 @@
         <v>30</v>
       </c>
       <c r="B31" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C31" t="str">
         <v>-</v>
@@ -1208,7 +1208,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F31" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G31" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1217,42 +1217,16 @@
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32">
-        <v>31</v>
-      </c>
-      <c r="B32" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C32" t="str">
-        <v>-</v>
-      </c>
-      <c r="D32" t="str">
-        <v>-</v>
-      </c>
-      <c r="E32" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F32" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G32" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H32" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H31"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2395,10 +2369,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>HEPPY LUCKITO, SST</v>
+        <v>KHOIRUZEN, ST</v>
       </c>
       <c r="C50" t="str">
-        <v>198110272023211008</v>
+        <v>197107222023211002</v>
       </c>
       <c r="D50" t="str">
         <v>-</v>
@@ -2407,7 +2381,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F50" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
       </c>
       <c r="G50" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2418,10 +2392,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>SRI PURWANINGSIH, S.Pd</v>
+        <v>HEPPY LUCKITO, SST</v>
       </c>
       <c r="C51" t="str">
-        <v>198203022023212020</v>
+        <v>198110272023211008</v>
       </c>
       <c r="D51" t="str">
         <v>-</v>
@@ -2430,7 +2404,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F51" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
       </c>
       <c r="G51" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2441,10 +2415,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+        <v>SRI PURWANINGSIH, S.Pd</v>
       </c>
       <c r="C52" t="str">
-        <v>199410282023211012</v>
+        <v>198203022023212020</v>
       </c>
       <c r="D52" t="str">
         <v>-</v>
@@ -2453,7 +2427,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F52" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
       </c>
       <c r="G52" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2464,10 +2438,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
       </c>
       <c r="C53" t="str">
-        <v>197509042024211002</v>
+        <v>199410282023211012</v>
       </c>
       <c r="D53" t="str">
         <v>-</v>
@@ -2476,7 +2450,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F53" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
       </c>
       <c r="G53" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2487,10 +2461,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="C54" t="str">
-        <v>198103052024211008</v>
+        <v>197509042024211002</v>
       </c>
       <c r="D54" t="str">
         <v>-</v>
@@ -2499,7 +2473,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F54" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="G54" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2510,10 +2484,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C55" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D55" t="str">
         <v>-</v>
@@ -2522,7 +2496,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F55" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G55" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2533,10 +2507,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C56" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D56" t="str">
         <v>-</v>
@@ -2545,7 +2519,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F56" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G56" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2556,10 +2530,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C57" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D57" t="str">
         <v>-</v>
@@ -2568,7 +2542,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F57" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G57" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2579,10 +2553,10 @@
         <v>57</v>
       </c>
       <c r="B58" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C58" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D58" t="str">
         <v>-</v>
@@ -2591,7 +2565,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F58" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G58" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2602,7 +2576,7 @@
         <v>58</v>
       </c>
       <c r="B59" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C59" t="str">
         <v>-</v>
@@ -2614,7 +2588,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F59" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G59" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2625,7 +2599,7 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C60" t="str">
         <v>-</v>
@@ -2637,7 +2611,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F60" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G60" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2648,7 +2622,7 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C61" t="str">
         <v>-</v>
@@ -2660,7 +2634,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F61" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G61" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2671,27 +2645,50 @@
         <v>61</v>
       </c>
       <c r="B62" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C62" t="str">
+        <v>-</v>
+      </c>
+      <c r="D62" t="str">
+        <v>-</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F62" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G62" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C62" t="str">
-        <v>-</v>
-      </c>
-      <c r="D62" t="str">
-        <v>-</v>
-      </c>
-      <c r="E62" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F62" t="str">
+      <c r="C63" t="str">
+        <v>-</v>
+      </c>
+      <c r="D63" t="str">
+        <v>-</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F63" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G62" t="str">
+      <c r="G63" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4131,13 +4128,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F55" t="str">
-        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
       </c>
       <c r="G55" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H55" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="56">

</xml_diff>

<commit_message>
Update WAHYU ROFIUL AMIN, S.Pd. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="30 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="62 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="29 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="63 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H30"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,19 +442,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
+        <v>EFRIDA ISBANDRIYAH, S.T.</v>
       </c>
       <c r="C2" t="str">
-        <v>199311072019031004</v>
+        <v>199511062019032010</v>
       </c>
       <c r="D2" t="str">
-        <v>XII TSM 1</v>
+        <v>XII DKV 1</v>
       </c>
       <c r="E2" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
+        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,19 +468,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>EFRIDA ISBANDRIYAH, S.T.</v>
+        <v>ETIK SULISTYOWATI, S.Pd.</v>
       </c>
       <c r="C3" t="str">
-        <v>199511062019032010</v>
+        <v>198304282022212026</v>
       </c>
       <c r="D3" t="str">
-        <v>XII DKV 1</v>
+        <v>-</v>
       </c>
       <c r="E3" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
+        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>ETIK SULISTYOWATI, S.Pd.</v>
+        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
       </c>
       <c r="C4" t="str">
-        <v>198304282022212026</v>
+        <v>198404192022211018</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
+        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
+        <v>YAYUK NURNANINGSIH, S.Pd</v>
       </c>
       <c r="C5" t="str">
-        <v>198404192022211018</v>
+        <v>198607052022212052</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
+        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>YAYUK NURNANINGSIH, S.Pd</v>
+        <v>DARIS UMAMI, S.Pd.</v>
       </c>
       <c r="C6" t="str">
-        <v>198607052022212052</v>
+        <v>198205042023212026</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
+        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>DARIS UMAMI, S.Pd.</v>
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
       </c>
       <c r="C7" t="str">
-        <v>198205042023212026</v>
+        <v>198808072023211018</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
       </c>
       <c r="C8" t="str">
-        <v>198808072023211018</v>
+        <v>199606142023212026</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,10 +624,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C9" t="str">
-        <v>199606142023212026</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,10 +650,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C10" t="str">
-        <v>197206202024211005</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,10 +676,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C11" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,10 +702,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C12" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,10 +728,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C13" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,10 +754,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C14" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,10 +780,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C15" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,10 +806,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C16" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,10 +832,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C17" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,10 +858,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C18" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,7 +884,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,7 +936,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C21" t="str">
         <v>-</v>
@@ -948,7 +948,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,7 +962,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C22" t="str">
         <v>-</v>
@@ -974,7 +974,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -988,7 +988,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C23" t="str">
         <v>-</v>
@@ -1000,7 +1000,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F23" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G23" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1014,7 +1014,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C24" t="str">
         <v>-</v>
@@ -1026,7 +1026,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F24" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G24" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1040,7 +1040,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C25" t="str">
         <v>-</v>
@@ -1052,7 +1052,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F25" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G25" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1066,7 +1066,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C26" t="str">
         <v>-</v>
@@ -1078,7 +1078,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F26" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G26" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1092,7 +1092,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C27" t="str">
         <v>-</v>
@@ -1104,7 +1104,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F27" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G27" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1118,7 +1118,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C28" t="str">
         <v>-</v>
@@ -1130,7 +1130,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F28" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G28" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1144,7 +1144,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C29" t="str">
         <v>-</v>
@@ -1156,7 +1156,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F29" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G29" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1170,7 +1170,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C30" t="str">
         <v>-</v>
@@ -1182,7 +1182,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F30" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G30" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1191,42 +1191,16 @@
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="A31">
-        <v>30</v>
-      </c>
-      <c r="B31" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C31" t="str">
-        <v>-</v>
-      </c>
-      <c r="D31" t="str">
-        <v>-</v>
-      </c>
-      <c r="E31" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F31" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G31" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H31" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H30"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2162,19 +2136,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="str">
-        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
+        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
       </c>
       <c r="C41" t="str">
-        <v>199410092019032012</v>
+        <v>199311072019031004</v>
       </c>
       <c r="D41" t="str">
-        <v>XII TSM 2</v>
+        <v>XII TSM 1</v>
       </c>
       <c r="E41" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F41" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSczNF2YAQXf9165kZ-FthvzailwmMrM-uSTecJzWHq0JCEldQ/viewform</v>
       </c>
       <c r="G41" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2185,19 +2159,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="str">
-        <v>SOTYA BAYUNTARA, S.Pd.</v>
+        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
       </c>
       <c r="C42" t="str">
-        <v>196906252022211004</v>
+        <v>199410092019032012</v>
       </c>
       <c r="D42" t="str">
-        <v>XII DKV 2</v>
+        <v>XII TSM 2</v>
       </c>
       <c r="E42" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F42" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
       </c>
       <c r="G42" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2208,19 +2182,19 @@
         <v>42</v>
       </c>
       <c r="B43" t="str">
-        <v>SRIGATI, SE</v>
+        <v>SOTYA BAYUNTARA, S.Pd.</v>
       </c>
       <c r="C43" t="str">
-        <v>197505052022212013</v>
+        <v>196906252022211004</v>
       </c>
       <c r="D43" t="str">
-        <v>XII DKV 3</v>
+        <v>XII DKV 2</v>
       </c>
       <c r="E43" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F43" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
       </c>
       <c r="G43" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2231,19 +2205,19 @@
         <v>43</v>
       </c>
       <c r="B44" t="str">
-        <v>HARI PURWANTO, ST</v>
+        <v>SRIGATI, SE</v>
       </c>
       <c r="C44" t="str">
-        <v>197711242022211006</v>
+        <v>197505052022212013</v>
       </c>
       <c r="D44" t="str">
-        <v>-</v>
+        <v>XII DKV 3</v>
       </c>
       <c r="E44" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F44" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
       </c>
       <c r="G44" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2254,10 +2228,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>ESTI WIDHIARNI, S.T</v>
+        <v>HARI PURWANTO, ST</v>
       </c>
       <c r="C45" t="str">
-        <v>197906032022212022</v>
+        <v>197711242022211006</v>
       </c>
       <c r="D45" t="str">
         <v>-</v>
@@ -2266,7 +2240,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F45" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
       </c>
       <c r="G45" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2277,19 +2251,19 @@
         <v>45</v>
       </c>
       <c r="B46" t="str">
-        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
+        <v>ESTI WIDHIARNI, S.T</v>
       </c>
       <c r="C46" t="str">
-        <v>198109092022211004</v>
+        <v>197906032022212022</v>
       </c>
       <c r="D46" t="str">
-        <v>XII TEI 2</v>
+        <v>-</v>
       </c>
       <c r="E46" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F46" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
       </c>
       <c r="G46" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2300,19 +2274,19 @@
         <v>46</v>
       </c>
       <c r="B47" t="str">
-        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
+        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
       </c>
       <c r="C47" t="str">
-        <v>198212102022211017</v>
+        <v>198109092022211004</v>
       </c>
       <c r="D47" t="str">
-        <v>-</v>
+        <v>XII TEI 2</v>
       </c>
       <c r="E47" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F47" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
       </c>
       <c r="G47" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2323,10 +2297,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>KHOIRUL AMIN, S.Pd</v>
+        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
       </c>
       <c r="C48" t="str">
-        <v>198701192022211009</v>
+        <v>198212102022211017</v>
       </c>
       <c r="D48" t="str">
         <v>-</v>
@@ -2335,7 +2309,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F48" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
       </c>
       <c r="G48" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2346,10 +2320,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="str">
-        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
+        <v>KHOIRUL AMIN, S.Pd</v>
       </c>
       <c r="C49" t="str">
-        <v>198712072022211015</v>
+        <v>198701192022211009</v>
       </c>
       <c r="D49" t="str">
         <v>-</v>
@@ -2358,7 +2332,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F49" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
       </c>
       <c r="G49" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2369,10 +2343,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>KHOIRUZEN, ST</v>
+        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
       </c>
       <c r="C50" t="str">
-        <v>197107222023211002</v>
+        <v>198712072022211015</v>
       </c>
       <c r="D50" t="str">
         <v>-</v>
@@ -2381,7 +2355,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F50" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
       </c>
       <c r="G50" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2392,10 +2366,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>HEPPY LUCKITO, SST</v>
+        <v>KHOIRUZEN, ST</v>
       </c>
       <c r="C51" t="str">
-        <v>198110272023211008</v>
+        <v>197107222023211002</v>
       </c>
       <c r="D51" t="str">
         <v>-</v>
@@ -2404,7 +2378,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F51" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
       </c>
       <c r="G51" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2415,10 +2389,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>SRI PURWANINGSIH, S.Pd</v>
+        <v>HEPPY LUCKITO, SST</v>
       </c>
       <c r="C52" t="str">
-        <v>198203022023212020</v>
+        <v>198110272023211008</v>
       </c>
       <c r="D52" t="str">
         <v>-</v>
@@ -2427,7 +2401,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F52" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
       </c>
       <c r="G52" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2438,10 +2412,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+        <v>SRI PURWANINGSIH, S.Pd</v>
       </c>
       <c r="C53" t="str">
-        <v>199410282023211012</v>
+        <v>198203022023212020</v>
       </c>
       <c r="D53" t="str">
         <v>-</v>
@@ -2450,7 +2424,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F53" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
       </c>
       <c r="G53" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2461,10 +2435,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
       </c>
       <c r="C54" t="str">
-        <v>197509042024211002</v>
+        <v>199410282023211012</v>
       </c>
       <c r="D54" t="str">
         <v>-</v>
@@ -2473,7 +2447,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F54" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
       </c>
       <c r="G54" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2484,10 +2458,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="C55" t="str">
-        <v>198103052024211008</v>
+        <v>197509042024211002</v>
       </c>
       <c r="D55" t="str">
         <v>-</v>
@@ -2496,7 +2470,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F55" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="G55" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2507,10 +2481,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C56" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D56" t="str">
         <v>-</v>
@@ -2519,7 +2493,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F56" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G56" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2530,10 +2504,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C57" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D57" t="str">
         <v>-</v>
@@ -2542,7 +2516,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F57" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G57" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2553,10 +2527,10 @@
         <v>57</v>
       </c>
       <c r="B58" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C58" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D58" t="str">
         <v>-</v>
@@ -2565,7 +2539,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F58" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G58" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2576,10 +2550,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C59" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D59" t="str">
         <v>-</v>
@@ -2588,7 +2562,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F59" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G59" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2599,7 +2573,7 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C60" t="str">
         <v>-</v>
@@ -2611,7 +2585,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F60" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G60" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2622,7 +2596,7 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C61" t="str">
         <v>-</v>
@@ -2634,7 +2608,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F61" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G61" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2645,7 +2619,7 @@
         <v>61</v>
       </c>
       <c r="B62" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C62" t="str">
         <v>-</v>
@@ -2657,7 +2631,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F62" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G62" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2668,27 +2642,50 @@
         <v>62</v>
       </c>
       <c r="B63" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C63" t="str">
+        <v>-</v>
+      </c>
+      <c r="D63" t="str">
+        <v>-</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F63" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G63" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C63" t="str">
-        <v>-</v>
-      </c>
-      <c r="D63" t="str">
-        <v>-</v>
-      </c>
-      <c r="E63" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F63" t="str">
+      <c r="C64" t="str">
+        <v>-</v>
+      </c>
+      <c r="D64" t="str">
+        <v>-</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F64" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G63" t="str">
+      <c r="G64" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G64"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3764,13 +3761,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F41" t="str">
-        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSczNF2YAQXf9165kZ-FthvzailwmMrM-uSTecJzWHq0JCEldQ/viewform</v>
       </c>
       <c r="G41" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H41" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="42">

</xml_diff>

<commit_message>
Update EFRIDA ISBANDRIYAH, S.T. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="29 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="63 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="28 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="64 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H29"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,19 +442,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>EFRIDA ISBANDRIYAH, S.T.</v>
+        <v>ETIK SULISTYOWATI, S.Pd.</v>
       </c>
       <c r="C2" t="str">
-        <v>199511062019032010</v>
+        <v>198304282022212026</v>
       </c>
       <c r="D2" t="str">
-        <v>XII DKV 1</v>
+        <v>-</v>
       </c>
       <c r="E2" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
+        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>ETIK SULISTYOWATI, S.Pd.</v>
+        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
       </c>
       <c r="C3" t="str">
-        <v>198304282022212026</v>
+        <v>198404192022211018</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
+        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
+        <v>YAYUK NURNANINGSIH, S.Pd</v>
       </c>
       <c r="C4" t="str">
-        <v>198404192022211018</v>
+        <v>198607052022212052</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
+        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>YAYUK NURNANINGSIH, S.Pd</v>
+        <v>DARIS UMAMI, S.Pd.</v>
       </c>
       <c r="C5" t="str">
-        <v>198607052022212052</v>
+        <v>198205042023212026</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
+        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>DARIS UMAMI, S.Pd.</v>
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
       </c>
       <c r="C6" t="str">
-        <v>198205042023212026</v>
+        <v>198808072023211018</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
       </c>
       <c r="C7" t="str">
-        <v>198808072023211018</v>
+        <v>199606142023212026</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C8" t="str">
-        <v>199606142023212026</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,10 +624,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C9" t="str">
-        <v>197206202024211005</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,10 +650,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C10" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,10 +676,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C11" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,10 +702,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C12" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,10 +728,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C13" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,10 +754,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C14" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,10 +780,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C15" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,10 +806,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C16" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,10 +832,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C17" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,7 +858,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,7 +884,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,7 +936,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C21" t="str">
         <v>-</v>
@@ -948,7 +948,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,7 +962,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C22" t="str">
         <v>-</v>
@@ -974,7 +974,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -988,7 +988,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C23" t="str">
         <v>-</v>
@@ -1000,7 +1000,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F23" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G23" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1014,7 +1014,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C24" t="str">
         <v>-</v>
@@ -1026,7 +1026,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F24" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G24" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1040,7 +1040,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C25" t="str">
         <v>-</v>
@@ -1052,7 +1052,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F25" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G25" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1066,7 +1066,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C26" t="str">
         <v>-</v>
@@ -1078,7 +1078,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F26" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G26" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1092,7 +1092,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C27" t="str">
         <v>-</v>
@@ -1104,7 +1104,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F27" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G27" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1118,7 +1118,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C28" t="str">
         <v>-</v>
@@ -1130,7 +1130,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F28" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G28" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1144,7 +1144,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C29" t="str">
         <v>-</v>
@@ -1156,7 +1156,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F29" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G29" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1165,42 +1165,16 @@
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30">
-        <v>29</v>
-      </c>
-      <c r="B30" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C30" t="str">
-        <v>-</v>
-      </c>
-      <c r="D30" t="str">
-        <v>-</v>
-      </c>
-      <c r="E30" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F30" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G30" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H30" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H29"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G65"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2182,19 +2156,19 @@
         <v>42</v>
       </c>
       <c r="B43" t="str">
-        <v>SOTYA BAYUNTARA, S.Pd.</v>
+        <v>EFRIDA ISBANDRIYAH, S.T.</v>
       </c>
       <c r="C43" t="str">
-        <v>196906252022211004</v>
+        <v>199511062019032010</v>
       </c>
       <c r="D43" t="str">
-        <v>XII DKV 2</v>
+        <v>XII DKV 1</v>
       </c>
       <c r="E43" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F43" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4Z31ED-5m9YP8u3CbOt0PWt94nwzJafZSig17a3DoqRlpCQ/viewform</v>
       </c>
       <c r="G43" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2205,19 +2179,19 @@
         <v>43</v>
       </c>
       <c r="B44" t="str">
-        <v>SRIGATI, SE</v>
+        <v>SOTYA BAYUNTARA, S.Pd.</v>
       </c>
       <c r="C44" t="str">
-        <v>197505052022212013</v>
+        <v>196906252022211004</v>
       </c>
       <c r="D44" t="str">
-        <v>XII DKV 3</v>
+        <v>XII DKV 2</v>
       </c>
       <c r="E44" t="str">
         <v>Walikelas</v>
       </c>
       <c r="F44" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
       </c>
       <c r="G44" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2228,19 +2202,19 @@
         <v>44</v>
       </c>
       <c r="B45" t="str">
-        <v>HARI PURWANTO, ST</v>
+        <v>SRIGATI, SE</v>
       </c>
       <c r="C45" t="str">
-        <v>197711242022211006</v>
+        <v>197505052022212013</v>
       </c>
       <c r="D45" t="str">
-        <v>-</v>
+        <v>XII DKV 3</v>
       </c>
       <c r="E45" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F45" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
       </c>
       <c r="G45" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2251,10 +2225,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="str">
-        <v>ESTI WIDHIARNI, S.T</v>
+        <v>HARI PURWANTO, ST</v>
       </c>
       <c r="C46" t="str">
-        <v>197906032022212022</v>
+        <v>197711242022211006</v>
       </c>
       <c r="D46" t="str">
         <v>-</v>
@@ -2263,7 +2237,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F46" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
       </c>
       <c r="G46" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2274,19 +2248,19 @@
         <v>46</v>
       </c>
       <c r="B47" t="str">
-        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
+        <v>ESTI WIDHIARNI, S.T</v>
       </c>
       <c r="C47" t="str">
-        <v>198109092022211004</v>
+        <v>197906032022212022</v>
       </c>
       <c r="D47" t="str">
-        <v>XII TEI 2</v>
+        <v>-</v>
       </c>
       <c r="E47" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="F47" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
       </c>
       <c r="G47" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2297,19 +2271,19 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
+        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
       </c>
       <c r="C48" t="str">
-        <v>198212102022211017</v>
+        <v>198109092022211004</v>
       </c>
       <c r="D48" t="str">
-        <v>-</v>
+        <v>XII TEI 2</v>
       </c>
       <c r="E48" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="F48" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
       </c>
       <c r="G48" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2320,10 +2294,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="str">
-        <v>KHOIRUL AMIN, S.Pd</v>
+        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
       </c>
       <c r="C49" t="str">
-        <v>198701192022211009</v>
+        <v>198212102022211017</v>
       </c>
       <c r="D49" t="str">
         <v>-</v>
@@ -2332,7 +2306,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F49" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
       </c>
       <c r="G49" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2343,10 +2317,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
+        <v>KHOIRUL AMIN, S.Pd</v>
       </c>
       <c r="C50" t="str">
-        <v>198712072022211015</v>
+        <v>198701192022211009</v>
       </c>
       <c r="D50" t="str">
         <v>-</v>
@@ -2355,7 +2329,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F50" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
       </c>
       <c r="G50" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2366,10 +2340,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>KHOIRUZEN, ST</v>
+        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
       </c>
       <c r="C51" t="str">
-        <v>197107222023211002</v>
+        <v>198712072022211015</v>
       </c>
       <c r="D51" t="str">
         <v>-</v>
@@ -2378,7 +2352,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F51" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
       </c>
       <c r="G51" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2389,10 +2363,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>HEPPY LUCKITO, SST</v>
+        <v>KHOIRUZEN, ST</v>
       </c>
       <c r="C52" t="str">
-        <v>198110272023211008</v>
+        <v>197107222023211002</v>
       </c>
       <c r="D52" t="str">
         <v>-</v>
@@ -2401,7 +2375,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F52" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
       </c>
       <c r="G52" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2412,10 +2386,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>SRI PURWANINGSIH, S.Pd</v>
+        <v>HEPPY LUCKITO, SST</v>
       </c>
       <c r="C53" t="str">
-        <v>198203022023212020</v>
+        <v>198110272023211008</v>
       </c>
       <c r="D53" t="str">
         <v>-</v>
@@ -2424,7 +2398,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F53" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
       </c>
       <c r="G53" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2435,10 +2409,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+        <v>SRI PURWANINGSIH, S.Pd</v>
       </c>
       <c r="C54" t="str">
-        <v>199410282023211012</v>
+        <v>198203022023212020</v>
       </c>
       <c r="D54" t="str">
         <v>-</v>
@@ -2447,7 +2421,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F54" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
       </c>
       <c r="G54" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2458,10 +2432,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
       </c>
       <c r="C55" t="str">
-        <v>197509042024211002</v>
+        <v>199410282023211012</v>
       </c>
       <c r="D55" t="str">
         <v>-</v>
@@ -2470,7 +2444,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F55" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
       </c>
       <c r="G55" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2481,10 +2455,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="C56" t="str">
-        <v>198103052024211008</v>
+        <v>197509042024211002</v>
       </c>
       <c r="D56" t="str">
         <v>-</v>
@@ -2493,7 +2467,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F56" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="G56" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2504,10 +2478,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C57" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D57" t="str">
         <v>-</v>
@@ -2516,7 +2490,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F57" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G57" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2527,10 +2501,10 @@
         <v>57</v>
       </c>
       <c r="B58" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C58" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D58" t="str">
         <v>-</v>
@@ -2539,7 +2513,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F58" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G58" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2550,10 +2524,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C59" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D59" t="str">
         <v>-</v>
@@ -2562,7 +2536,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F59" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G59" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2573,10 +2547,10 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C60" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D60" t="str">
         <v>-</v>
@@ -2585,7 +2559,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F60" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G60" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2596,7 +2570,7 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C61" t="str">
         <v>-</v>
@@ -2608,7 +2582,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F61" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G61" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2619,7 +2593,7 @@
         <v>61</v>
       </c>
       <c r="B62" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C62" t="str">
         <v>-</v>
@@ -2631,7 +2605,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F62" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G62" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2642,7 +2616,7 @@
         <v>62</v>
       </c>
       <c r="B63" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C63" t="str">
         <v>-</v>
@@ -2654,7 +2628,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F63" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G63" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2665,27 +2639,50 @@
         <v>63</v>
       </c>
       <c r="B64" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C64" t="str">
+        <v>-</v>
+      </c>
+      <c r="D64" t="str">
+        <v>-</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F64" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G64" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C64" t="str">
-        <v>-</v>
-      </c>
-      <c r="D64" t="str">
-        <v>-</v>
-      </c>
-      <c r="E64" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F64" t="str">
+      <c r="C65" t="str">
+        <v>-</v>
+      </c>
+      <c r="D65" t="str">
+        <v>-</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F65" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G64" t="str">
+      <c r="G65" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G65"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3813,13 +3810,13 @@
         <v>Walikelas</v>
       </c>
       <c r="F43" t="str">
-        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4Z31ED-5m9YP8u3CbOt0PWt94nwzJafZSig17a3DoqRlpCQ/viewform</v>
       </c>
       <c r="G43" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H43" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="44">

</xml_diff>

<commit_message>
Update ETIK SULISTYOWATI, S.Pd. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="28 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="64 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="27 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="65 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H28"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>ETIK SULISTYOWATI, S.Pd.</v>
+        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
       </c>
       <c r="C2" t="str">
-        <v>198304282022212026</v>
+        <v>198404192022211018</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
+        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
+        <v>YAYUK NURNANINGSIH, S.Pd</v>
       </c>
       <c r="C3" t="str">
-        <v>198404192022211018</v>
+        <v>198607052022212052</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
+        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>YAYUK NURNANINGSIH, S.Pd</v>
+        <v>DARIS UMAMI, S.Pd.</v>
       </c>
       <c r="C4" t="str">
-        <v>198607052022212052</v>
+        <v>198205042023212026</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
+        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>DARIS UMAMI, S.Pd.</v>
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
       </c>
       <c r="C5" t="str">
-        <v>198205042023212026</v>
+        <v>198808072023211018</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
       </c>
       <c r="C6" t="str">
-        <v>198808072023211018</v>
+        <v>199606142023212026</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C7" t="str">
-        <v>199606142023212026</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C8" t="str">
-        <v>197206202024211005</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,10 +624,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C9" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,10 +650,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C10" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,10 +676,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C11" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,10 +702,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C12" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,10 +728,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C13" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,10 +754,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C14" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,10 +780,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C15" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,10 +806,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C16" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,7 +832,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,7 +858,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,7 +884,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,7 +936,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C21" t="str">
         <v>-</v>
@@ -948,7 +948,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,7 +962,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C22" t="str">
         <v>-</v>
@@ -974,7 +974,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -988,7 +988,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C23" t="str">
         <v>-</v>
@@ -1000,7 +1000,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F23" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G23" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1014,7 +1014,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C24" t="str">
         <v>-</v>
@@ -1026,7 +1026,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F24" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G24" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1040,7 +1040,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C25" t="str">
         <v>-</v>
@@ -1052,7 +1052,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F25" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G25" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1066,7 +1066,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C26" t="str">
         <v>-</v>
@@ -1078,7 +1078,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F26" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G26" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1092,7 +1092,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C27" t="str">
         <v>-</v>
@@ -1104,7 +1104,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F27" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G27" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1118,7 +1118,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C28" t="str">
         <v>-</v>
@@ -1130,7 +1130,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F28" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G28" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1139,42 +1139,16 @@
         <v/>
       </c>
     </row>
-    <row r="29">
-      <c r="A29">
-        <v>28</v>
-      </c>
-      <c r="B29" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C29" t="str">
-        <v>-</v>
-      </c>
-      <c r="D29" t="str">
-        <v>-</v>
-      </c>
-      <c r="E29" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F29" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G29" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H29" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H28"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G66"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2317,10 +2291,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="str">
-        <v>KHOIRUL AMIN, S.Pd</v>
+        <v>ETIK SULISTYOWATI, S.Pd.</v>
       </c>
       <c r="C50" t="str">
-        <v>198701192022211009</v>
+        <v>198304282022212026</v>
       </c>
       <c r="D50" t="str">
         <v>-</v>
@@ -2329,7 +2303,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F50" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdUwe7or4Y0G1-MxBUlVlO5CHIQU7My-9_OxXNA87sJhdXBZA/viewform</v>
       </c>
       <c r="G50" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2340,10 +2314,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
+        <v>KHOIRUL AMIN, S.Pd</v>
       </c>
       <c r="C51" t="str">
-        <v>198712072022211015</v>
+        <v>198701192022211009</v>
       </c>
       <c r="D51" t="str">
         <v>-</v>
@@ -2352,7 +2326,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F51" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
       </c>
       <c r="G51" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2363,10 +2337,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>KHOIRUZEN, ST</v>
+        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
       </c>
       <c r="C52" t="str">
-        <v>197107222023211002</v>
+        <v>198712072022211015</v>
       </c>
       <c r="D52" t="str">
         <v>-</v>
@@ -2375,7 +2349,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F52" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
       </c>
       <c r="G52" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2386,10 +2360,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>HEPPY LUCKITO, SST</v>
+        <v>KHOIRUZEN, ST</v>
       </c>
       <c r="C53" t="str">
-        <v>198110272023211008</v>
+        <v>197107222023211002</v>
       </c>
       <c r="D53" t="str">
         <v>-</v>
@@ -2398,7 +2372,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F53" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
       </c>
       <c r="G53" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2409,10 +2383,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="str">
-        <v>SRI PURWANINGSIH, S.Pd</v>
+        <v>HEPPY LUCKITO, SST</v>
       </c>
       <c r="C54" t="str">
-        <v>198203022023212020</v>
+        <v>198110272023211008</v>
       </c>
       <c r="D54" t="str">
         <v>-</v>
@@ -2421,7 +2395,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F54" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
       </c>
       <c r="G54" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2432,10 +2406,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+        <v>SRI PURWANINGSIH, S.Pd</v>
       </c>
       <c r="C55" t="str">
-        <v>199410282023211012</v>
+        <v>198203022023212020</v>
       </c>
       <c r="D55" t="str">
         <v>-</v>
@@ -2444,7 +2418,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F55" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
       </c>
       <c r="G55" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2455,10 +2429,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
       </c>
       <c r="C56" t="str">
-        <v>197509042024211002</v>
+        <v>199410282023211012</v>
       </c>
       <c r="D56" t="str">
         <v>-</v>
@@ -2467,7 +2441,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F56" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
       </c>
       <c r="G56" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2478,10 +2452,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="C57" t="str">
-        <v>198103052024211008</v>
+        <v>197509042024211002</v>
       </c>
       <c r="D57" t="str">
         <v>-</v>
@@ -2490,7 +2464,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F57" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="G57" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2501,10 +2475,10 @@
         <v>57</v>
       </c>
       <c r="B58" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C58" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D58" t="str">
         <v>-</v>
@@ -2513,7 +2487,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F58" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G58" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2524,10 +2498,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C59" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D59" t="str">
         <v>-</v>
@@ -2536,7 +2510,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F59" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G59" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2547,10 +2521,10 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C60" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D60" t="str">
         <v>-</v>
@@ -2559,7 +2533,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F60" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G60" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2570,10 +2544,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C61" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D61" t="str">
         <v>-</v>
@@ -2582,7 +2556,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F61" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G61" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2593,7 +2567,7 @@
         <v>61</v>
       </c>
       <c r="B62" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C62" t="str">
         <v>-</v>
@@ -2605,7 +2579,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F62" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G62" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2616,7 +2590,7 @@
         <v>62</v>
       </c>
       <c r="B63" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C63" t="str">
         <v>-</v>
@@ -2628,7 +2602,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F63" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G63" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2639,7 +2613,7 @@
         <v>63</v>
       </c>
       <c r="B64" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C64" t="str">
         <v>-</v>
@@ -2651,7 +2625,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F64" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G64" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2662,27 +2636,50 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C65" t="str">
+        <v>-</v>
+      </c>
+      <c r="D65" t="str">
+        <v>-</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F65" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G65" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C65" t="str">
-        <v>-</v>
-      </c>
-      <c r="D65" t="str">
-        <v>-</v>
-      </c>
-      <c r="E65" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F65" t="str">
+      <c r="C66" t="str">
+        <v>-</v>
+      </c>
+      <c r="D66" t="str">
+        <v>-</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F66" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G65" t="str">
+      <c r="G66" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G66"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3992,13 +3989,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F50" t="str">
-        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdUwe7or4Y0G1-MxBUlVlO5CHIQU7My-9_OxXNA87sJhdXBZA/viewform</v>
       </c>
       <c r="G50" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H50" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="51">

</xml_diff>

<commit_message>
Update NOVAN EKO SETYAWAN, S.Kom. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="27 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="65 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="26 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="66 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H27"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
+        <v>YAYUK NURNANINGSIH, S.Pd</v>
       </c>
       <c r="C2" t="str">
-        <v>198404192022211018</v>
+        <v>198607052022212052</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
+        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>YAYUK NURNANINGSIH, S.Pd</v>
+        <v>DARIS UMAMI, S.Pd.</v>
       </c>
       <c r="C3" t="str">
-        <v>198607052022212052</v>
+        <v>198205042023212026</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
+        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>DARIS UMAMI, S.Pd.</v>
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
       </c>
       <c r="C4" t="str">
-        <v>198205042023212026</v>
+        <v>198808072023211018</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
       </c>
       <c r="C5" t="str">
-        <v>198808072023211018</v>
+        <v>199606142023212026</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C6" t="str">
-        <v>199606142023212026</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C7" t="str">
-        <v>197206202024211005</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C8" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,10 +624,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C9" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,10 +650,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C10" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,10 +676,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C11" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,10 +702,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C12" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,10 +728,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C13" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,10 +754,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C14" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,10 +780,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C15" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,7 +832,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,7 +858,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,7 +884,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,7 +936,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C21" t="str">
         <v>-</v>
@@ -948,7 +948,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,7 +962,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C22" t="str">
         <v>-</v>
@@ -974,7 +974,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -988,7 +988,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C23" t="str">
         <v>-</v>
@@ -1000,7 +1000,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F23" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G23" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1014,7 +1014,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C24" t="str">
         <v>-</v>
@@ -1026,7 +1026,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F24" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G24" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1040,7 +1040,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C25" t="str">
         <v>-</v>
@@ -1052,7 +1052,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F25" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G25" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1066,7 +1066,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C26" t="str">
         <v>-</v>
@@ -1078,7 +1078,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F26" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G26" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1092,7 +1092,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C27" t="str">
         <v>-</v>
@@ -1104,7 +1104,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F27" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G27" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1113,42 +1113,16 @@
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C28" t="str">
-        <v>-</v>
-      </c>
-      <c r="D28" t="str">
-        <v>-</v>
-      </c>
-      <c r="E28" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F28" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G28" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H28" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H27"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G67"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2314,10 +2288,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="str">
-        <v>KHOIRUL AMIN, S.Pd</v>
+        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
       </c>
       <c r="C51" t="str">
-        <v>198701192022211009</v>
+        <v>198404192022211018</v>
       </c>
       <c r="D51" t="str">
         <v>-</v>
@@ -2326,7 +2300,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F51" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe4vBzUIUsBJNN39klf82XO2jf2iJXqigXNdhNMkSI7-lcsEw/viewform</v>
       </c>
       <c r="G51" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2337,10 +2311,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
+        <v>KHOIRUL AMIN, S.Pd</v>
       </c>
       <c r="C52" t="str">
-        <v>198712072022211015</v>
+        <v>198701192022211009</v>
       </c>
       <c r="D52" t="str">
         <v>-</v>
@@ -2349,7 +2323,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F52" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
       </c>
       <c r="G52" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2360,10 +2334,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>KHOIRUZEN, ST</v>
+        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
       </c>
       <c r="C53" t="str">
-        <v>197107222023211002</v>
+        <v>198712072022211015</v>
       </c>
       <c r="D53" t="str">
         <v>-</v>
@@ -2372,7 +2346,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F53" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
       </c>
       <c r="G53" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2383,10 +2357,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="str">
-        <v>HEPPY LUCKITO, SST</v>
+        <v>KHOIRUZEN, ST</v>
       </c>
       <c r="C54" t="str">
-        <v>198110272023211008</v>
+        <v>197107222023211002</v>
       </c>
       <c r="D54" t="str">
         <v>-</v>
@@ -2395,7 +2369,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F54" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
       </c>
       <c r="G54" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2406,10 +2380,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="str">
-        <v>SRI PURWANINGSIH, S.Pd</v>
+        <v>HEPPY LUCKITO, SST</v>
       </c>
       <c r="C55" t="str">
-        <v>198203022023212020</v>
+        <v>198110272023211008</v>
       </c>
       <c r="D55" t="str">
         <v>-</v>
@@ -2418,7 +2392,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F55" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
       </c>
       <c r="G55" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2429,10 +2403,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+        <v>SRI PURWANINGSIH, S.Pd</v>
       </c>
       <c r="C56" t="str">
-        <v>199410282023211012</v>
+        <v>198203022023212020</v>
       </c>
       <c r="D56" t="str">
         <v>-</v>
@@ -2441,7 +2415,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F56" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
       </c>
       <c r="G56" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2452,10 +2426,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
       </c>
       <c r="C57" t="str">
-        <v>197509042024211002</v>
+        <v>199410282023211012</v>
       </c>
       <c r="D57" t="str">
         <v>-</v>
@@ -2464,7 +2438,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F57" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
       </c>
       <c r="G57" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2475,10 +2449,10 @@
         <v>57</v>
       </c>
       <c r="B58" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="C58" t="str">
-        <v>198103052024211008</v>
+        <v>197509042024211002</v>
       </c>
       <c r="D58" t="str">
         <v>-</v>
@@ -2487,7 +2461,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F58" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="G58" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2498,10 +2472,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C59" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D59" t="str">
         <v>-</v>
@@ -2510,7 +2484,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F59" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G59" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2521,10 +2495,10 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C60" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D60" t="str">
         <v>-</v>
@@ -2533,7 +2507,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F60" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G60" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2544,10 +2518,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C61" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D61" t="str">
         <v>-</v>
@@ -2556,7 +2530,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F61" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G61" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2567,10 +2541,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C62" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D62" t="str">
         <v>-</v>
@@ -2579,7 +2553,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F62" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G62" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2590,7 +2564,7 @@
         <v>62</v>
       </c>
       <c r="B63" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C63" t="str">
         <v>-</v>
@@ -2602,7 +2576,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F63" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G63" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2613,7 +2587,7 @@
         <v>63</v>
       </c>
       <c r="B64" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C64" t="str">
         <v>-</v>
@@ -2625,7 +2599,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F64" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G64" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2636,7 +2610,7 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C65" t="str">
         <v>-</v>
@@ -2648,7 +2622,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F65" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G65" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2659,27 +2633,50 @@
         <v>65</v>
       </c>
       <c r="B66" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C66" t="str">
+        <v>-</v>
+      </c>
+      <c r="D66" t="str">
+        <v>-</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F66" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G66" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C66" t="str">
-        <v>-</v>
-      </c>
-      <c r="D66" t="str">
-        <v>-</v>
-      </c>
-      <c r="E66" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F66" t="str">
+      <c r="C67" t="str">
+        <v>-</v>
+      </c>
+      <c r="D67" t="str">
+        <v>-</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F67" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G66" t="str">
+      <c r="G67" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G67"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4015,13 +4012,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F51" t="str">
-        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe4vBzUIUsBJNN39klf82XO2jf2iJXqigXNdhNMkSI7-lcsEw/viewform</v>
       </c>
       <c r="G51" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H51" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="52">

</xml_diff>

<commit_message>
Update YAYUK NURNANINGSIH, S.Pd Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="26 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="66 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="25 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="67 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H26"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>YAYUK NURNANINGSIH, S.Pd</v>
+        <v>DARIS UMAMI, S.Pd.</v>
       </c>
       <c r="C2" t="str">
-        <v>198607052022212052</v>
+        <v>198205042023212026</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
+        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>DARIS UMAMI, S.Pd.</v>
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
       </c>
       <c r="C3" t="str">
-        <v>198205042023212026</v>
+        <v>198808072023211018</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
       </c>
       <c r="C4" t="str">
-        <v>198808072023211018</v>
+        <v>199606142023212026</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C5" t="str">
-        <v>199606142023212026</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C6" t="str">
-        <v>197206202024211005</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C7" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C8" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,10 +624,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C9" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,10 +650,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C10" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,10 +676,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C11" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,10 +702,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C12" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,10 +728,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C13" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,10 +754,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C14" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,7 +780,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,7 +832,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,7 +858,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,7 +884,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,7 +936,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C21" t="str">
         <v>-</v>
@@ -948,7 +948,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,7 +962,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C22" t="str">
         <v>-</v>
@@ -974,7 +974,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -988,7 +988,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C23" t="str">
         <v>-</v>
@@ -1000,7 +1000,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F23" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G23" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1014,7 +1014,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C24" t="str">
         <v>-</v>
@@ -1026,7 +1026,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F24" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G24" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1040,7 +1040,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C25" t="str">
         <v>-</v>
@@ -1052,7 +1052,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F25" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G25" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1066,7 +1066,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C26" t="str">
         <v>-</v>
@@ -1078,7 +1078,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F26" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G26" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1087,42 +1087,16 @@
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C27" t="str">
-        <v>-</v>
-      </c>
-      <c r="D27" t="str">
-        <v>-</v>
-      </c>
-      <c r="E27" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F27" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G27" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H27" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H26"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G68"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2311,10 +2285,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="str">
-        <v>KHOIRUL AMIN, S.Pd</v>
+        <v>YAYUK NURNANINGSIH, S.Pd</v>
       </c>
       <c r="C52" t="str">
-        <v>198701192022211009</v>
+        <v>198607052022212052</v>
       </c>
       <c r="D52" t="str">
         <v>-</v>
@@ -2323,7 +2297,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F52" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFgOYb82K7kj70lOwDL28zNyaVYlK3CX9WHttQtR-KGtb2Mg/viewform</v>
       </c>
       <c r="G52" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2334,10 +2308,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="str">
-        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
+        <v>KHOIRUL AMIN, S.Pd</v>
       </c>
       <c r="C53" t="str">
-        <v>198712072022211015</v>
+        <v>198701192022211009</v>
       </c>
       <c r="D53" t="str">
         <v>-</v>
@@ -2346,7 +2320,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F53" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
       </c>
       <c r="G53" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2357,10 +2331,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="str">
-        <v>KHOIRUZEN, ST</v>
+        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
       </c>
       <c r="C54" t="str">
-        <v>197107222023211002</v>
+        <v>198712072022211015</v>
       </c>
       <c r="D54" t="str">
         <v>-</v>
@@ -2369,7 +2343,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F54" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
       </c>
       <c r="G54" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2380,10 +2354,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="str">
-        <v>HEPPY LUCKITO, SST</v>
+        <v>KHOIRUZEN, ST</v>
       </c>
       <c r="C55" t="str">
-        <v>198110272023211008</v>
+        <v>197107222023211002</v>
       </c>
       <c r="D55" t="str">
         <v>-</v>
@@ -2392,7 +2366,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F55" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
       </c>
       <c r="G55" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2403,10 +2377,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="str">
-        <v>SRI PURWANINGSIH, S.Pd</v>
+        <v>HEPPY LUCKITO, SST</v>
       </c>
       <c r="C56" t="str">
-        <v>198203022023212020</v>
+        <v>198110272023211008</v>
       </c>
       <c r="D56" t="str">
         <v>-</v>
@@ -2415,7 +2389,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F56" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
       </c>
       <c r="G56" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2426,10 +2400,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+        <v>SRI PURWANINGSIH, S.Pd</v>
       </c>
       <c r="C57" t="str">
-        <v>199410282023211012</v>
+        <v>198203022023212020</v>
       </c>
       <c r="D57" t="str">
         <v>-</v>
@@ -2438,7 +2412,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F57" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
       </c>
       <c r="G57" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2449,10 +2423,10 @@
         <v>57</v>
       </c>
       <c r="B58" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
       </c>
       <c r="C58" t="str">
-        <v>197509042024211002</v>
+        <v>199410282023211012</v>
       </c>
       <c r="D58" t="str">
         <v>-</v>
@@ -2461,7 +2435,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F58" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
       </c>
       <c r="G58" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2472,10 +2446,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="C59" t="str">
-        <v>198103052024211008</v>
+        <v>197509042024211002</v>
       </c>
       <c r="D59" t="str">
         <v>-</v>
@@ -2484,7 +2458,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F59" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="G59" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2495,10 +2469,10 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C60" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D60" t="str">
         <v>-</v>
@@ -2507,7 +2481,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F60" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G60" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2518,10 +2492,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C61" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D61" t="str">
         <v>-</v>
@@ -2530,7 +2504,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F61" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G61" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2541,10 +2515,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C62" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D62" t="str">
         <v>-</v>
@@ -2553,7 +2527,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F62" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G62" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2564,10 +2538,10 @@
         <v>62</v>
       </c>
       <c r="B63" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C63" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D63" t="str">
         <v>-</v>
@@ -2576,7 +2550,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F63" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G63" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2587,7 +2561,7 @@
         <v>63</v>
       </c>
       <c r="B64" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C64" t="str">
         <v>-</v>
@@ -2599,7 +2573,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F64" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G64" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2610,7 +2584,7 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C65" t="str">
         <v>-</v>
@@ -2622,7 +2596,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F65" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G65" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2633,7 +2607,7 @@
         <v>65</v>
       </c>
       <c r="B66" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C66" t="str">
         <v>-</v>
@@ -2645,7 +2619,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F66" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G66" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2656,27 +2630,50 @@
         <v>66</v>
       </c>
       <c r="B67" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C67" t="str">
+        <v>-</v>
+      </c>
+      <c r="D67" t="str">
+        <v>-</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F67" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G67" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C67" t="str">
-        <v>-</v>
-      </c>
-      <c r="D67" t="str">
-        <v>-</v>
-      </c>
-      <c r="E67" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F67" t="str">
+      <c r="C68" t="str">
+        <v>-</v>
+      </c>
+      <c r="D68" t="str">
+        <v>-</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F68" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G67" t="str">
+      <c r="G68" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G67"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G68"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4038,13 +4035,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F52" t="str">
-        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFgOYb82K7kj70lOwDL28zNyaVYlK3CX9WHttQtR-KGtb2Mg/viewform</v>
       </c>
       <c r="G52" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H52" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="53">

</xml_diff>

<commit_message>
Update DARIS UMAMI, S.Pd. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="25 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="67 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="24 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="68 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>DARIS UMAMI, S.Pd.</v>
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
       </c>
       <c r="C2" t="str">
-        <v>198205042023212026</v>
+        <v>198808072023211018</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
       </c>
       <c r="C3" t="str">
-        <v>198808072023211018</v>
+        <v>199606142023212026</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C4" t="str">
-        <v>199606142023212026</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C5" t="str">
-        <v>197206202024211005</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C6" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C7" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C8" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,10 +624,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C9" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,10 +650,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C10" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,10 +676,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C11" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,10 +702,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C12" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,10 +728,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C13" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,7 +754,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,7 +780,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,7 +832,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,7 +858,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,7 +884,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,7 +936,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C21" t="str">
         <v>-</v>
@@ -948,7 +948,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,7 +962,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C22" t="str">
         <v>-</v>
@@ -974,7 +974,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -988,7 +988,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C23" t="str">
         <v>-</v>
@@ -1000,7 +1000,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F23" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G23" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1014,7 +1014,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C24" t="str">
         <v>-</v>
@@ -1026,7 +1026,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F24" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G24" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1040,7 +1040,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C25" t="str">
         <v>-</v>
@@ -1052,7 +1052,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F25" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G25" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1061,42 +1061,16 @@
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C26" t="str">
-        <v>-</v>
-      </c>
-      <c r="D26" t="str">
-        <v>-</v>
-      </c>
-      <c r="E26" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F26" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G26" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H26" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H25"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G69"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2423,10 +2397,10 @@
         <v>57</v>
       </c>
       <c r="B58" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+        <v>DARIS UMAMI, S.Pd.</v>
       </c>
       <c r="C58" t="str">
-        <v>199410282023211012</v>
+        <v>198205042023212026</v>
       </c>
       <c r="D58" t="str">
         <v>-</v>
@@ -2435,7 +2409,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F58" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSety3ZkhI7AVI8v-VQRPaTax5rflclagowfHbFtFrNjSSZNHg/viewform</v>
       </c>
       <c r="G58" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2446,10 +2420,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
       </c>
       <c r="C59" t="str">
-        <v>197509042024211002</v>
+        <v>199410282023211012</v>
       </c>
       <c r="D59" t="str">
         <v>-</v>
@@ -2458,7 +2432,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F59" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
       </c>
       <c r="G59" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2469,10 +2443,10 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="C60" t="str">
-        <v>198103052024211008</v>
+        <v>197509042024211002</v>
       </c>
       <c r="D60" t="str">
         <v>-</v>
@@ -2481,7 +2455,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F60" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="G60" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2492,10 +2466,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C61" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D61" t="str">
         <v>-</v>
@@ -2504,7 +2478,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F61" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G61" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2515,10 +2489,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C62" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D62" t="str">
         <v>-</v>
@@ -2527,7 +2501,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F62" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G62" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2538,10 +2512,10 @@
         <v>62</v>
       </c>
       <c r="B63" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C63" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D63" t="str">
         <v>-</v>
@@ -2550,7 +2524,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F63" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G63" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2561,10 +2535,10 @@
         <v>63</v>
       </c>
       <c r="B64" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C64" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D64" t="str">
         <v>-</v>
@@ -2573,7 +2547,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F64" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G64" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2584,7 +2558,7 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C65" t="str">
         <v>-</v>
@@ -2596,7 +2570,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F65" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G65" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2607,7 +2581,7 @@
         <v>65</v>
       </c>
       <c r="B66" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C66" t="str">
         <v>-</v>
@@ -2619,7 +2593,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F66" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G66" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2630,7 +2604,7 @@
         <v>66</v>
       </c>
       <c r="B67" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C67" t="str">
         <v>-</v>
@@ -2642,7 +2616,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F67" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G67" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2653,27 +2627,50 @@
         <v>67</v>
       </c>
       <c r="B68" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C68" t="str">
+        <v>-</v>
+      </c>
+      <c r="D68" t="str">
+        <v>-</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F68" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G68" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C68" t="str">
-        <v>-</v>
-      </c>
-      <c r="D68" t="str">
-        <v>-</v>
-      </c>
-      <c r="E68" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F68" t="str">
+      <c r="C69" t="str">
+        <v>-</v>
+      </c>
+      <c r="D69" t="str">
+        <v>-</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F69" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G68" t="str">
+      <c r="G69" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G68"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G69"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4191,13 +4188,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F58" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSety3ZkhI7AVI8v-VQRPaTax5rflclagowfHbFtFrNjSSZNHg/viewform</v>
       </c>
       <c r="G58" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H58" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="59">

</xml_diff>

<commit_message>
Update AKHMAD ROFI SAFUAT, S.Pd. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="24 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="68 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="23 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="69 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H24"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
       </c>
       <c r="C2" t="str">
-        <v>198808072023211018</v>
+        <v>199606142023212026</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C3" t="str">
-        <v>199606142023212026</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C4" t="str">
-        <v>197206202024211005</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C5" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C6" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C7" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C8" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,10 +624,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C9" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,10 +650,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C10" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,10 +676,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C11" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,10 +702,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C12" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,7 +728,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,7 +754,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,7 +780,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,7 +832,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,7 +858,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,7 +884,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,7 +936,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C21" t="str">
         <v>-</v>
@@ -948,7 +948,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,7 +962,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C22" t="str">
         <v>-</v>
@@ -974,7 +974,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -988,7 +988,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C23" t="str">
         <v>-</v>
@@ -1000,7 +1000,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F23" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G23" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1014,7 +1014,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C24" t="str">
         <v>-</v>
@@ -1026,7 +1026,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F24" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G24" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1035,42 +1035,16 @@
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C25" t="str">
-        <v>-</v>
-      </c>
-      <c r="D25" t="str">
-        <v>-</v>
-      </c>
-      <c r="E25" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F25" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G25" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H25" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H24"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G70"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2420,10 +2394,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
       </c>
       <c r="C59" t="str">
-        <v>199410282023211012</v>
+        <v>198808072023211018</v>
       </c>
       <c r="D59" t="str">
         <v>-</v>
@@ -2432,7 +2406,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F59" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScLoRQkJKESig6rf-hq4Hq-9UsA2rpsBuDhVX6113r1OrYeLw/viewform</v>
       </c>
       <c r="G59" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2443,10 +2417,10 @@
         <v>59</v>
       </c>
       <c r="B60" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
       </c>
       <c r="C60" t="str">
-        <v>197509042024211002</v>
+        <v>199410282023211012</v>
       </c>
       <c r="D60" t="str">
         <v>-</v>
@@ -2455,7 +2429,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F60" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
       </c>
       <c r="G60" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2466,10 +2440,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="C61" t="str">
-        <v>198103052024211008</v>
+        <v>197509042024211002</v>
       </c>
       <c r="D61" t="str">
         <v>-</v>
@@ -2478,7 +2452,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F61" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="G61" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2489,10 +2463,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C62" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D62" t="str">
         <v>-</v>
@@ -2501,7 +2475,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F62" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G62" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2512,10 +2486,10 @@
         <v>62</v>
       </c>
       <c r="B63" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C63" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D63" t="str">
         <v>-</v>
@@ -2524,7 +2498,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F63" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G63" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2535,10 +2509,10 @@
         <v>63</v>
       </c>
       <c r="B64" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C64" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D64" t="str">
         <v>-</v>
@@ -2547,7 +2521,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F64" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G64" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2558,10 +2532,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C65" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D65" t="str">
         <v>-</v>
@@ -2570,7 +2544,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F65" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G65" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2581,7 +2555,7 @@
         <v>65</v>
       </c>
       <c r="B66" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C66" t="str">
         <v>-</v>
@@ -2593,7 +2567,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F66" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G66" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2604,7 +2578,7 @@
         <v>66</v>
       </c>
       <c r="B67" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C67" t="str">
         <v>-</v>
@@ -2616,7 +2590,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F67" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G67" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2627,7 +2601,7 @@
         <v>67</v>
       </c>
       <c r="B68" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C68" t="str">
         <v>-</v>
@@ -2639,7 +2613,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F68" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G68" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2650,27 +2624,50 @@
         <v>68</v>
       </c>
       <c r="B69" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C69" t="str">
+        <v>-</v>
+      </c>
+      <c r="D69" t="str">
+        <v>-</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F69" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G69" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C69" t="str">
-        <v>-</v>
-      </c>
-      <c r="D69" t="str">
-        <v>-</v>
-      </c>
-      <c r="E69" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F69" t="str">
+      <c r="C70" t="str">
+        <v>-</v>
+      </c>
+      <c r="D70" t="str">
+        <v>-</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F70" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G69" t="str">
+      <c r="G70" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G70"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4214,13 +4211,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F59" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScLoRQkJKESig6rf-hq4Hq-9UsA2rpsBuDhVX6113r1OrYeLw/viewform</v>
       </c>
       <c r="G59" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H59" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="60">

</xml_diff>

<commit_message>
Update ASYITAH ALMUFIDAH, S.Pd Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="23 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="69 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="22 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="70 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H23"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C2" t="str">
-        <v>199606142023212026</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C3" t="str">
-        <v>197206202024211005</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C4" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C5" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C6" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C7" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C8" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,10 +624,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C9" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,10 +650,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C10" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,10 +676,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C11" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,7 +702,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,7 +728,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,7 +754,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,7 +780,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,7 +832,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,7 +858,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,7 +884,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,7 +936,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C21" t="str">
         <v>-</v>
@@ -948,7 +948,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,7 +962,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C22" t="str">
         <v>-</v>
@@ -974,7 +974,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -988,7 +988,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C23" t="str">
         <v>-</v>
@@ -1000,7 +1000,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F23" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G23" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -1009,42 +1009,16 @@
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C24" t="str">
-        <v>-</v>
-      </c>
-      <c r="D24" t="str">
-        <v>-</v>
-      </c>
-      <c r="E24" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F24" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G24" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H24" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H23"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2440,10 +2414,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
       </c>
       <c r="C61" t="str">
-        <v>197509042024211002</v>
+        <v>199606142023212026</v>
       </c>
       <c r="D61" t="str">
         <v>-</v>
@@ -2452,7 +2426,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F61" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeBM6FY62A84yCrWK-O8XZ_ehP9cDsy6qNu0MHDEXeCZlsATA/viewform</v>
       </c>
       <c r="G61" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2463,10 +2437,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="C62" t="str">
-        <v>198103052024211008</v>
+        <v>197509042024211002</v>
       </c>
       <c r="D62" t="str">
         <v>-</v>
@@ -2475,7 +2449,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F62" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="G62" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2486,10 +2460,10 @@
         <v>62</v>
       </c>
       <c r="B63" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C63" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D63" t="str">
         <v>-</v>
@@ -2498,7 +2472,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F63" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G63" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2509,10 +2483,10 @@
         <v>63</v>
       </c>
       <c r="B64" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C64" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D64" t="str">
         <v>-</v>
@@ -2521,7 +2495,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F64" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G64" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2532,10 +2506,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C65" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D65" t="str">
         <v>-</v>
@@ -2544,7 +2518,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F65" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G65" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2555,10 +2529,10 @@
         <v>65</v>
       </c>
       <c r="B66" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C66" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D66" t="str">
         <v>-</v>
@@ -2567,7 +2541,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F66" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G66" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2578,7 +2552,7 @@
         <v>66</v>
       </c>
       <c r="B67" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C67" t="str">
         <v>-</v>
@@ -2590,7 +2564,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F67" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G67" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2601,7 +2575,7 @@
         <v>67</v>
       </c>
       <c r="B68" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C68" t="str">
         <v>-</v>
@@ -2613,7 +2587,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F68" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G68" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2624,7 +2598,7 @@
         <v>68</v>
       </c>
       <c r="B69" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C69" t="str">
         <v>-</v>
@@ -2636,7 +2610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F69" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G69" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2647,27 +2621,50 @@
         <v>69</v>
       </c>
       <c r="B70" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C70" t="str">
+        <v>-</v>
+      </c>
+      <c r="D70" t="str">
+        <v>-</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F70" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G70" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C70" t="str">
-        <v>-</v>
-      </c>
-      <c r="D70" t="str">
-        <v>-</v>
-      </c>
-      <c r="E70" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F70" t="str">
+      <c r="C71" t="str">
+        <v>-</v>
+      </c>
+      <c r="D71" t="str">
+        <v>-</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F71" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G70" t="str">
+      <c r="G71" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G71"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4263,13 +4260,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F61" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeBM6FY62A84yCrWK-O8XZ_ehP9cDsy6qNu0MHDEXeCZlsATA/viewform</v>
       </c>
       <c r="G61" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H61" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="62">

</xml_diff>

<commit_message>
Update SUDARMONO, ST Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="22 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="70 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="21 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="71 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H22"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>SUDARMONO, ST</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C2" t="str">
-        <v>197206202024211005</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C3" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C4" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C5" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C6" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C7" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C8" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,10 +624,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C9" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,10 +650,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C10" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,7 +676,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,7 +702,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,7 +728,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,7 +754,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,7 +780,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,7 +832,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,7 +858,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,7 +884,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,7 +936,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C21" t="str">
         <v>-</v>
@@ -948,7 +948,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -962,7 +962,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C22" t="str">
         <v>-</v>
@@ -974,7 +974,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G22" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -983,42 +983,16 @@
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C23" t="str">
-        <v>-</v>
-      </c>
-      <c r="D23" t="str">
-        <v>-</v>
-      </c>
-      <c r="E23" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F23" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G23" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H23" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H22"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G72"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2437,10 +2411,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SUDARMONO, ST</v>
       </c>
       <c r="C62" t="str">
-        <v>197509042024211002</v>
+        <v>197206202024211005</v>
       </c>
       <c r="D62" t="str">
         <v>-</v>
@@ -2449,7 +2423,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F62" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGR9KnW2FGcWAVjUfLzEpLkENkH6O1XpstPv9041fsBK4r7A/viewform</v>
       </c>
       <c r="G62" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2460,10 +2434,10 @@
         <v>62</v>
       </c>
       <c r="B63" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="C63" t="str">
-        <v>198103052024211008</v>
+        <v>197509042024211002</v>
       </c>
       <c r="D63" t="str">
         <v>-</v>
@@ -2472,7 +2446,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F63" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="G63" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2483,10 +2457,10 @@
         <v>63</v>
       </c>
       <c r="B64" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C64" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D64" t="str">
         <v>-</v>
@@ -2495,7 +2469,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F64" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G64" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2506,10 +2480,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C65" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D65" t="str">
         <v>-</v>
@@ -2518,7 +2492,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F65" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G65" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2529,10 +2503,10 @@
         <v>65</v>
       </c>
       <c r="B66" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C66" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D66" t="str">
         <v>-</v>
@@ -2541,7 +2515,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F66" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G66" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2552,10 +2526,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C67" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D67" t="str">
         <v>-</v>
@@ -2564,7 +2538,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F67" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G67" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2575,7 +2549,7 @@
         <v>67</v>
       </c>
       <c r="B68" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C68" t="str">
         <v>-</v>
@@ -2587,7 +2561,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F68" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G68" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2598,7 +2572,7 @@
         <v>68</v>
       </c>
       <c r="B69" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C69" t="str">
         <v>-</v>
@@ -2610,7 +2584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F69" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G69" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2621,7 +2595,7 @@
         <v>69</v>
       </c>
       <c r="B70" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C70" t="str">
         <v>-</v>
@@ -2633,7 +2607,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F70" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G70" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2644,27 +2618,50 @@
         <v>70</v>
       </c>
       <c r="B71" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C71" t="str">
+        <v>-</v>
+      </c>
+      <c r="D71" t="str">
+        <v>-</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F71" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G71" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C71" t="str">
-        <v>-</v>
-      </c>
-      <c r="D71" t="str">
-        <v>-</v>
-      </c>
-      <c r="E71" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F71" t="str">
+      <c r="C72" t="str">
+        <v>-</v>
+      </c>
+      <c r="D72" t="str">
+        <v>-</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F72" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G71" t="str">
+      <c r="G72" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G71"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G72"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4286,13 +4283,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F62" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGR9KnW2FGcWAVjUfLzEpLkENkH6O1XpstPv9041fsBK4r7A/viewform</v>
       </c>
       <c r="G62" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H62" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="63">

</xml_diff>

<commit_message>
Update ANDRI YUDHI PRASETYO, ST Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="21 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="71 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="20 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="72 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H21"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C2" t="str">
-        <v>197907232024211002</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C3" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C4" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C5" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C6" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C7" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C8" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,10 +624,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C9" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,7 +650,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,7 +676,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,7 +702,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,7 +728,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,7 +754,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,7 +780,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,7 +832,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,7 +858,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,7 +884,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -936,7 +936,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C21" t="str">
         <v>-</v>
@@ -948,7 +948,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F21" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G21" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -957,42 +957,16 @@
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C22" t="str">
-        <v>-</v>
-      </c>
-      <c r="D22" t="str">
-        <v>-</v>
-      </c>
-      <c r="E22" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F22" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G22" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H22" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H21"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G73"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2457,10 +2431,10 @@
         <v>63</v>
       </c>
       <c r="B64" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>ANDRI YUDHI PRASETYO, ST</v>
       </c>
       <c r="C64" t="str">
-        <v>198103052024211008</v>
+        <v>197907232024211002</v>
       </c>
       <c r="D64" t="str">
         <v>-</v>
@@ -2469,7 +2443,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F64" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4F9PoN3h1R3EmQmS-KTPCmUB2ghq3K7N1e00Ni4NE30hESw/viewform</v>
       </c>
       <c r="G64" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2480,10 +2454,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C65" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D65" t="str">
         <v>-</v>
@@ -2492,7 +2466,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F65" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G65" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2503,10 +2477,10 @@
         <v>65</v>
       </c>
       <c r="B66" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C66" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D66" t="str">
         <v>-</v>
@@ -2515,7 +2489,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F66" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G66" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2526,10 +2500,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C67" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D67" t="str">
         <v>-</v>
@@ -2538,7 +2512,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F67" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G67" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2549,10 +2523,10 @@
         <v>67</v>
       </c>
       <c r="B68" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C68" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D68" t="str">
         <v>-</v>
@@ -2561,7 +2535,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F68" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G68" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2572,7 +2546,7 @@
         <v>68</v>
       </c>
       <c r="B69" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C69" t="str">
         <v>-</v>
@@ -2584,7 +2558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F69" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G69" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2595,7 +2569,7 @@
         <v>69</v>
       </c>
       <c r="B70" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C70" t="str">
         <v>-</v>
@@ -2607,7 +2581,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F70" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G70" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2618,7 +2592,7 @@
         <v>70</v>
       </c>
       <c r="B71" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C71" t="str">
         <v>-</v>
@@ -2630,7 +2604,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F71" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G71" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2641,27 +2615,50 @@
         <v>71</v>
       </c>
       <c r="B72" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C72" t="str">
+        <v>-</v>
+      </c>
+      <c r="D72" t="str">
+        <v>-</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F72" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G72" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C72" t="str">
-        <v>-</v>
-      </c>
-      <c r="D72" t="str">
-        <v>-</v>
-      </c>
-      <c r="E72" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F72" t="str">
+      <c r="C73" t="str">
+        <v>-</v>
+      </c>
+      <c r="D73" t="str">
+        <v>-</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F73" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G72" t="str">
+      <c r="G73" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G72"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G73"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4335,13 +4332,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F64" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4F9PoN3h1R3EmQmS-KTPCmUB2ghq3K7N1e00Ni4NE30hESw/viewform</v>
       </c>
       <c r="G64" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H64" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="65">

</xml_diff>

<commit_message>
Update MIANTO, S.Kom. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="20 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="72 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="19 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="73 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H20"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>MIANTO, S.Kom.</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C2" t="str">
-        <v>198005222024211005</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C3" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C4" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C5" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C6" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C7" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,10 +598,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C8" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,7 +650,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,7 +676,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,7 +702,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,7 +728,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,7 +754,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,7 +780,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,7 +832,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,7 +858,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,7 +884,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -910,7 +910,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C20" t="str">
         <v>-</v>
@@ -922,7 +922,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F20" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G20" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -931,42 +931,16 @@
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C21" t="str">
-        <v>-</v>
-      </c>
-      <c r="D21" t="str">
-        <v>-</v>
-      </c>
-      <c r="E21" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F21" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G21" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H21" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H20"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G74"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2454,10 +2428,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>MIANTO, S.Kom.</v>
       </c>
       <c r="C65" t="str">
-        <v>198103052024211008</v>
+        <v>198005222024211005</v>
       </c>
       <c r="D65" t="str">
         <v>-</v>
@@ -2466,7 +2440,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F65" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSee6t_4PgxzeHNbhtwqZROlfNE9Iz6Sf5QJvGMjzkmAGvhcAw/viewform</v>
       </c>
       <c r="G65" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2477,10 +2451,10 @@
         <v>65</v>
       </c>
       <c r="B66" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="C66" t="str">
-        <v>198403072024211011</v>
+        <v>198103052024211008</v>
       </c>
       <c r="D66" t="str">
         <v>-</v>
@@ -2489,7 +2463,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F66" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="G66" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2500,10 +2474,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C67" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D67" t="str">
         <v>-</v>
@@ -2512,7 +2486,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F67" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G67" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2523,10 +2497,10 @@
         <v>67</v>
       </c>
       <c r="B68" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C68" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D68" t="str">
         <v>-</v>
@@ -2535,7 +2509,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F68" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G68" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2546,10 +2520,10 @@
         <v>68</v>
       </c>
       <c r="B69" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C69" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D69" t="str">
         <v>-</v>
@@ -2558,7 +2532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F69" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G69" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2569,7 +2543,7 @@
         <v>69</v>
       </c>
       <c r="B70" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C70" t="str">
         <v>-</v>
@@ -2581,7 +2555,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F70" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G70" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2592,7 +2566,7 @@
         <v>70</v>
       </c>
       <c r="B71" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C71" t="str">
         <v>-</v>
@@ -2604,7 +2578,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F71" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G71" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2615,7 +2589,7 @@
         <v>71</v>
       </c>
       <c r="B72" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C72" t="str">
         <v>-</v>
@@ -2627,7 +2601,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F72" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G72" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2638,27 +2612,50 @@
         <v>72</v>
       </c>
       <c r="B73" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C73" t="str">
+        <v>-</v>
+      </c>
+      <c r="D73" t="str">
+        <v>-</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F73" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G73" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C73" t="str">
-        <v>-</v>
-      </c>
-      <c r="D73" t="str">
-        <v>-</v>
-      </c>
-      <c r="E73" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F73" t="str">
+      <c r="C74" t="str">
+        <v>-</v>
+      </c>
+      <c r="D74" t="str">
+        <v>-</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F74" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G73" t="str">
+      <c r="G74" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G73"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G74"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4358,13 +4355,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F65" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSee6t_4PgxzeHNbhtwqZROlfNE9Iz6Sf5QJvGMjzkmAGvhcAw/viewform</v>
       </c>
       <c r="G65" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H65" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="66">

</xml_diff>

<commit_message>
Update MAMIEK ZUHRIYAH. S.Hum Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="19 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="73 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="18 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="74 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H19"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C2" t="str">
-        <v>198112142024212008</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C3" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C4" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C5" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C6" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C7" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,7 +598,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,7 +650,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,7 +676,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,7 +702,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,7 +728,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,7 +754,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,7 +780,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,7 +832,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,7 +858,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -884,7 +884,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C19" t="str">
         <v>-</v>
@@ -896,7 +896,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F19" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G19" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -905,42 +905,16 @@
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C20" t="str">
-        <v>-</v>
-      </c>
-      <c r="D20" t="str">
-        <v>-</v>
-      </c>
-      <c r="E20" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F20" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G20" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H20" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H19"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G75"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2474,10 +2448,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
       </c>
       <c r="C67" t="str">
-        <v>198403072024211011</v>
+        <v>198112142024212008</v>
       </c>
       <c r="D67" t="str">
         <v>-</v>
@@ -2486,7 +2460,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F67" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf_FdCdD6ohlhQX_f3H7SVBGc4nrC2Ui3-rcrQZRPNnltfamQ/viewform</v>
       </c>
       <c r="G67" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2497,10 +2471,10 @@
         <v>67</v>
       </c>
       <c r="B68" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C68" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D68" t="str">
         <v>-</v>
@@ -2509,7 +2483,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F68" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G68" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2520,10 +2494,10 @@
         <v>68</v>
       </c>
       <c r="B69" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C69" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D69" t="str">
         <v>-</v>
@@ -2532,7 +2506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F69" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G69" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2543,10 +2517,10 @@
         <v>69</v>
       </c>
       <c r="B70" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C70" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D70" t="str">
         <v>-</v>
@@ -2555,7 +2529,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F70" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G70" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2566,7 +2540,7 @@
         <v>70</v>
       </c>
       <c r="B71" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C71" t="str">
         <v>-</v>
@@ -2578,7 +2552,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F71" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G71" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2589,7 +2563,7 @@
         <v>71</v>
       </c>
       <c r="B72" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C72" t="str">
         <v>-</v>
@@ -2601,7 +2575,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F72" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G72" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2612,7 +2586,7 @@
         <v>72</v>
       </c>
       <c r="B73" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C73" t="str">
         <v>-</v>
@@ -2624,7 +2598,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F73" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G73" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2635,27 +2609,50 @@
         <v>73</v>
       </c>
       <c r="B74" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C74" t="str">
+        <v>-</v>
+      </c>
+      <c r="D74" t="str">
+        <v>-</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F74" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G74" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C74" t="str">
-        <v>-</v>
-      </c>
-      <c r="D74" t="str">
-        <v>-</v>
-      </c>
-      <c r="E74" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F74" t="str">
+      <c r="C75" t="str">
+        <v>-</v>
+      </c>
+      <c r="D75" t="str">
+        <v>-</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F75" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G74" t="str">
+      <c r="G75" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G75"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4407,13 +4404,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F67" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf_FdCdD6ohlhQX_f3H7SVBGc4nrC2Ui3-rcrQZRPNnltfamQ/viewform</v>
       </c>
       <c r="G67" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H67" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="68">

</xml_diff>

<commit_message>
Update UMI RU'YATIN, S.Pd Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="18 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="74 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="17 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="75 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H18"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C2" t="str">
-        <v>198201062024212001</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C3" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C4" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C5" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,10 +546,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C6" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,7 +572,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,7 +598,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,7 +650,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,7 +676,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,7 +702,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,7 +728,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,7 +754,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,7 +780,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,7 +832,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -858,7 +858,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C18" t="str">
         <v>-</v>
@@ -870,7 +870,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F18" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G18" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -879,42 +879,16 @@
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C19" t="str">
-        <v>-</v>
-      </c>
-      <c r="D19" t="str">
-        <v>-</v>
-      </c>
-      <c r="E19" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F19" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G19" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H19" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H18"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G76"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2471,10 +2445,10 @@
         <v>67</v>
       </c>
       <c r="B68" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>UMI RU'YATIN, S.Pd</v>
       </c>
       <c r="C68" t="str">
-        <v>198403072024211011</v>
+        <v>198201062024212001</v>
       </c>
       <c r="D68" t="str">
         <v>-</v>
@@ -2483,7 +2457,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F68" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfnkOblKHmHEQZv7mSD1vVCZo9F05r9j_4cB8Gf13YpClrBEA/viewform</v>
       </c>
       <c r="G68" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2494,10 +2468,10 @@
         <v>68</v>
       </c>
       <c r="B69" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C69" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D69" t="str">
         <v>-</v>
@@ -2506,7 +2480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F69" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G69" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2517,10 +2491,10 @@
         <v>69</v>
       </c>
       <c r="B70" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C70" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D70" t="str">
         <v>-</v>
@@ -2529,7 +2503,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F70" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G70" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2540,10 +2514,10 @@
         <v>70</v>
       </c>
       <c r="B71" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C71" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D71" t="str">
         <v>-</v>
@@ -2552,7 +2526,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F71" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G71" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2563,7 +2537,7 @@
         <v>71</v>
       </c>
       <c r="B72" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C72" t="str">
         <v>-</v>
@@ -2575,7 +2549,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F72" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G72" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2586,7 +2560,7 @@
         <v>72</v>
       </c>
       <c r="B73" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C73" t="str">
         <v>-</v>
@@ -2598,7 +2572,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F73" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G73" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2609,7 +2583,7 @@
         <v>73</v>
       </c>
       <c r="B74" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C74" t="str">
         <v>-</v>
@@ -2621,7 +2595,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F74" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G74" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2632,27 +2606,50 @@
         <v>74</v>
       </c>
       <c r="B75" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C75" t="str">
+        <v>-</v>
+      </c>
+      <c r="D75" t="str">
+        <v>-</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F75" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G75" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C75" t="str">
-        <v>-</v>
-      </c>
-      <c r="D75" t="str">
-        <v>-</v>
-      </c>
-      <c r="E75" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F75" t="str">
+      <c r="C76" t="str">
+        <v>-</v>
+      </c>
+      <c r="D76" t="str">
+        <v>-</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F76" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G75" t="str">
+      <c r="G76" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G75"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G76"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4430,13 +4427,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F68" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfnkOblKHmHEQZv7mSD1vVCZo9F05r9j_4cB8Gf13YpClrBEA/viewform</v>
       </c>
       <c r="G68" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H68" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="69">

</xml_diff>

<commit_message>
Update YEFI WULANDARI, SE Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="17 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="75 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="16 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="76 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H17"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>YEFI WULANDARI, SE</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C2" t="str">
-        <v>198204272024212014</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C3" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C4" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,10 +520,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C5" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,7 +546,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,7 +572,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,7 +598,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,7 +650,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,7 +676,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,7 +702,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,7 +728,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,7 +754,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,7 +780,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -832,7 +832,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C17" t="str">
         <v>-</v>
@@ -844,7 +844,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F17" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G17" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -853,42 +853,16 @@
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C18" t="str">
-        <v>-</v>
-      </c>
-      <c r="D18" t="str">
-        <v>-</v>
-      </c>
-      <c r="E18" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F18" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G18" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H18" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H17"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G77"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2468,10 +2442,10 @@
         <v>68</v>
       </c>
       <c r="B69" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>YEFI WULANDARI, SE</v>
       </c>
       <c r="C69" t="str">
-        <v>198403072024211011</v>
+        <v>198204272024212014</v>
       </c>
       <c r="D69" t="str">
         <v>-</v>
@@ -2480,7 +2454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F69" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdWSaS-TIna_zsswr8VBL4h5etsBLiiX8g9DDJoMFMbqcqRaQ/viewform</v>
       </c>
       <c r="G69" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2491,10 +2465,10 @@
         <v>69</v>
       </c>
       <c r="B70" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C70" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D70" t="str">
         <v>-</v>
@@ -2503,7 +2477,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F70" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G70" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2514,10 +2488,10 @@
         <v>70</v>
       </c>
       <c r="B71" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C71" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D71" t="str">
         <v>-</v>
@@ -2526,7 +2500,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F71" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G71" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2537,10 +2511,10 @@
         <v>71</v>
       </c>
       <c r="B72" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C72" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D72" t="str">
         <v>-</v>
@@ -2549,7 +2523,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F72" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G72" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2560,7 +2534,7 @@
         <v>72</v>
       </c>
       <c r="B73" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C73" t="str">
         <v>-</v>
@@ -2572,7 +2546,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F73" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G73" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2583,7 +2557,7 @@
         <v>73</v>
       </c>
       <c r="B74" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C74" t="str">
         <v>-</v>
@@ -2595,7 +2569,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F74" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G74" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2606,7 +2580,7 @@
         <v>74</v>
       </c>
       <c r="B75" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C75" t="str">
         <v>-</v>
@@ -2618,7 +2592,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F75" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G75" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2629,27 +2603,50 @@
         <v>75</v>
       </c>
       <c r="B76" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C76" t="str">
+        <v>-</v>
+      </c>
+      <c r="D76" t="str">
+        <v>-</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F76" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G76" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C76" t="str">
-        <v>-</v>
-      </c>
-      <c r="D76" t="str">
-        <v>-</v>
-      </c>
-      <c r="E76" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F76" t="str">
+      <c r="C77" t="str">
+        <v>-</v>
+      </c>
+      <c r="D77" t="str">
+        <v>-</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F77" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G76" t="str">
+      <c r="G77" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G76"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G77"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4453,13 +4450,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F69" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdWSaS-TIna_zsswr8VBL4h5etsBLiiX8g9DDJoMFMbqcqRaQ/viewform</v>
       </c>
       <c r="G69" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H69" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="70">

</xml_diff>

<commit_message>
Update SARI NURHIDAYATI, S.Pd. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="16 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="76 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="15 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="77 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H16"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C2" t="str">
-        <v>198209202024212008</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C3" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,10 +494,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C4" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,7 +520,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,7 +546,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,7 +572,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,7 +598,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,7 +650,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,7 +676,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,7 +702,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,7 +728,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,7 +754,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,7 +780,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C16" t="str">
         <v>-</v>
@@ -818,7 +818,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F16" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G16" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -827,42 +827,16 @@
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C17" t="str">
-        <v>-</v>
-      </c>
-      <c r="D17" t="str">
-        <v>-</v>
-      </c>
-      <c r="E17" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F17" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G17" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H17" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G78"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2465,10 +2439,10 @@
         <v>69</v>
       </c>
       <c r="B70" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>SARI NURHIDAYATI, S.Pd.</v>
       </c>
       <c r="C70" t="str">
-        <v>198403072024211011</v>
+        <v>198209202024212008</v>
       </c>
       <c r="D70" t="str">
         <v>-</v>
@@ -2477,7 +2451,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F70" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdEXPOLI2_EBQt6mzHWAdm2mEw2qMyBnYwO7RHZF7l_PG5XoQ/viewform</v>
       </c>
       <c r="G70" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2488,10 +2462,10 @@
         <v>70</v>
       </c>
       <c r="B71" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="C71" t="str">
-        <v>198410082024211016</v>
+        <v>198403072024211011</v>
       </c>
       <c r="D71" t="str">
         <v>-</v>
@@ -2500,7 +2474,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F71" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="G71" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2511,10 +2485,10 @@
         <v>71</v>
       </c>
       <c r="B72" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="C72" t="str">
-        <v>197411202025212006</v>
+        <v>198410082024211016</v>
       </c>
       <c r="D72" t="str">
         <v>-</v>
@@ -2523,7 +2497,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F72" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="G72" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2534,10 +2508,10 @@
         <v>72</v>
       </c>
       <c r="B73" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C73" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D73" t="str">
         <v>-</v>
@@ -2546,7 +2520,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F73" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G73" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2557,7 +2531,7 @@
         <v>73</v>
       </c>
       <c r="B74" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C74" t="str">
         <v>-</v>
@@ -2569,7 +2543,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F74" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G74" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2580,7 +2554,7 @@
         <v>74</v>
       </c>
       <c r="B75" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C75" t="str">
         <v>-</v>
@@ -2592,7 +2566,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F75" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G75" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2603,7 +2577,7 @@
         <v>75</v>
       </c>
       <c r="B76" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C76" t="str">
         <v>-</v>
@@ -2615,7 +2589,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F76" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G76" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2626,27 +2600,50 @@
         <v>76</v>
       </c>
       <c r="B77" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C77" t="str">
+        <v>-</v>
+      </c>
+      <c r="D77" t="str">
+        <v>-</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F77" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G77" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C77" t="str">
-        <v>-</v>
-      </c>
-      <c r="D77" t="str">
-        <v>-</v>
-      </c>
-      <c r="E77" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F77" t="str">
+      <c r="C78" t="str">
+        <v>-</v>
+      </c>
+      <c r="D78" t="str">
+        <v>-</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F78" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G77" t="str">
+      <c r="G78" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G77"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G78"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4476,13 +4473,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F70" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdEXPOLI2_EBQt6mzHWAdm2mEw2qMyBnYwO7RHZF7l_PG5XoQ/viewform</v>
       </c>
       <c r="G70" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H70" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
Update YUNITA DWI WIRANTI, S.Pd Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="15 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="77 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="14 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="78 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H15"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C2" t="str">
-        <v>198606052024212013</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,10 +468,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C3" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,7 +494,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,7 +520,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,7 +546,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,7 +572,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,7 +598,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,7 +650,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,7 +676,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,7 +702,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,7 +728,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,7 +754,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -780,7 +780,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C15" t="str">
         <v>-</v>
@@ -792,7 +792,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F15" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G15" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -801,42 +801,16 @@
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C16" t="str">
-        <v>-</v>
-      </c>
-      <c r="D16" t="str">
-        <v>-</v>
-      </c>
-      <c r="E16" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F16" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G16" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H16" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G79"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2508,10 +2482,10 @@
         <v>72</v>
       </c>
       <c r="B73" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
       </c>
       <c r="C73" t="str">
-        <v>197411202025212006</v>
+        <v>198606052024212013</v>
       </c>
       <c r="D73" t="str">
         <v>-</v>
@@ -2520,7 +2494,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F73" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeqYfnPkvY4AdwC8V4UHvNEndqvqZuSZZj_2LqzOVCpFLaKXg/viewform</v>
       </c>
       <c r="G73" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2531,10 +2505,10 @@
         <v>73</v>
       </c>
       <c r="B74" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="C74" t="str">
-        <v>-</v>
+        <v>197411202025212006</v>
       </c>
       <c r="D74" t="str">
         <v>-</v>
@@ -2543,7 +2517,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F74" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="G74" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2554,7 +2528,7 @@
         <v>74</v>
       </c>
       <c r="B75" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C75" t="str">
         <v>-</v>
@@ -2566,7 +2540,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F75" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G75" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2577,7 +2551,7 @@
         <v>75</v>
       </c>
       <c r="B76" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C76" t="str">
         <v>-</v>
@@ -2589,7 +2563,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F76" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G76" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2600,7 +2574,7 @@
         <v>76</v>
       </c>
       <c r="B77" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C77" t="str">
         <v>-</v>
@@ -2612,7 +2586,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F77" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G77" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2623,27 +2597,50 @@
         <v>77</v>
       </c>
       <c r="B78" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C78" t="str">
+        <v>-</v>
+      </c>
+      <c r="D78" t="str">
+        <v>-</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F78" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G78" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C78" t="str">
-        <v>-</v>
-      </c>
-      <c r="D78" t="str">
-        <v>-</v>
-      </c>
-      <c r="E78" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F78" t="str">
+      <c r="C79" t="str">
+        <v>-</v>
+      </c>
+      <c r="D79" t="str">
+        <v>-</v>
+      </c>
+      <c r="E79" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F79" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G78" t="str">
+      <c r="G79" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G78"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G79"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4551,13 +4548,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F73" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeqYfnPkvY4AdwC8V4UHvNEndqvqZuSZZj_2LqzOVCpFLaKXg/viewform</v>
       </c>
       <c r="G73" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H73" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="74">

</xml_diff>

<commit_message>
Update SUYANTI, S.Kom. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="14 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="78 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="13 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="79 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H14"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,10 +442,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>SUYANTI, S.Kom.</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C2" t="str">
-        <v>198206012025212027</v>
+        <v>-</v>
       </c>
       <c r="D2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,7 +494,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,7 +520,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,7 +546,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,7 +572,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,7 +598,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,7 +650,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,7 +676,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,7 +702,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,7 +728,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -754,7 +754,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C14" t="str">
         <v>-</v>
@@ -766,7 +766,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F14" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G14" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -775,42 +775,16 @@
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C15" t="str">
-        <v>-</v>
-      </c>
-      <c r="D15" t="str">
-        <v>-</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F15" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G15" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H15" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H14"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G80"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2528,10 +2502,10 @@
         <v>74</v>
       </c>
       <c r="B75" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>SUYANTI, S.Kom.</v>
       </c>
       <c r="C75" t="str">
-        <v>-</v>
+        <v>198206012025212027</v>
       </c>
       <c r="D75" t="str">
         <v>-</v>
@@ -2540,7 +2514,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F75" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf9LjiU4ww9Pt_xAA8_SHzsqfA3_tENCX11_lJEl64I8BOmrw/viewform</v>
       </c>
       <c r="G75" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2551,7 +2525,7 @@
         <v>75</v>
       </c>
       <c r="B76" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C76" t="str">
         <v>-</v>
@@ -2563,7 +2537,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F76" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G76" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2574,7 +2548,7 @@
         <v>76</v>
       </c>
       <c r="B77" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C77" t="str">
         <v>-</v>
@@ -2586,7 +2560,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F77" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G77" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2597,7 +2571,7 @@
         <v>77</v>
       </c>
       <c r="B78" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C78" t="str">
         <v>-</v>
@@ -2609,7 +2583,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F78" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G78" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2620,27 +2594,50 @@
         <v>78</v>
       </c>
       <c r="B79" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C79" t="str">
+        <v>-</v>
+      </c>
+      <c r="D79" t="str">
+        <v>-</v>
+      </c>
+      <c r="E79" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F79" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G79" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C79" t="str">
-        <v>-</v>
-      </c>
-      <c r="D79" t="str">
-        <v>-</v>
-      </c>
-      <c r="E79" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F79" t="str">
+      <c r="C80" t="str">
+        <v>-</v>
+      </c>
+      <c r="D80" t="str">
+        <v>-</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F80" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G79" t="str">
+      <c r="G80" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G79"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G80"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4600,13 +4597,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F75" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf9LjiU4ww9Pt_xAA8_SHzsqfA3_tENCX11_lJEl64I8BOmrw/viewform</v>
       </c>
       <c r="G75" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H75" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="76">

</xml_diff>

<commit_message>
Update DELIA NURUL AFIFAH, S.Pd Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="13 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="79 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="12 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="80 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H13"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,7 +494,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,7 +520,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,7 +546,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,7 +572,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,7 +598,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,7 +650,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,7 +676,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,7 +702,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -728,7 +728,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C13" t="str">
         <v>-</v>
@@ -740,7 +740,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F13" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G13" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -749,42 +749,16 @@
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C14" t="str">
-        <v>-</v>
-      </c>
-      <c r="D14" t="str">
-        <v>-</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F14" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G14" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H14" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G81"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2525,7 +2499,7 @@
         <v>75</v>
       </c>
       <c r="B76" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
       </c>
       <c r="C76" t="str">
         <v>-</v>
@@ -2537,7 +2511,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F76" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdSOrQUklEFC17Wn9lGEgECqp4VP7B7A76ywjj7aydH8lBisA/viewform</v>
       </c>
       <c r="G76" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2548,7 +2522,7 @@
         <v>76</v>
       </c>
       <c r="B77" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="C77" t="str">
         <v>-</v>
@@ -2560,7 +2534,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F77" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="G77" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2571,7 +2545,7 @@
         <v>77</v>
       </c>
       <c r="B78" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C78" t="str">
         <v>-</v>
@@ -2583,7 +2557,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F78" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G78" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2594,7 +2568,7 @@
         <v>78</v>
       </c>
       <c r="B79" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C79" t="str">
         <v>-</v>
@@ -2606,7 +2580,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F79" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G79" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2617,27 +2591,50 @@
         <v>79</v>
       </c>
       <c r="B80" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C80" t="str">
+        <v>-</v>
+      </c>
+      <c r="D80" t="str">
+        <v>-</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F80" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G80" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C80" t="str">
-        <v>-</v>
-      </c>
-      <c r="D80" t="str">
-        <v>-</v>
-      </c>
-      <c r="E80" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F80" t="str">
+      <c r="C81" t="str">
+        <v>-</v>
+      </c>
+      <c r="D81" t="str">
+        <v>-</v>
+      </c>
+      <c r="E81" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F81" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G80" t="str">
+      <c r="G81" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G80"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G81"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4623,13 +4620,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F76" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdSOrQUklEFC17Wn9lGEgECqp4VP7B7A76ywjj7aydH8lBisA/viewform</v>
       </c>
       <c r="G76" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H76" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="77">

</xml_diff>

<commit_message>
Update EVY KUSHARDIANY, S.Pd Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="12 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="80 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="11 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="81 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H12"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,7 +494,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,7 +520,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,7 +546,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,7 +572,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,7 +598,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,7 +650,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,7 +676,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -702,7 +702,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C12" t="str">
         <v>-</v>
@@ -714,7 +714,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F12" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G12" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -723,42 +723,16 @@
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C13" t="str">
-        <v>-</v>
-      </c>
-      <c r="D13" t="str">
-        <v>-</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F13" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G13" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H13" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G82"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2545,7 +2519,7 @@
         <v>77</v>
       </c>
       <c r="B78" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>EVY KUSHARDIANY, S.Pd</v>
       </c>
       <c r="C78" t="str">
         <v>-</v>
@@ -2557,7 +2531,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F78" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe-iUqyVQtHbDMTfC_7ufj97I7ZUaQqm6A5AEb35wPuyyYjtw/viewform</v>
       </c>
       <c r="G78" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2568,7 +2542,7 @@
         <v>78</v>
       </c>
       <c r="B79" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="C79" t="str">
         <v>-</v>
@@ -2580,7 +2554,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F79" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="G79" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2591,7 +2565,7 @@
         <v>79</v>
       </c>
       <c r="B80" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="C80" t="str">
         <v>-</v>
@@ -2603,7 +2577,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F80" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="G80" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2614,27 +2588,50 @@
         <v>80</v>
       </c>
       <c r="B81" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C81" t="str">
+        <v>-</v>
+      </c>
+      <c r="D81" t="str">
+        <v>-</v>
+      </c>
+      <c r="E81" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F81" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G81" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C81" t="str">
-        <v>-</v>
-      </c>
-      <c r="D81" t="str">
-        <v>-</v>
-      </c>
-      <c r="E81" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F81" t="str">
+      <c r="C82" t="str">
+        <v>-</v>
+      </c>
+      <c r="D82" t="str">
+        <v>-</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F82" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G81" t="str">
+      <c r="G82" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G81"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G82"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4672,13 +4669,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F78" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe-iUqyVQtHbDMTfC_7ufj97I7ZUaQqm6A5AEb35wPuyyYjtw/viewform</v>
       </c>
       <c r="G78" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H78" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="79">

</xml_diff>

<commit_message>
Update BENY WIJAYANTO, SS Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="11 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="81 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="10 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="82 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H11"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>BENY WIJAYANTO, SS</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,7 +494,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,7 +520,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,7 +546,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,7 +572,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,7 +598,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,7 +650,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -676,7 +676,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C11" t="str">
         <v>-</v>
@@ -688,7 +688,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F11" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G11" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -697,42 +697,16 @@
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C12" t="str">
-        <v>-</v>
-      </c>
-      <c r="D12" t="str">
-        <v>-</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F12" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G12" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H12" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G83"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2588,7 +2562,7 @@
         <v>80</v>
       </c>
       <c r="B81" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>BENY WIJAYANTO, SS</v>
       </c>
       <c r="C81" t="str">
         <v>-</v>
@@ -2600,7 +2574,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F81" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdoJpvoEo84fRoDbBiej0XGRlAW9_Ws8hrrM4HYvg1UuY08-A/viewform</v>
       </c>
       <c r="G81" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2611,27 +2585,50 @@
         <v>81</v>
       </c>
       <c r="B82" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C82" t="str">
+        <v>-</v>
+      </c>
+      <c r="D82" t="str">
+        <v>-</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F82" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G82" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C82" t="str">
-        <v>-</v>
-      </c>
-      <c r="D82" t="str">
-        <v>-</v>
-      </c>
-      <c r="E82" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F82" t="str">
+      <c r="C83" t="str">
+        <v>-</v>
+      </c>
+      <c r="D83" t="str">
+        <v>-</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F83" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G82" t="str">
+      <c r="G83" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G82"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G83"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4747,13 +4744,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F81" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdoJpvoEo84fRoDbBiej0XGRlAW9_Ws8hrrM4HYvg1UuY08-A/viewform</v>
       </c>
       <c r="G81" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H81" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="82">

</xml_diff>

<commit_message>
Update NURUL JAMILAH, S.Hum. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="10 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="82 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="9 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="83 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H10"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,7 +494,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,7 +520,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,7 +546,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,7 +572,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,7 +598,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -650,7 +650,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C10" t="str">
         <v>-</v>
@@ -662,7 +662,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F10" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G10" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -671,42 +671,16 @@
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C11" t="str">
-        <v>-</v>
-      </c>
-      <c r="D11" t="str">
-        <v>-</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F11" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G11" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H11" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G84"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2585,7 +2559,7 @@
         <v>81</v>
       </c>
       <c r="B82" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>NURUL JAMILAH, S.Hum.</v>
       </c>
       <c r="C82" t="str">
         <v>-</v>
@@ -2597,7 +2571,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F82" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdvb6XVfWMHXObfg9Qt1qHVFJG91UMNtxkOVmOl8rIiMWyflw/viewform</v>
       </c>
       <c r="G82" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2608,27 +2582,50 @@
         <v>82</v>
       </c>
       <c r="B83" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C83" t="str">
+        <v>-</v>
+      </c>
+      <c r="D83" t="str">
+        <v>-</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F83" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G83" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C83" t="str">
-        <v>-</v>
-      </c>
-      <c r="D83" t="str">
-        <v>-</v>
-      </c>
-      <c r="E83" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F83" t="str">
+      <c r="C84" t="str">
+        <v>-</v>
+      </c>
+      <c r="D84" t="str">
+        <v>-</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F84" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G83" t="str">
+      <c r="G84" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G83"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G84"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4770,13 +4767,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F82" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdvb6XVfWMHXObfg9Qt1qHVFJG91UMNtxkOVmOl8rIiMWyflw/viewform</v>
       </c>
       <c r="G82" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H82" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="83">

</xml_diff>

<commit_message>
Update ENDANG MULYANI, S.Pd. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="9 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="83 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="8 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="84 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,7 +494,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,7 +520,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,7 +546,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,7 +572,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,7 +598,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -624,7 +624,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C9" t="str">
         <v>-</v>
@@ -636,7 +636,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F9" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G9" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -645,42 +645,16 @@
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C10" t="str">
-        <v>-</v>
-      </c>
-      <c r="D10" t="str">
-        <v>-</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F10" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G10" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G85"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2582,7 +2556,7 @@
         <v>82</v>
       </c>
       <c r="B83" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>ENDANG MULYANI, S.Pd.</v>
       </c>
       <c r="C83" t="str">
         <v>-</v>
@@ -2594,7 +2568,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F83" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfIKb0_RA5kQm53YRXY6XxgtyTJnWLyMt8rbszzAxQM5OVfcw/viewform</v>
       </c>
       <c r="G83" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2605,27 +2579,50 @@
         <v>83</v>
       </c>
       <c r="B84" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C84" t="str">
+        <v>-</v>
+      </c>
+      <c r="D84" t="str">
+        <v>-</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F84" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G84" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C84" t="str">
-        <v>-</v>
-      </c>
-      <c r="D84" t="str">
-        <v>-</v>
-      </c>
-      <c r="E84" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F84" t="str">
+      <c r="C85" t="str">
+        <v>-</v>
+      </c>
+      <c r="D85" t="str">
+        <v>-</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F85" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G84" t="str">
+      <c r="G85" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G84"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G85"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4793,13 +4790,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F83" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfIKb0_RA5kQm53YRXY6XxgtyTJnWLyMt8rbszzAxQM5OVfcw/viewform</v>
       </c>
       <c r="G83" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H83" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="84">

</xml_diff>

<commit_message>
Update AGUS IRIANTO, S.Pd. Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="8 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="84 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="7 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="85 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,7 +494,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,7 +520,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,7 +546,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,7 +572,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -598,7 +598,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C8" t="str">
         <v>-</v>
@@ -610,7 +610,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F8" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G8" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -619,42 +619,16 @@
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C9" t="str">
-        <v>-</v>
-      </c>
-      <c r="D9" t="str">
-        <v>-</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F9" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G9" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G86"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2579,7 +2553,7 @@
         <v>83</v>
       </c>
       <c r="B84" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>AGUS IRIANTO, S.Pd</v>
       </c>
       <c r="C84" t="str">
         <v>-</v>
@@ -2591,7 +2565,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F84" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdVc_vPbnRafJ0MFj_iMwBjMvcx-SWamCBstx-Zx0eEWJWpow/viewform</v>
       </c>
       <c r="G84" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2602,27 +2576,50 @@
         <v>84</v>
       </c>
       <c r="B85" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C85" t="str">
+        <v>-</v>
+      </c>
+      <c r="D85" t="str">
+        <v>-</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F85" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G85" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C85" t="str">
-        <v>-</v>
-      </c>
-      <c r="D85" t="str">
-        <v>-</v>
-      </c>
-      <c r="E85" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F85" t="str">
+      <c r="C86" t="str">
+        <v>-</v>
+      </c>
+      <c r="D86" t="str">
+        <v>-</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F86" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G85" t="str">
+      <c r="G86" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G85"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G86"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4816,13 +4813,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F84" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdVc_vPbnRafJ0MFj_iMwBjMvcx-SWamCBstx-Zx0eEWJWpow/viewform</v>
       </c>
       <c r="G84" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H84" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="85">

</xml_diff>

<commit_message>
Update SAMUJI, S.Ag Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="7 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="85 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="6 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="86 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H7"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>SAMUJI, S.Ag</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,7 +494,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,7 +520,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,7 +546,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -572,7 +572,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C7" t="str">
         <v>-</v>
@@ -584,7 +584,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F7" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G7" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -593,42 +593,16 @@
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C8" t="str">
-        <v>-</v>
-      </c>
-      <c r="D8" t="str">
-        <v>-</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F8" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G8" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H8" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G87"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2576,7 +2550,7 @@
         <v>84</v>
       </c>
       <c r="B85" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>SAMUJI, S.Ag</v>
       </c>
       <c r="C85" t="str">
         <v>-</v>
@@ -2588,7 +2562,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F85" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeH_z8k1zjOPd5-ALKEBIwAwnlGEYxrGSwIvU53bPzn4pVj5w/viewform</v>
       </c>
       <c r="G85" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2599,27 +2573,50 @@
         <v>85</v>
       </c>
       <c r="B86" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C86" t="str">
+        <v>-</v>
+      </c>
+      <c r="D86" t="str">
+        <v>-</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F86" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G86" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C86" t="str">
-        <v>-</v>
-      </c>
-      <c r="D86" t="str">
-        <v>-</v>
-      </c>
-      <c r="E86" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F86" t="str">
+      <c r="C87" t="str">
+        <v>-</v>
+      </c>
+      <c r="D87" t="str">
+        <v>-</v>
+      </c>
+      <c r="E87" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F87" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G86" t="str">
+      <c r="G87" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G86"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G87"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4839,13 +4836,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F85" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeH_z8k1zjOPd5-ALKEBIwAwnlGEYxrGSwIvU53bPzn4pVj5w/viewform</v>
       </c>
       <c r="G85" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H85" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="86">

</xml_diff>

<commit_message>
Update IKA UMAYA MARDIANA, S.Pd Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="6 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="86 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="5 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="87 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H6"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
+        <v>AIDA QONITATILLAH, S.Pd</v>
       </c>
       <c r="C2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,7 +494,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,7 +520,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -546,7 +546,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C6" t="str">
         <v>-</v>
@@ -558,7 +558,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F6" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G6" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -567,42 +567,16 @@
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C7" t="str">
-        <v>-</v>
-      </c>
-      <c r="D7" t="str">
-        <v>-</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F7" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G7" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G87"/>
+  <dimension ref="A1:G88"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2573,7 +2547,7 @@
         <v>85</v>
       </c>
       <c r="B86" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
       </c>
       <c r="C86" t="str">
         <v>-</v>
@@ -2585,7 +2559,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F86" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdvQigaXQYmjPnCMU-VOYwFW7tL_wdiEQWFrrEHjwgPUriWVQ/viewform</v>
       </c>
       <c r="G86" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2596,27 +2570,50 @@
         <v>86</v>
       </c>
       <c r="B87" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="C87" t="str">
+        <v>-</v>
+      </c>
+      <c r="D87" t="str">
+        <v>-</v>
+      </c>
+      <c r="E87" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F87" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="G87" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C87" t="str">
-        <v>-</v>
-      </c>
-      <c r="D87" t="str">
-        <v>-</v>
-      </c>
-      <c r="E87" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F87" t="str">
+      <c r="C88" t="str">
+        <v>-</v>
+      </c>
+      <c r="D88" t="str">
+        <v>-</v>
+      </c>
+      <c r="E88" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F88" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G87" t="str">
+      <c r="G88" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G87"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G88"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4862,13 +4859,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F86" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdvQigaXQYmjPnCMU-VOYwFW7tL_wdiEQWFrrEHjwgPUriWVQ/viewform</v>
       </c>
       <c r="G86" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H86" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="87">

</xml_diff>

<commit_message>
Update AIDA QONITATILLAH, S.Pd Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="5 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="87 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="4 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="88 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
+        <v>YULI ANDRIYANI,  S.Pd</v>
       </c>
       <c r="C2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,7 +494,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -520,7 +520,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C5" t="str">
         <v>-</v>
@@ -532,7 +532,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F5" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G5" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -541,42 +541,16 @@
         <v/>
       </c>
     </row>
-    <row r="6">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C6" t="str">
-        <v>-</v>
-      </c>
-      <c r="D6" t="str">
-        <v>-</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F6" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G6" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G89"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2593,27 +2567,50 @@
         <v>87</v>
       </c>
       <c r="B88" t="str">
+        <v>AIDA QONITATILLAH, S.Pd</v>
+      </c>
+      <c r="C88" t="str">
+        <v>-</v>
+      </c>
+      <c r="D88" t="str">
+        <v>-</v>
+      </c>
+      <c r="E88" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F88" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScO5dWuDM9bbQPPRFU7wj2KYpndQWl6MjW4aeBRmp2gd1zsIg/viewform</v>
+      </c>
+      <c r="G88" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C88" t="str">
-        <v>-</v>
-      </c>
-      <c r="D88" t="str">
-        <v>-</v>
-      </c>
-      <c r="E88" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F88" t="str">
+      <c r="C89" t="str">
+        <v>-</v>
+      </c>
+      <c r="D89" t="str">
+        <v>-</v>
+      </c>
+      <c r="E89" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F89" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G88" t="str">
+      <c r="G89" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G88"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G89"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4911,13 +4908,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F88" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScO5dWuDM9bbQPPRFU7wj2KYpndQWl6MjW4aeBRmp2gd1zsIg/viewform</v>
       </c>
       <c r="G88" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H88" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="89">

</xml_diff>

<commit_message>
Update YULI ANDRIYANI, S.Pd Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="4 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="88 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="3 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="89 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H4"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
+        <v>VITA EKA RAHAYU, S.Pd</v>
       </c>
       <c r="C2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -494,7 +494,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C4" t="str">
         <v>-</v>
@@ -506,7 +506,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F4" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G4" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -515,42 +515,16 @@
         <v/>
       </c>
     </row>
-    <row r="5">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C5" t="str">
-        <v>-</v>
-      </c>
-      <c r="D5" t="str">
-        <v>-</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F5" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G5" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G90"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2590,27 +2564,50 @@
         <v>88</v>
       </c>
       <c r="B89" t="str">
+        <v>YULI ANDRIYANI,  S.Pd</v>
+      </c>
+      <c r="C89" t="str">
+        <v>-</v>
+      </c>
+      <c r="D89" t="str">
+        <v>-</v>
+      </c>
+      <c r="E89" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F89" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSetc4dTjz3vYbJvKTJp6Fev2T1Omw8up-uaiqGjN911bM5VhQ/viewform</v>
+      </c>
+      <c r="G89" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C89" t="str">
-        <v>-</v>
-      </c>
-      <c r="D89" t="str">
-        <v>-</v>
-      </c>
-      <c r="E89" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F89" t="str">
+      <c r="C90" t="str">
+        <v>-</v>
+      </c>
+      <c r="D90" t="str">
+        <v>-</v>
+      </c>
+      <c r="E90" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F90" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G89" t="str">
+      <c r="G90" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G89"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G90"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4934,13 +4931,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F89" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSetc4dTjz3vYbJvKTJp6Fev2T1Omw8up-uaiqGjN911bM5VhQ/viewform</v>
       </c>
       <c r="G89" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H89" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="90">

</xml_diff>

<commit_message>
Update VITA EKA RAHAYU, S.Pd Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="3 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="89 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="2 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="90 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H3"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
+        <v>HERI SUGIANTORO, S.Ag</v>
       </c>
       <c r="C2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -468,7 +468,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C3" t="str">
         <v>-</v>
@@ -480,7 +480,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F3" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G3" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -489,42 +489,16 @@
         <v/>
       </c>
     </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C4" t="str">
-        <v>-</v>
-      </c>
-      <c r="D4" t="str">
-        <v>-</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F4" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G4" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G90"/>
+  <dimension ref="A1:G91"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2587,27 +2561,50 @@
         <v>89</v>
       </c>
       <c r="B90" t="str">
+        <v>VITA EKA RAHAYU, S.Pd</v>
+      </c>
+      <c r="C90" t="str">
+        <v>-</v>
+      </c>
+      <c r="D90" t="str">
+        <v>-</v>
+      </c>
+      <c r="E90" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F90" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSegF6rlZWgN9LSLJ-b_0D-Q5rIwzgMKjDZb7njyjkb9m175Cw/viewform</v>
+      </c>
+      <c r="G90" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="C90" t="str">
-        <v>-</v>
-      </c>
-      <c r="D90" t="str">
-        <v>-</v>
-      </c>
-      <c r="E90" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F90" t="str">
+      <c r="C91" t="str">
+        <v>-</v>
+      </c>
+      <c r="D91" t="str">
+        <v>-</v>
+      </c>
+      <c r="E91" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F91" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="G90" t="str">
+      <c r="G91" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G90"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G91"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4957,13 +4954,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F90" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSegF6rlZWgN9LSLJ-b_0D-Q5rIwzgMKjDZb7njyjkb9m175Cw/viewform</v>
       </c>
       <c r="G90" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H90" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="91">

</xml_diff>

<commit_message>
Update HERI SUGIANTORO, S.Ag Google Form URL and update Excel export
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="2 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="90 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="1 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="91 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
       </c>
       <c r="C2" t="str">
         <v>-</v>
@@ -454,7 +454,7 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F2" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="G2" t="str">
         <v>⚠️ Perlu Update URL Panjang</v>
@@ -463,42 +463,16 @@
         <v/>
       </c>
     </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C3" t="str">
-        <v>-</v>
-      </c>
-      <c r="D3" t="str">
-        <v>-</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F3" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G3" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G92"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2602,9 +2576,32 @@
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="str">
+        <v>HERI SUGIANTORO, S.Ag</v>
+      </c>
+      <c r="C92" t="str">
+        <v>-</v>
+      </c>
+      <c r="D92" t="str">
+        <v>-</v>
+      </c>
+      <c r="E92" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F92" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc8hB1Jne1cZcXsMyyah9zkwsD-5XKk5o91E4fXfHBFtfeheg/viewform</v>
+      </c>
+      <c r="G92" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G91"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G92"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5006,13 +5003,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F92" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc8hB1Jne1cZcXsMyyah9zkwsD-5XKk5o91E4fXfHBFtfeheg/viewform</v>
       </c>
       <c r="G92" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H92" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="93">

</xml_diff>

<commit_message>
Update AKBAR ILHAM BAGASKARA PRATAMA, S.T Google Form URL - 100% 92 teachers complete
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="1 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="91 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="0 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="92 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -410,69 +410,16 @@
     <col min="7" max="7" width="30.83203125" customWidth="1"/>
     <col min="8" max="8" width="70.83203125" customWidth="1"/>
   </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>No</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Nama Guru</v>
-      </c>
-      <c r="C1" t="str">
-        <v>NIP</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Kelas Binaan</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Peran</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Shortlink Lama</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Link Baru (docs.google.com/forms/d/e/.../viewform)</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="C2" t="str">
-        <v>-</v>
-      </c>
-      <c r="D2" t="str">
-        <v>-</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="F2" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="G2" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G93"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -2599,9 +2546,32 @@
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
+    <row r="93">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="str">
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
+      </c>
+      <c r="C93" t="str">
+        <v>-</v>
+      </c>
+      <c r="D93" t="str">
+        <v>-</v>
+      </c>
+      <c r="E93" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="F93" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe9TyB66OIRNYnCfIgvtMfcDfVMgbJpD-JByezy7I4Gp20-Bw/viewform</v>
+      </c>
+      <c r="G93" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G92"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G93"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5029,13 +4999,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="F93" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe9TyB66OIRNYnCfIgvtMfcDfVMgbJpD-JByezy7I4Gp20-Bw/viewform</v>
       </c>
       <c r="G93" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="H93" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(firebase): lock target project to form-autoform and update 92 master teachers canonical data
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="0 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="92 Guru Link Valid" sheetId="2" r:id="rId2"/>
-    <sheet name="Master 94 Guru Lengkap" sheetId="3" r:id="rId3"/>
+    <sheet name="52 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="40 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:I53"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -414,24 +414,1551 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>No</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Order</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Nama Guru</v>
+      </c>
+      <c r="D1" t="str">
+        <v>NIP</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Kelas Binaan</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Peran</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Shortlink Lama</v>
+      </c>
+      <c r="H1" t="str">
         <v>Status</v>
       </c>
+      <c r="I1" t="str">
+        <v>Link Baru (docs.google.com/forms/d/e/.../viewform)</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>Semua guru telah valid 100%!</v>
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Drs. MOEHAIMIN</v>
+      </c>
+      <c r="D2" t="str">
+        <v>196709041997031005</v>
+      </c>
+      <c r="E2" t="str">
+        <v>X TEI 2</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G2" t="str">
+        <v>https://forms.gle/ekQJWbDbi72DSNHX9</v>
+      </c>
+      <c r="H2" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>6</v>
+      </c>
+      <c r="C3" t="str">
+        <v>MUNASRI, S.Pd.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>197003282008012013</v>
+      </c>
+      <c r="E3" t="str">
+        <v>X TPM 1</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G3" t="str">
+        <v>https://forms.gle/FzjMqjr2bhYB4mFGA</v>
+      </c>
+      <c r="H3" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>8</v>
+      </c>
+      <c r="C4" t="str">
+        <v>DWI RETNO TUGAS ERNAWATI, S.Pd</v>
+      </c>
+      <c r="D4" t="str">
+        <v>196702142008012009</v>
+      </c>
+      <c r="E4" t="str">
+        <v>X TKR1</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G4" t="str">
+        <v>https://forms.gle/hpaJmjc4TSuY21187</v>
+      </c>
+      <c r="H4" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>9</v>
+      </c>
+      <c r="C5" t="str">
+        <v>KASIATIN, S.Pd</v>
+      </c>
+      <c r="D5" t="str">
+        <v>196908112007012019</v>
+      </c>
+      <c r="E5" t="str">
+        <v>X TKR2</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G5" t="str">
+        <v>https://forms.gle/zCXw2UY7hgtbguuc6</v>
+      </c>
+      <c r="H5" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>10</v>
+      </c>
+      <c r="C6" t="str">
+        <v>SUHARTO DWI SUHERNOWO, ST</v>
+      </c>
+      <c r="D6" t="str">
+        <v>197803262009011007</v>
+      </c>
+      <c r="E6" t="str">
+        <v>X TBKR</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G6" t="str">
+        <v>https://forms.gle/8SMDhw8YpsNPPHPK7</v>
+      </c>
+      <c r="H6" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>11</v>
+      </c>
+      <c r="C7" t="str">
+        <v>ARSYL NOVA ARIRI, ST, M.Pd.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>197811142009012007</v>
+      </c>
+      <c r="E7" t="str">
+        <v>X TSM 1</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G7" t="str">
+        <v>https://forms.gle/sZ2Rff4sL9N4FTrh9</v>
+      </c>
+      <c r="H7" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>16</v>
+      </c>
+      <c r="C8" t="str">
+        <v>WAWAN SISWANTO, SS</v>
+      </c>
+      <c r="D8" t="str">
+        <v>196904012007011025</v>
+      </c>
+      <c r="E8" t="str">
+        <v>XI TAV</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G8" t="str">
+        <v>https://forms.gle/ghNaoJYp7o2SbkjS8</v>
+      </c>
+      <c r="H8" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>17</v>
+      </c>
+      <c r="C9" t="str">
+        <v>R.A. RATNA KARTIKAWATI, S.Pd</v>
+      </c>
+      <c r="D9" t="str">
+        <v>196905132008012023</v>
+      </c>
+      <c r="E9" t="str">
+        <v>XI TEI 1</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G9" t="str">
+        <v>https://forms.gle/bPxWzjgFDES2StGo6</v>
+      </c>
+      <c r="H9" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>19</v>
+      </c>
+      <c r="C10" t="str">
+        <v>NURUL HUDA, ST, M.Si.</v>
+      </c>
+      <c r="D10" t="str">
+        <v>197102162008011009</v>
+      </c>
+      <c r="E10" t="str">
+        <v>XI TPL 1</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G10" t="str">
+        <v>https://forms.gle/aaS7YNQQ97713C18A</v>
+      </c>
+      <c r="H10" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>20</v>
+      </c>
+      <c r="C11" t="str">
+        <v>NUR 'AFIIFAH, M.Pd.</v>
+      </c>
+      <c r="D11" t="str">
+        <v>197208052007012020</v>
+      </c>
+      <c r="E11" t="str">
+        <v>XI TPL 2</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G11" t="str">
+        <v>https://forms.gle/6YPzECievjrGJZBnA</v>
+      </c>
+      <c r="H11" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>21</v>
+      </c>
+      <c r="C12" t="str">
+        <v>TRIBUDI HARTONO, S.Pd</v>
+      </c>
+      <c r="D12" t="str">
+        <v>197511052003121004</v>
+      </c>
+      <c r="E12" t="str">
+        <v>XI TPM 1</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G12" t="str">
+        <v>https://forms.gle/2mog9vghqCw6TSTw7</v>
+      </c>
+      <c r="H12" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>24</v>
+      </c>
+      <c r="C13" t="str">
+        <v>SAMSUL HADI, M.Pd.</v>
+      </c>
+      <c r="D13" t="str">
+        <v>197509262008011011</v>
+      </c>
+      <c r="E13" t="str">
+        <v>XI TKR2</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G13" t="str">
+        <v>https://forms.gle/DSDoMKgI8XxbcPr78</v>
+      </c>
+      <c r="H13" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>25</v>
+      </c>
+      <c r="C14" t="str">
+        <v>HISBULLOH HUDA, M.Pd.</v>
+      </c>
+      <c r="D14" t="str">
+        <v>197602072010011006</v>
+      </c>
+      <c r="E14" t="str">
+        <v>XI TBKR</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G14" t="str">
+        <v>https://forms.gle/jVwhLYXebas1GSZQJ6</v>
+      </c>
+      <c r="H14" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>27</v>
+      </c>
+      <c r="C15" t="str">
+        <v>AGUS HARIYANTO, ST. M.Pd</v>
+      </c>
+      <c r="D15" t="str">
+        <v>198010032010011010</v>
+      </c>
+      <c r="E15" t="str">
+        <v>XI TSM 2</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G15" t="str">
+        <v>https://forms.gle/r3mekFxufrTcJjgRA</v>
+      </c>
+      <c r="H15" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>31</v>
+      </c>
+      <c r="C16" t="str">
+        <v>SIGIT EKO PRAMONO, S.Pd</v>
+      </c>
+      <c r="D16" t="str">
+        <v>198301122009011006</v>
+      </c>
+      <c r="E16" t="str">
+        <v>XII TAV</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G16" t="str">
+        <v>https://forms.gle/PSXtPwi7yQN3Mfi8</v>
+      </c>
+      <c r="H16" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>33</v>
+      </c>
+      <c r="C17" t="str">
+        <v>MOHAMAD ARIEF PRIYO UTOMO, S.Pd</v>
+      </c>
+      <c r="D17" t="str">
+        <v>198209292010011011</v>
+      </c>
+      <c r="E17" t="str">
+        <v>XII TPL 1</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G17" t="str">
+        <v>https://forms.gle/ESlazXu6aQ3PklsD9</v>
+      </c>
+      <c r="H17" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>34</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Dr. RIRIN DIYANNITA SASANTI, M.Pd.</v>
+      </c>
+      <c r="D18" t="str">
+        <v>198212022014062003</v>
+      </c>
+      <c r="E18" t="str">
+        <v>XII TPL 2</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G18" t="str">
+        <v>https://forms.gle/KwfitQjMYbtsnr4UZV6</v>
+      </c>
+      <c r="H18" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>35</v>
+      </c>
+      <c r="C19" t="str">
+        <v>SULIADI, S.Pd</v>
+      </c>
+      <c r="D19" t="str">
+        <v>198403262010011008</v>
+      </c>
+      <c r="E19" t="str">
+        <v>XII TPM 1</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G19" t="str">
+        <v>https://forms.gle/DStwfQQGe3W3gc73A</v>
+      </c>
+      <c r="H19" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>36</v>
+      </c>
+      <c r="C20" t="str">
+        <v>TUTIK QOMARIYAH, S.Si</v>
+      </c>
+      <c r="D20" t="str">
+        <v>198504032010012014</v>
+      </c>
+      <c r="E20" t="str">
+        <v>XII TPM 2</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G20" t="str">
+        <v>https://forms.gle/8Z33XXUnWmhZCY9S9</v>
+      </c>
+      <c r="H20" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>38</v>
+      </c>
+      <c r="C21" t="str">
+        <v>FIRMAN ARDIANSYAH, S.Pd.</v>
+      </c>
+      <c r="D21" t="str">
+        <v>198706172011011010</v>
+      </c>
+      <c r="E21" t="str">
+        <v>XII TKR2</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G21" t="str">
+        <v>https://forms.gle/iGQNqJij1huPUYbk8</v>
+      </c>
+      <c r="H21" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>39</v>
+      </c>
+      <c r="C22" t="str">
+        <v>AZIZ CAHYA PRADANA, S.Pd.</v>
+      </c>
+      <c r="D22" t="str">
+        <v>199103072019031014</v>
+      </c>
+      <c r="E22" t="str">
+        <v>XII TBKR</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G22" t="str">
+        <v>https://forms.gle/RvBNnww2vjNe3gNo76</v>
+      </c>
+      <c r="H22" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>40</v>
+      </c>
+      <c r="C23" t="str">
+        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
+      </c>
+      <c r="D23" t="str">
+        <v>199311072019031004</v>
+      </c>
+      <c r="E23" t="str">
+        <v>XII TSM 1</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G23" t="str">
+        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
+      </c>
+      <c r="H23" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>42</v>
+      </c>
+      <c r="C24" t="str">
+        <v>EFRIDA ISBANDRIYAH, S.T.</v>
+      </c>
+      <c r="D24" t="str">
+        <v>199511062019032010</v>
+      </c>
+      <c r="E24" t="str">
+        <v>XII DKV 1</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G24" t="str">
+        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
+      </c>
+      <c r="H24" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>49</v>
+      </c>
+      <c r="C25" t="str">
+        <v>ETIK SULISTYOWATI, S.Pd.</v>
+      </c>
+      <c r="D25" t="str">
+        <v>198304282022212026</v>
+      </c>
+      <c r="E25" t="str">
+        <v>-</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G25" t="str">
+        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
+      </c>
+      <c r="H25" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>50</v>
+      </c>
+      <c r="C26" t="str">
+        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
+      </c>
+      <c r="D26" t="str">
+        <v>198404192022211018</v>
+      </c>
+      <c r="E26" t="str">
+        <v>-</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G26" t="str">
+        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
+      </c>
+      <c r="H26" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>51</v>
+      </c>
+      <c r="C27" t="str">
+        <v>YAYUK NURNANINGSIH, S.Pd</v>
+      </c>
+      <c r="D27" t="str">
+        <v>198607052022212052</v>
+      </c>
+      <c r="E27" t="str">
+        <v>-</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G27" t="str">
+        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
+      </c>
+      <c r="H27" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>54</v>
+      </c>
+      <c r="C28" t="str">
+        <v>KHOIRUZEN, ST</v>
+      </c>
+      <c r="D28" t="str">
+        <v>197107222023211002</v>
+      </c>
+      <c r="E28" t="str">
+        <v>-</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G28" t="str">
+        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
+      </c>
+      <c r="H28" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>57</v>
+      </c>
+      <c r="C29" t="str">
+        <v>DARIS UMAMI, S.Pd.</v>
+      </c>
+      <c r="D29" t="str">
+        <v>198205042023212026</v>
+      </c>
+      <c r="E29" t="str">
+        <v>-</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G29" t="str">
+        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+      </c>
+      <c r="H29" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>58</v>
+      </c>
+      <c r="C30" t="str">
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+      </c>
+      <c r="D30" t="str">
+        <v>198808072023211018</v>
+      </c>
+      <c r="E30" t="str">
+        <v>-</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G30" t="str">
+        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+      </c>
+      <c r="H30" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>60</v>
+      </c>
+      <c r="C31" t="str">
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+      </c>
+      <c r="D31" t="str">
+        <v>199606142023212026</v>
+      </c>
+      <c r="E31" t="str">
+        <v>-</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G31" t="str">
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+      </c>
+      <c r="H31" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>61</v>
+      </c>
+      <c r="C32" t="str">
+        <v>SUDARMONO, ST</v>
+      </c>
+      <c r="D32" t="str">
+        <v>197206202024211005</v>
+      </c>
+      <c r="E32" t="str">
+        <v>-</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G32" t="str">
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+      </c>
+      <c r="H32" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>63</v>
+      </c>
+      <c r="C33" t="str">
+        <v>ANDRI YUDHI PRASETYO, ST</v>
+      </c>
+      <c r="D33" t="str">
+        <v>197907232024211002</v>
+      </c>
+      <c r="E33" t="str">
+        <v>-</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G33" t="str">
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+      </c>
+      <c r="H33" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>64</v>
+      </c>
+      <c r="C34" t="str">
+        <v>MIANTO, S.Kom.</v>
+      </c>
+      <c r="D34" t="str">
+        <v>198005222024211005</v>
+      </c>
+      <c r="E34" t="str">
+        <v>-</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G34" t="str">
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+      </c>
+      <c r="H34" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>66</v>
+      </c>
+      <c r="C35" t="str">
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+      </c>
+      <c r="D35" t="str">
+        <v>198112142024212008</v>
+      </c>
+      <c r="E35" t="str">
+        <v>-</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G35" t="str">
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+      </c>
+      <c r="H35" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>67</v>
+      </c>
+      <c r="C36" t="str">
+        <v>UMI RU'YATIN, S.Pd</v>
+      </c>
+      <c r="D36" t="str">
+        <v>198201062024212001</v>
+      </c>
+      <c r="E36" t="str">
+        <v>-</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G36" t="str">
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+      </c>
+      <c r="H36" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>68</v>
+      </c>
+      <c r="C37" t="str">
+        <v>YEFI WULANDARI, SE</v>
+      </c>
+      <c r="D37" t="str">
+        <v>198204272024212014</v>
+      </c>
+      <c r="E37" t="str">
+        <v>-</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G37" t="str">
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+      </c>
+      <c r="H37" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>69</v>
+      </c>
+      <c r="C38" t="str">
+        <v>SARI NURHIDAYATI, S.Pd.</v>
+      </c>
+      <c r="D38" t="str">
+        <v>198209202024212008</v>
+      </c>
+      <c r="E38" t="str">
+        <v>-</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G38" t="str">
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+      </c>
+      <c r="H38" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>72</v>
+      </c>
+      <c r="C39" t="str">
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
+      </c>
+      <c r="D39" t="str">
+        <v>198606052024212013</v>
+      </c>
+      <c r="E39" t="str">
+        <v>-</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G39" t="str">
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+      </c>
+      <c r="H39" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>74</v>
+      </c>
+      <c r="C40" t="str">
+        <v>SUYANTI, S.Kom.</v>
+      </c>
+      <c r="D40" t="str">
+        <v>198206012025212027</v>
+      </c>
+      <c r="E40" t="str">
+        <v>-</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G40" t="str">
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+      </c>
+      <c r="H40" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>75</v>
+      </c>
+      <c r="C41" t="str">
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
+      </c>
+      <c r="D41" t="str">
+        <v>-</v>
+      </c>
+      <c r="E41" t="str">
+        <v>-</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G41" t="str">
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+      </c>
+      <c r="H41" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>77</v>
+      </c>
+      <c r="C42" t="str">
+        <v>EVY KUSHARDIANY, S.Pd</v>
+      </c>
+      <c r="D42" t="str">
+        <v>-</v>
+      </c>
+      <c r="E42" t="str">
+        <v>-</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G42" t="str">
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+      </c>
+      <c r="H42" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>80</v>
+      </c>
+      <c r="C43" t="str">
+        <v>BENY WIJAYANTO, SS</v>
+      </c>
+      <c r="D43" t="str">
+        <v>-</v>
+      </c>
+      <c r="E43" t="str">
+        <v>-</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G43" t="str">
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+      </c>
+      <c r="H43" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>81</v>
+      </c>
+      <c r="C44" t="str">
+        <v>NURUL JAMILAH, S.Hum.</v>
+      </c>
+      <c r="D44" t="str">
+        <v>-</v>
+      </c>
+      <c r="E44" t="str">
+        <v>-</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G44" t="str">
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+      </c>
+      <c r="H44" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>82</v>
+      </c>
+      <c r="C45" t="str">
+        <v>ENDANG MULYANI, S.Pd.</v>
+      </c>
+      <c r="D45" t="str">
+        <v>-</v>
+      </c>
+      <c r="E45" t="str">
+        <v>-</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G45" t="str">
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
+      </c>
+      <c r="H45" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>83</v>
+      </c>
+      <c r="C46" t="str">
+        <v>AGUS IRIANTO, S.Pd</v>
+      </c>
+      <c r="D46" t="str">
+        <v>-</v>
+      </c>
+      <c r="E46" t="str">
+        <v>-</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G46" t="str">
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
+      </c>
+      <c r="H46" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>84</v>
+      </c>
+      <c r="C47" t="str">
+        <v>SAMUJI, S.Ag</v>
+      </c>
+      <c r="D47" t="str">
+        <v>-</v>
+      </c>
+      <c r="E47" t="str">
+        <v>-</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G47" t="str">
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+      </c>
+      <c r="H47" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>85</v>
+      </c>
+      <c r="C48" t="str">
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
+      </c>
+      <c r="D48" t="str">
+        <v>-</v>
+      </c>
+      <c r="E48" t="str">
+        <v>-</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G48" t="str">
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+      </c>
+      <c r="H48" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <v>87</v>
+      </c>
+      <c r="C49" t="str">
+        <v>AIDA QONITATILLAH, S.Pd</v>
+      </c>
+      <c r="D49" t="str">
+        <v>-</v>
+      </c>
+      <c r="E49" t="str">
+        <v>-</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G49" t="str">
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+      </c>
+      <c r="H49" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <v>88</v>
+      </c>
+      <c r="C50" t="str">
+        <v>YULI ANDRIYANI,  S.Pd</v>
+      </c>
+      <c r="D50" t="str">
+        <v>-</v>
+      </c>
+      <c r="E50" t="str">
+        <v>-</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G50" t="str">
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+      </c>
+      <c r="H50" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>89</v>
+      </c>
+      <c r="C51" t="str">
+        <v>VITA EKA RAHAYU, S.Pd</v>
+      </c>
+      <c r="D51" t="str">
+        <v>-</v>
+      </c>
+      <c r="E51" t="str">
+        <v>-</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G51" t="str">
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+      </c>
+      <c r="H51" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I51" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52">
+        <v>91</v>
+      </c>
+      <c r="C52" t="str">
+        <v>HERI SUGIANTORO, S.Ag</v>
+      </c>
+      <c r="D52" t="str">
+        <v>-</v>
+      </c>
+      <c r="E52" t="str">
+        <v>-</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G52" t="str">
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+      </c>
+      <c r="H52" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53">
+        <v>92</v>
+      </c>
+      <c r="C53" t="str">
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
+      </c>
+      <c r="D53" t="str">
+        <v>-</v>
+      </c>
+      <c r="E53" t="str">
+        <v>-</v>
+      </c>
+      <c r="F53" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G53" t="str">
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
+      </c>
+      <c r="H53" t="str">
+        <v>⚠️ Perlu Update URL Panjang</v>
+      </c>
+      <c r="I53" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I53"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H41"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -526,22 +2053,22 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" t="str">
-        <v>Drs. MOEHAIMIN</v>
+        <v>DHURROTUL FARIDAH, S.Pd</v>
       </c>
       <c r="D4" t="str">
-        <v>196709041997031005</v>
+        <v>196707142006042005</v>
       </c>
       <c r="E4" t="str">
-        <v>X TEI 2</v>
+        <v>X TPL 1</v>
       </c>
       <c r="F4" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G4" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSez4gjTar2bPbopGm6ErVaBlugek0rGtLocS5azfCCp0MDSIA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeMVWzzDZ53AHLlhGUhchbGtjSPh774mpA2M0nanLr8yfuENQ/viewform</v>
       </c>
       <c r="H4" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -552,22 +2079,22 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" t="str">
-        <v>DHURROTUL FARIDAH, S.Pd</v>
+        <v>SRI WINARTI, S.Pd</v>
       </c>
       <c r="D5" t="str">
-        <v>196707142006042005</v>
+        <v>197307112007012008</v>
       </c>
       <c r="E5" t="str">
-        <v>X TPL 1</v>
+        <v>X TPL 2</v>
       </c>
       <c r="F5" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G5" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeMVWzzDZ53AHLlhGUhchbGtjSPh774mpA2M0nanLr8yfuENQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeDax_Aw_bF0ozmHf2395mK0_9K9QaIgPxKL3Msw8FyZrsKJw/viewform</v>
       </c>
       <c r="H5" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -578,22 +2105,22 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C6" t="str">
-        <v>SRI WINARTI, S.Pd</v>
+        <v>NUR HAYATI, S.Psi, M.Pd.</v>
       </c>
       <c r="D6" t="str">
-        <v>197307112007012008</v>
+        <v>197310152009012003</v>
       </c>
       <c r="E6" t="str">
-        <v>X TPL 2</v>
+        <v>X TPM 2</v>
       </c>
       <c r="F6" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G6" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeDax_Aw_bF0ozmHf2395mK0_9K9QaIgPxKL3Msw8FyZrsKJw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeD8S_m6otgqVphxM7Ux4fGC0wrPh7aPQIKMKg_uaW5tKl42w/viewform</v>
       </c>
       <c r="H6" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -604,22 +2131,22 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C7" t="str">
-        <v>MUNASRI, S.Pd.</v>
+        <v>LAILA FITRIYA, S.Pd.I</v>
       </c>
       <c r="D7" t="str">
-        <v>197003282008012013</v>
+        <v>198506172009012006</v>
       </c>
       <c r="E7" t="str">
-        <v>X TPM 1</v>
+        <v>X TSM 2</v>
       </c>
       <c r="F7" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G7" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfb21fBd9nBHkgM2MBTbSNxfeTgWiXbFL43E9QIZX-zGLzq0g/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfLY_MCLONnsdcq8EWaQayXJZ8_9cAWE7IYKvdeEhm2S0GL9A/viewform</v>
       </c>
       <c r="H7" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -630,22 +2157,22 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C8" t="str">
-        <v>NUR HAYATI, S.Psi, M.Pd.</v>
+        <v>EKA PRAMITASARI, S.Pd. M.Pd.</v>
       </c>
       <c r="D8" t="str">
-        <v>197310152009012003</v>
+        <v>198710302010012005</v>
       </c>
       <c r="E8" t="str">
-        <v>X TPM 2</v>
+        <v>X DKV 1</v>
       </c>
       <c r="F8" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G8" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeD8S_m6otgqVphxM7Ux4fGC0wrPh7aPQIKMKg_uaW5tKl42w/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFNOjWRONIbFscUAVy_gPYaD8c1ehSpS2dTykzwJAn_RUDGw/viewform</v>
       </c>
       <c r="H8" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -656,22 +2183,22 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C9" t="str">
-        <v>DWI RETNO TUGAS ERNAWATI, S.Pd</v>
+        <v>MISBAHUR ROSYIDIN, S.Pd.</v>
       </c>
       <c r="D9" t="str">
-        <v>196702142008012009</v>
+        <v>196802112008011008</v>
       </c>
       <c r="E9" t="str">
-        <v>X TKR1</v>
+        <v>X DKV 2</v>
       </c>
       <c r="F9" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G9" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe-IzLFr71Gdhgd06mjpg2ToTRv1yEa_u8WYc9JsSpikG-NuA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe7MHsr1k2S6apY2TP7L_VulJ7MaQqcKaEsASfOrFV2WfDKSw/viewform</v>
       </c>
       <c r="H9" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -682,22 +2209,22 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C10" t="str">
-        <v>KASIATIN, S.Pd</v>
+        <v>Dra. DYAH CHUSNUL CHOTIMAH</v>
       </c>
       <c r="D10" t="str">
-        <v>196908112007012019</v>
+        <v>196802142007012016</v>
       </c>
       <c r="E10" t="str">
-        <v>X TKR2</v>
+        <v>X DKV 3</v>
       </c>
       <c r="F10" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G10" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf3zl2VpfYKhir9CPBloLYg_xU95VEOzo28tGm9RxY8hWf_8Q/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScl7wa5Pd4jitd3sxqnpqk8tlBpTw-Bx1jl50JwfjGXK_v6ZQ/viewform</v>
       </c>
       <c r="H10" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -708,22 +2235,22 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C11" t="str">
-        <v>SUHARTO DWI SUHERNOWO, ST</v>
+        <v>HERI SUBYANTORO, ST, M.Pd.</v>
       </c>
       <c r="D11" t="str">
-        <v>197803262009011007</v>
+        <v>196910102008011021</v>
       </c>
       <c r="E11" t="str">
-        <v>X TBKR</v>
+        <v>XI TEI 2</v>
       </c>
       <c r="F11" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G11" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdEgJQrGVluy9utuyyeyZ7psIgxX5H9-OTYUG63if-14TLXNg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdHmC5tO01PGYfeU-it6vioHYot6MO4Enq9Nbw1oA8DLgGJog/viewform</v>
       </c>
       <c r="H11" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -734,22 +2261,22 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C12" t="str">
-        <v>ARSYL NOVA ARIRI, ST, M.Pd.</v>
+        <v>DEDY HENDRIANA, S.Pd. M.Pd.</v>
       </c>
       <c r="D12" t="str">
-        <v>197811142009012007</v>
+        <v>197904072010011002</v>
       </c>
       <c r="E12" t="str">
-        <v>X TSM 1</v>
+        <v>XI TPM 2</v>
       </c>
       <c r="F12" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G12" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeYIRHhpNjh1FmGBMMlPQPwu6jnRfYLe__qCNtcIES7ZefQvQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSecBLlEDfTwutpIfoRhoxlk9TykVgqtywzFBczl8dG7w3nLgg/viewform</v>
       </c>
       <c r="H12" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -760,22 +2287,22 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C13" t="str">
-        <v>LAILA FITRIYA, S.Pd.I</v>
+        <v>AGUS HIDAYAT, S.Pd</v>
       </c>
       <c r="D13" t="str">
-        <v>198506172009012006</v>
+        <v>196907272007011018</v>
       </c>
       <c r="E13" t="str">
-        <v>X TSM 2</v>
+        <v>XI TKR1</v>
       </c>
       <c r="F13" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G13" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfLY_MCLONnsdcq8EWaQayXJZ8_9cAWE7IYKvdeEhm2S0GL9A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4cLrLtqJrSQCZlTZvjVDTqCqwr0Ezvo9jj1xlEEVIA1TgLQ/viewform</v>
       </c>
       <c r="H13" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -786,22 +2313,22 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="C14" t="str">
-        <v>EKA PRAMITASARI, S.Pd. M.Pd.</v>
+        <v>DWI SANTOSO, S.Pd</v>
       </c>
       <c r="D14" t="str">
-        <v>198710302010012005</v>
+        <v>197908082006041019</v>
       </c>
       <c r="E14" t="str">
-        <v>X DKV 1</v>
+        <v>XI TSM 1</v>
       </c>
       <c r="F14" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G14" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFNOjWRONIbFscUAVy_gPYaD8c1ehSpS2dTykzwJAn_RUDGw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc3pPlG2fg8z9mrKutplhHQxr-oLEDr0OrG2tbckE403avEiw/viewform</v>
       </c>
       <c r="H14" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -812,22 +2339,22 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="C15" t="str">
-        <v>MISBAHUR ROSYIDIN, S.Pd.</v>
+        <v>ZAINUL ARIFIN, M.Pd.</v>
       </c>
       <c r="D15" t="str">
-        <v>196802112008011008</v>
+        <v>198210112010011009</v>
       </c>
       <c r="E15" t="str">
-        <v>X DKV 2</v>
+        <v>XI DKV 1</v>
       </c>
       <c r="F15" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G15" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe7MHsr1k2S6apY2TP7L_VulJ7MaQqcKaEsASfOrFV2WfDKSw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc1knrp09uNEhFpIHg2HnTVcw1HE0-aoR7bacYb4cXIsHAleQ/viewform</v>
       </c>
       <c r="H15" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -838,22 +2365,22 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="C16" t="str">
-        <v>Dra. DYAH CHUSNUL CHOTIMAH</v>
+        <v>BAMBANG SUJATMIKO, S.Pd</v>
       </c>
       <c r="D16" t="str">
-        <v>196802142007012016</v>
+        <v>198211222006041009</v>
       </c>
       <c r="E16" t="str">
-        <v>X DKV 3</v>
+        <v>XI DKV 2</v>
       </c>
       <c r="F16" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G16" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScl7wa5Pd4jitd3sxqnpqk8tlBpTw-Bx1jl50JwfjGXK_v6ZQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYyOzS9TUnTH79m-niYDGHWqxmhbtWyxFehMM6Td06hqBh1A/viewform</v>
       </c>
       <c r="H16" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -864,22 +2391,22 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C17" t="str">
-        <v>WAWAN SISWANTO, SS</v>
+        <v>HARTONO, S.Pd</v>
       </c>
       <c r="D17" t="str">
-        <v>196904012007011025</v>
+        <v>198205122009011009</v>
       </c>
       <c r="E17" t="str">
-        <v>XI TAV</v>
+        <v>XI DKV 3</v>
       </c>
       <c r="F17" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G17" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYaU-G7gAyHPvwtYTw67xI_BcR43imBjiP3RB58jOjnU1XeQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSczcB1-HoNbq4XLNVL6d22ps_sHXrr_yAMrTdi-SXUI9dyDiA/viewform</v>
       </c>
       <c r="H17" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -890,22 +2417,22 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C18" t="str">
-        <v>R.A. RATNA KARTIKAWATI, S.Pd</v>
+        <v>AGUNG RAKHMANDA, S.Kom.</v>
       </c>
       <c r="D18" t="str">
-        <v>196905132008012023</v>
+        <v>198303272009031002</v>
       </c>
       <c r="E18" t="str">
-        <v>XI TEI 1</v>
+        <v>XII TEI 1</v>
       </c>
       <c r="F18" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G18" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSd2bLbWa9Pca9QT7JTzZAnSSDZOakUabHJxB_JnNT3CQEv4gA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe3WNA-vHAA16POkCpcvBUl2Kc57HtjVXCkAQEm_mMB69NPow/viewform</v>
       </c>
       <c r="H18" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -916,22 +2443,22 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="C19" t="str">
-        <v>HERI SUBYANTORO, ST, M.Pd.</v>
+        <v>IMAM SUFERI, ST.</v>
       </c>
       <c r="D19" t="str">
-        <v>196910102008011021</v>
+        <v>197712302008011013</v>
       </c>
       <c r="E19" t="str">
-        <v>XI TEI 2</v>
+        <v>XII TKR1</v>
       </c>
       <c r="F19" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G19" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdHmC5tO01PGYfeU-it6vioHYot6MO4Enq9Nbw1oA8DLgGJog/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe8sSOVeefXvVkHVMUzrTdYO8RrfqdFwT5AQRWWlJ3ZzJAluQ/viewform</v>
       </c>
       <c r="H19" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -942,22 +2469,22 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="C20" t="str">
-        <v>NURUL HUDA, ST, M.Si.</v>
+        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
       </c>
       <c r="D20" t="str">
-        <v>197102162008011009</v>
+        <v>199410092019032012</v>
       </c>
       <c r="E20" t="str">
-        <v>XI TPL 1</v>
+        <v>XII TSM 2</v>
       </c>
       <c r="F20" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G20" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSd4Etrlv7kK9gUfKVu1OwwyBhjLAn4-l3PArWhzLxF13MmmVw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
       </c>
       <c r="H20" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -968,22 +2495,22 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="C21" t="str">
-        <v>NUR 'AFIIFAH, M.Pd.</v>
+        <v>SOTYA BAYUNTARA, S.Pd.</v>
       </c>
       <c r="D21" t="str">
-        <v>197208052007012020</v>
+        <v>196906252022211004</v>
       </c>
       <c r="E21" t="str">
-        <v>XI TPL 2</v>
+        <v>XII DKV 2</v>
       </c>
       <c r="F21" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G21" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScZ2l8R4TTNeJdfXVZvYAgc3WGgT9QtEVz0-ANUsebuRgsWsQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
       </c>
       <c r="H21" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -994,22 +2521,22 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="C22" t="str">
-        <v>TRIBUDI HARTONO, S.Pd</v>
+        <v>SRIGATI, SE</v>
       </c>
       <c r="D22" t="str">
-        <v>197511052003121004</v>
+        <v>197505052022212013</v>
       </c>
       <c r="E22" t="str">
-        <v>XI TPM 1</v>
+        <v>XII DKV 3</v>
       </c>
       <c r="F22" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G22" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdcvHzA1p4OhUC9iXA97o8okqRsjziPMeWoPw6g-Nvt7Pr9jg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
       </c>
       <c r="H22" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1020,22 +2547,22 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="C23" t="str">
-        <v>DEDY HENDRIANA, S.Pd. M.Pd.</v>
+        <v>HARI PURWANTO, ST</v>
       </c>
       <c r="D23" t="str">
-        <v>197904072010011002</v>
+        <v>197711242022211006</v>
       </c>
       <c r="E23" t="str">
-        <v>XI TPM 2</v>
+        <v>-</v>
       </c>
       <c r="F23" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G23" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSecBLlEDfTwutpIfoRhoxlk9TykVgqtywzFBczl8dG7w3nLgg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
       </c>
       <c r="H23" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1046,22 +2573,22 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="C24" t="str">
-        <v>AGUS HIDAYAT, S.Pd</v>
+        <v>ESTI WIDHIARNI, S.T</v>
       </c>
       <c r="D24" t="str">
-        <v>196907272007011018</v>
+        <v>197906032022212022</v>
       </c>
       <c r="E24" t="str">
-        <v>XI TKR1</v>
+        <v>-</v>
       </c>
       <c r="F24" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G24" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4cLrLtqJrSQCZlTZvjVDTqCqwr0Ezvo9jj1xlEEVIA1TgLQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
       </c>
       <c r="H24" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1072,22 +2599,22 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="C25" t="str">
-        <v>SAMSUL HADI, M.Pd.</v>
+        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
       </c>
       <c r="D25" t="str">
-        <v>197509262008011011</v>
+        <v>198109092022211004</v>
       </c>
       <c r="E25" t="str">
-        <v>XI TKR2</v>
+        <v>XII TEI 2</v>
       </c>
       <c r="F25" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G25" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdoHRTHs-yCXOAaQukleNcx5jWI79dOK6qbeeCW4p45bJ9CLg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
       </c>
       <c r="H25" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1098,22 +2625,22 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="C26" t="str">
-        <v>HISBULLOH HUDA, M.Pd.</v>
+        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
       </c>
       <c r="D26" t="str">
-        <v>197602072010011006</v>
+        <v>198212102022211017</v>
       </c>
       <c r="E26" t="str">
-        <v>XI TBKR</v>
+        <v>-</v>
       </c>
       <c r="F26" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G26" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSftHQdc5-VZ5uwLLimFvRnkwycT7Ys50sjgRzMN-ALHGSjCqA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
       </c>
       <c r="H26" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1124,22 +2651,22 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>26</v>
+        <v>52</v>
       </c>
       <c r="C27" t="str">
-        <v>DWI SANTOSO, S.Pd</v>
+        <v>KHOIRUL AMIN, S.Pd</v>
       </c>
       <c r="D27" t="str">
-        <v>197908082006041019</v>
+        <v>198701192022211009</v>
       </c>
       <c r="E27" t="str">
-        <v>XI TSM 1</v>
+        <v>-</v>
       </c>
       <c r="F27" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G27" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc3pPlG2fg8z9mrKutplhHQxr-oLEDr0OrG2tbckE403avEiw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
       </c>
       <c r="H27" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1150,22 +2677,22 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="C28" t="str">
-        <v>AGUS HARIYANTO, ST. M.Pd</v>
+        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
       </c>
       <c r="D28" t="str">
-        <v>198010032010011010</v>
+        <v>198712072022211015</v>
       </c>
       <c r="E28" t="str">
-        <v>XI TSM 2</v>
+        <v>-</v>
       </c>
       <c r="F28" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G28" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNEYg6DAPuUemLNfKalqh5_nN6m2oxlOxSvPG1Fu55a4gqNA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
       </c>
       <c r="H28" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1176,22 +2703,22 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="C29" t="str">
-        <v>ZAINUL ARIFIN, M.Pd.</v>
+        <v>HEPPY LUCKITO, SST</v>
       </c>
       <c r="D29" t="str">
-        <v>198210112010011009</v>
+        <v>198110272023211008</v>
       </c>
       <c r="E29" t="str">
-        <v>XI DKV 1</v>
+        <v>-</v>
       </c>
       <c r="F29" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G29" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc1knrp09uNEhFpIHg2HnTVcw1HE0-aoR7bacYb4cXIsHAleQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
       </c>
       <c r="H29" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1202,22 +2729,22 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="C30" t="str">
-        <v>BAMBANG SUJATMIKO, S.Pd</v>
+        <v>SRI PURWANINGSIH, S.Pd</v>
       </c>
       <c r="D30" t="str">
-        <v>198211222006041009</v>
+        <v>198203022023212020</v>
       </c>
       <c r="E30" t="str">
-        <v>XI DKV 2</v>
+        <v>-</v>
       </c>
       <c r="F30" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G30" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYyOzS9TUnTH79m-niYDGHWqxmhbtWyxFehMM6Td06hqBh1A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
       </c>
       <c r="H30" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1228,22 +2755,22 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="C31" t="str">
-        <v>HARTONO, S.Pd</v>
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
       </c>
       <c r="D31" t="str">
-        <v>198205122009011009</v>
+        <v>199410282023211012</v>
       </c>
       <c r="E31" t="str">
-        <v>XI DKV 3</v>
+        <v>-</v>
       </c>
       <c r="F31" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G31" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSczcB1-HoNbq4XLNVL6d22ps_sHXrr_yAMrTdi-SXUI9dyDiA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
       </c>
       <c r="H31" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1254,22 +2781,22 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="C32" t="str">
-        <v>SIGIT EKO PRAMONO, S.Pd</v>
+        <v>ROHMAN, S.T.</v>
       </c>
       <c r="D32" t="str">
-        <v>198301122009011006</v>
+        <v>197509042024211002</v>
       </c>
       <c r="E32" t="str">
-        <v>XII TAV</v>
+        <v>-</v>
       </c>
       <c r="F32" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G32" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdRlmK9kl1qIAOcGpf1Uu18upIQ0GWK8VkTv12k_6AEAERRMQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
       </c>
       <c r="H32" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1280,22 +2807,22 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>32</v>
+        <v>65</v>
       </c>
       <c r="C33" t="str">
-        <v>AGUNG RAKHMANDA, S.Kom.</v>
+        <v>HARIS ALI MUHYIDIN, S.T</v>
       </c>
       <c r="D33" t="str">
-        <v>198303272009031002</v>
+        <v>198103052024211008</v>
       </c>
       <c r="E33" t="str">
-        <v>XII TEI 1</v>
+        <v>-</v>
       </c>
       <c r="F33" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G33" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe3WNA-vHAA16POkCpcvBUl2Kc57HtjVXCkAQEm_mMB69NPow/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
       </c>
       <c r="H33" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1306,22 +2833,22 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="C34" t="str">
-        <v>MOHAMAD ARIEF PRIYO UTOMO, S.Pd</v>
+        <v>SUWOYO, S.Kom</v>
       </c>
       <c r="D34" t="str">
-        <v>198209292010011011</v>
+        <v>198403072024211011</v>
       </c>
       <c r="E34" t="str">
-        <v>XII TPL 1</v>
+        <v>-</v>
       </c>
       <c r="F34" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G34" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdPW1l4LaclpGdRqS2jqaCtnP9mivQff9TM2a9if71auoCj6g/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
       </c>
       <c r="H34" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1332,22 +2859,22 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="C35" t="str">
-        <v>Dr. RIRIN DIYANNITA SASANTI, M.Pd.</v>
+        <v>AAN SUSANTO, S.Pd.</v>
       </c>
       <c r="D35" t="str">
-        <v>198212022014062003</v>
+        <v>198410082024211016</v>
       </c>
       <c r="E35" t="str">
-        <v>XII TPL 2</v>
+        <v>-</v>
       </c>
       <c r="F35" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G35" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSejtfmzSD3f24E8Z4AXVPgC0RTs8brRuZ_KCxV9-lmsq4C5iQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
       </c>
       <c r="H35" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1358,22 +2885,22 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>35</v>
+        <v>73</v>
       </c>
       <c r="C36" t="str">
-        <v>SULIADI, S.Pd</v>
+        <v>NUR FAUZIYAH, S.Ag.</v>
       </c>
       <c r="D36" t="str">
-        <v>198403262010011008</v>
+        <v>197411202025212006</v>
       </c>
       <c r="E36" t="str">
-        <v>XII TPM 1</v>
+        <v>-</v>
       </c>
       <c r="F36" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G36" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdaT-LhGEwSzPtm9G3LL6KRs-gFmbNF2uiIykR7J7HDmdC2uQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
       </c>
       <c r="H36" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1384,22 +2911,22 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="C37" t="str">
-        <v>TUTIK QOMARIYAH, S.Si</v>
+        <v>CAHYA ISKANDAR, S.T</v>
       </c>
       <c r="D37" t="str">
-        <v>198504032010012014</v>
+        <v>-</v>
       </c>
       <c r="E37" t="str">
-        <v>XII TPM 2</v>
+        <v>-</v>
       </c>
       <c r="F37" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G37" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFjcTg73409mYsq9RTVwH8IBBBz5ya0_y6K1t74WjfpPWMhA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
       </c>
       <c r="H37" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1410,22 +2937,22 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>37</v>
+        <v>78</v>
       </c>
       <c r="C38" t="str">
-        <v>IMAM SUFERI, ST.</v>
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
       </c>
       <c r="D38" t="str">
-        <v>197712302008011013</v>
+        <v>-</v>
       </c>
       <c r="E38" t="str">
-        <v>XII TKR1</v>
+        <v>-</v>
       </c>
       <c r="F38" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G38" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe8sSOVeefXvVkHVMUzrTdYO8RrfqdFwT5AQRWWlJ3ZzJAluQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
       </c>
       <c r="H38" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1436,22 +2963,22 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>38</v>
+        <v>79</v>
       </c>
       <c r="C39" t="str">
-        <v>FIRMAN ARDIANSYAH, S.Pd.</v>
+        <v>YUNIAR DWI LISTYANTO, ST</v>
       </c>
       <c r="D39" t="str">
-        <v>198706172011011010</v>
+        <v>-</v>
       </c>
       <c r="E39" t="str">
-        <v>XII TKR2</v>
+        <v>-</v>
       </c>
       <c r="F39" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G39" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScUo8DXP3Tp38IveX-Bq5eu4aD3aJBRVAjTA8896rGx1WUsNQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
       </c>
       <c r="H39" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1462,22 +2989,22 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>39</v>
+        <v>86</v>
       </c>
       <c r="C40" t="str">
-        <v>AZIZ CAHYA PRADANA, S.Pd.</v>
+        <v>NUR KHOLIFAH, S.Pd.</v>
       </c>
       <c r="D40" t="str">
-        <v>199103072019031014</v>
+        <v>-</v>
       </c>
       <c r="E40" t="str">
-        <v>XII TBKR</v>
+        <v>-</v>
       </c>
       <c r="F40" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G40" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScKk6RYj6qkwSYwir5SH2zma20b5qhM4boLx8UqeQ19DUTIfA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
       </c>
       <c r="H40" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -1488,1389 +3015,37 @@
         <v>40</v>
       </c>
       <c r="B41">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="C41" t="str">
-        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
+        <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
       <c r="D41" t="str">
-        <v>199311072019031004</v>
+        <v>-</v>
       </c>
       <c r="E41" t="str">
-        <v>XII TSM 1</v>
+        <v>-</v>
       </c>
       <c r="F41" t="str">
-        <v>Walikelas</v>
+        <v>Guru Pengajar</v>
       </c>
       <c r="G41" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSczNF2YAQXf9165kZ-FthvzailwmMrM-uSTecJzWHq0JCEldQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
       <c r="H41" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42">
-        <v>41</v>
-      </c>
-      <c r="B42">
-        <v>41</v>
-      </c>
-      <c r="C42" t="str">
-        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
-      </c>
-      <c r="D42" t="str">
-        <v>199410092019032012</v>
-      </c>
-      <c r="E42" t="str">
-        <v>XII TSM 2</v>
-      </c>
-      <c r="F42" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G42" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
-      </c>
-      <c r="H42" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43">
-        <v>42</v>
-      </c>
-      <c r="B43">
-        <v>42</v>
-      </c>
-      <c r="C43" t="str">
-        <v>EFRIDA ISBANDRIYAH, S.T.</v>
-      </c>
-      <c r="D43" t="str">
-        <v>199511062019032010</v>
-      </c>
-      <c r="E43" t="str">
-        <v>XII DKV 1</v>
-      </c>
-      <c r="F43" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G43" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4Z31ED-5m9YP8u3CbOt0PWt94nwzJafZSig17a3DoqRlpCQ/viewform</v>
-      </c>
-      <c r="H43" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44">
-        <v>43</v>
-      </c>
-      <c r="B44">
-        <v>43</v>
-      </c>
-      <c r="C44" t="str">
-        <v>SOTYA BAYUNTARA, S.Pd.</v>
-      </c>
-      <c r="D44" t="str">
-        <v>196906252022211004</v>
-      </c>
-      <c r="E44" t="str">
-        <v>XII DKV 2</v>
-      </c>
-      <c r="F44" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G44" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
-      </c>
-      <c r="H44" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45">
-        <v>44</v>
-      </c>
-      <c r="B45">
-        <v>44</v>
-      </c>
-      <c r="C45" t="str">
-        <v>SRIGATI, SE</v>
-      </c>
-      <c r="D45" t="str">
-        <v>197505052022212013</v>
-      </c>
-      <c r="E45" t="str">
-        <v>XII DKV 3</v>
-      </c>
-      <c r="F45" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G45" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
-      </c>
-      <c r="H45" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46">
-        <v>45</v>
-      </c>
-      <c r="B46">
-        <v>45</v>
-      </c>
-      <c r="C46" t="str">
-        <v>HARI PURWANTO, ST</v>
-      </c>
-      <c r="D46" t="str">
-        <v>197711242022211006</v>
-      </c>
-      <c r="E46" t="str">
-        <v>-</v>
-      </c>
-      <c r="F46" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G46" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
-      </c>
-      <c r="H46" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47">
-        <v>46</v>
-      </c>
-      <c r="B47">
-        <v>46</v>
-      </c>
-      <c r="C47" t="str">
-        <v>ESTI WIDHIARNI, S.T</v>
-      </c>
-      <c r="D47" t="str">
-        <v>197906032022212022</v>
-      </c>
-      <c r="E47" t="str">
-        <v>-</v>
-      </c>
-      <c r="F47" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G47" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
-      </c>
-      <c r="H47" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48">
-        <v>47</v>
-      </c>
-      <c r="B48">
-        <v>47</v>
-      </c>
-      <c r="C48" t="str">
-        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
-      </c>
-      <c r="D48" t="str">
-        <v>198109092022211004</v>
-      </c>
-      <c r="E48" t="str">
-        <v>XII TEI 2</v>
-      </c>
-      <c r="F48" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G48" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
-      </c>
-      <c r="H48" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49">
-        <v>48</v>
-      </c>
-      <c r="B49">
-        <v>48</v>
-      </c>
-      <c r="C49" t="str">
-        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
-      </c>
-      <c r="D49" t="str">
-        <v>198212102022211017</v>
-      </c>
-      <c r="E49" t="str">
-        <v>-</v>
-      </c>
-      <c r="F49" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G49" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
-      </c>
-      <c r="H49" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50">
-        <v>49</v>
-      </c>
-      <c r="B50">
-        <v>49</v>
-      </c>
-      <c r="C50" t="str">
-        <v>ETIK SULISTYOWATI, S.Pd.</v>
-      </c>
-      <c r="D50" t="str">
-        <v>198304282022212026</v>
-      </c>
-      <c r="E50" t="str">
-        <v>-</v>
-      </c>
-      <c r="F50" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G50" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdUwe7or4Y0G1-MxBUlVlO5CHIQU7My-9_OxXNA87sJhdXBZA/viewform</v>
-      </c>
-      <c r="H50" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51">
-        <v>50</v>
-      </c>
-      <c r="B51">
-        <v>50</v>
-      </c>
-      <c r="C51" t="str">
-        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
-      </c>
-      <c r="D51" t="str">
-        <v>198404192022211018</v>
-      </c>
-      <c r="E51" t="str">
-        <v>-</v>
-      </c>
-      <c r="F51" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G51" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe4vBzUIUsBJNN39klf82XO2jf2iJXqigXNdhNMkSI7-lcsEw/viewform</v>
-      </c>
-      <c r="H51" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52">
-        <v>51</v>
-      </c>
-      <c r="B52">
-        <v>51</v>
-      </c>
-      <c r="C52" t="str">
-        <v>YAYUK NURNANINGSIH, S.Pd</v>
-      </c>
-      <c r="D52" t="str">
-        <v>198607052022212052</v>
-      </c>
-      <c r="E52" t="str">
-        <v>-</v>
-      </c>
-      <c r="F52" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G52" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFgOYb82K7kj70lOwDL28zNyaVYlK3CX9WHttQtR-KGtb2Mg/viewform</v>
-      </c>
-      <c r="H52" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53">
-        <v>52</v>
-      </c>
-      <c r="B53">
-        <v>52</v>
-      </c>
-      <c r="C53" t="str">
-        <v>KHOIRUL AMIN, S.Pd</v>
-      </c>
-      <c r="D53" t="str">
-        <v>198701192022211009</v>
-      </c>
-      <c r="E53" t="str">
-        <v>-</v>
-      </c>
-      <c r="F53" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G53" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
-      </c>
-      <c r="H53" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54">
-        <v>53</v>
-      </c>
-      <c r="B54">
-        <v>53</v>
-      </c>
-      <c r="C54" t="str">
-        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
-      </c>
-      <c r="D54" t="str">
-        <v>198712072022211015</v>
-      </c>
-      <c r="E54" t="str">
-        <v>-</v>
-      </c>
-      <c r="F54" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G54" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
-      </c>
-      <c r="H54" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55">
-        <v>54</v>
-      </c>
-      <c r="B55">
-        <v>54</v>
-      </c>
-      <c r="C55" t="str">
-        <v>KHOIRUZEN, ST</v>
-      </c>
-      <c r="D55" t="str">
-        <v>197107222023211002</v>
-      </c>
-      <c r="E55" t="str">
-        <v>-</v>
-      </c>
-      <c r="F55" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G55" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
-      </c>
-      <c r="H55" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56">
-        <v>55</v>
-      </c>
-      <c r="B56">
-        <v>55</v>
-      </c>
-      <c r="C56" t="str">
-        <v>HEPPY LUCKITO, SST</v>
-      </c>
-      <c r="D56" t="str">
-        <v>198110272023211008</v>
-      </c>
-      <c r="E56" t="str">
-        <v>-</v>
-      </c>
-      <c r="F56" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G56" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
-      </c>
-      <c r="H56" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57">
-        <v>56</v>
-      </c>
-      <c r="B57">
-        <v>56</v>
-      </c>
-      <c r="C57" t="str">
-        <v>SRI PURWANINGSIH, S.Pd</v>
-      </c>
-      <c r="D57" t="str">
-        <v>198203022023212020</v>
-      </c>
-      <c r="E57" t="str">
-        <v>-</v>
-      </c>
-      <c r="F57" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G57" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
-      </c>
-      <c r="H57" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58">
-        <v>57</v>
-      </c>
-      <c r="B58">
-        <v>57</v>
-      </c>
-      <c r="C58" t="str">
-        <v>DARIS UMAMI, S.Pd.</v>
-      </c>
-      <c r="D58" t="str">
-        <v>198205042023212026</v>
-      </c>
-      <c r="E58" t="str">
-        <v>-</v>
-      </c>
-      <c r="F58" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G58" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSety3ZkhI7AVI8v-VQRPaTax5rflclagowfHbFtFrNjSSZNHg/viewform</v>
-      </c>
-      <c r="H58" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59">
-        <v>58</v>
-      </c>
-      <c r="B59">
-        <v>58</v>
-      </c>
-      <c r="C59" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
-      </c>
-      <c r="D59" t="str">
-        <v>198808072023211018</v>
-      </c>
-      <c r="E59" t="str">
-        <v>-</v>
-      </c>
-      <c r="F59" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G59" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScLoRQkJKESig6rf-hq4Hq-9UsA2rpsBuDhVX6113r1OrYeLw/viewform</v>
-      </c>
-      <c r="H59" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60">
-        <v>59</v>
-      </c>
-      <c r="B60">
-        <v>59</v>
-      </c>
-      <c r="C60" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
-      </c>
-      <c r="D60" t="str">
-        <v>199410282023211012</v>
-      </c>
-      <c r="E60" t="str">
-        <v>-</v>
-      </c>
-      <c r="F60" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G60" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
-      </c>
-      <c r="H60" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61">
-        <v>60</v>
-      </c>
-      <c r="B61">
-        <v>60</v>
-      </c>
-      <c r="C61" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
-      </c>
-      <c r="D61" t="str">
-        <v>199606142023212026</v>
-      </c>
-      <c r="E61" t="str">
-        <v>-</v>
-      </c>
-      <c r="F61" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G61" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeBM6FY62A84yCrWK-O8XZ_ehP9cDsy6qNu0MHDEXeCZlsATA/viewform</v>
-      </c>
-      <c r="H61" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62">
-        <v>61</v>
-      </c>
-      <c r="B62">
-        <v>61</v>
-      </c>
-      <c r="C62" t="str">
-        <v>SUDARMONO, ST</v>
-      </c>
-      <c r="D62" t="str">
-        <v>197206202024211005</v>
-      </c>
-      <c r="E62" t="str">
-        <v>-</v>
-      </c>
-      <c r="F62" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G62" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGR9KnW2FGcWAVjUfLzEpLkENkH6O1XpstPv9041fsBK4r7A/viewform</v>
-      </c>
-      <c r="H62" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63">
-        <v>62</v>
-      </c>
-      <c r="B63">
-        <v>62</v>
-      </c>
-      <c r="C63" t="str">
-        <v>ROHMAN, S.T.</v>
-      </c>
-      <c r="D63" t="str">
-        <v>197509042024211002</v>
-      </c>
-      <c r="E63" t="str">
-        <v>-</v>
-      </c>
-      <c r="F63" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G63" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
-      </c>
-      <c r="H63" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64">
-        <v>63</v>
-      </c>
-      <c r="B64">
-        <v>63</v>
-      </c>
-      <c r="C64" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
-      </c>
-      <c r="D64" t="str">
-        <v>197907232024211002</v>
-      </c>
-      <c r="E64" t="str">
-        <v>-</v>
-      </c>
-      <c r="F64" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G64" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4F9PoN3h1R3EmQmS-KTPCmUB2ghq3K7N1e00Ni4NE30hESw/viewform</v>
-      </c>
-      <c r="H64" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65">
-        <v>64</v>
-      </c>
-      <c r="B65">
-        <v>64</v>
-      </c>
-      <c r="C65" t="str">
-        <v>MIANTO, S.Kom.</v>
-      </c>
-      <c r="D65" t="str">
-        <v>198005222024211005</v>
-      </c>
-      <c r="E65" t="str">
-        <v>-</v>
-      </c>
-      <c r="F65" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G65" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSee6t_4PgxzeHNbhtwqZROlfNE9Iz6Sf5QJvGMjzkmAGvhcAw/viewform</v>
-      </c>
-      <c r="H65" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66">
-        <v>65</v>
-      </c>
-      <c r="B66">
-        <v>65</v>
-      </c>
-      <c r="C66" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
-      </c>
-      <c r="D66" t="str">
-        <v>198103052024211008</v>
-      </c>
-      <c r="E66" t="str">
-        <v>-</v>
-      </c>
-      <c r="F66" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G66" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
-      </c>
-      <c r="H66" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67">
-        <v>66</v>
-      </c>
-      <c r="B67">
-        <v>66</v>
-      </c>
-      <c r="C67" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
-      </c>
-      <c r="D67" t="str">
-        <v>198112142024212008</v>
-      </c>
-      <c r="E67" t="str">
-        <v>-</v>
-      </c>
-      <c r="F67" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G67" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf_FdCdD6ohlhQX_f3H7SVBGc4nrC2Ui3-rcrQZRPNnltfamQ/viewform</v>
-      </c>
-      <c r="H67" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68">
-        <v>67</v>
-      </c>
-      <c r="B68">
-        <v>67</v>
-      </c>
-      <c r="C68" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
-      </c>
-      <c r="D68" t="str">
-        <v>198201062024212001</v>
-      </c>
-      <c r="E68" t="str">
-        <v>-</v>
-      </c>
-      <c r="F68" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G68" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfnkOblKHmHEQZv7mSD1vVCZo9F05r9j_4cB8Gf13YpClrBEA/viewform</v>
-      </c>
-      <c r="H68" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69">
-        <v>68</v>
-      </c>
-      <c r="B69">
-        <v>68</v>
-      </c>
-      <c r="C69" t="str">
-        <v>YEFI WULANDARI, SE</v>
-      </c>
-      <c r="D69" t="str">
-        <v>198204272024212014</v>
-      </c>
-      <c r="E69" t="str">
-        <v>-</v>
-      </c>
-      <c r="F69" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G69" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdWSaS-TIna_zsswr8VBL4h5etsBLiiX8g9DDJoMFMbqcqRaQ/viewform</v>
-      </c>
-      <c r="H69" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70">
-        <v>69</v>
-      </c>
-      <c r="B70">
-        <v>69</v>
-      </c>
-      <c r="C70" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
-      </c>
-      <c r="D70" t="str">
-        <v>198209202024212008</v>
-      </c>
-      <c r="E70" t="str">
-        <v>-</v>
-      </c>
-      <c r="F70" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G70" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdEXPOLI2_EBQt6mzHWAdm2mEw2qMyBnYwO7RHZF7l_PG5XoQ/viewform</v>
-      </c>
-      <c r="H70" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71">
-        <v>70</v>
-      </c>
-      <c r="B71">
-        <v>70</v>
-      </c>
-      <c r="C71" t="str">
-        <v>SUWOYO, S.Kom</v>
-      </c>
-      <c r="D71" t="str">
-        <v>198403072024211011</v>
-      </c>
-      <c r="E71" t="str">
-        <v>-</v>
-      </c>
-      <c r="F71" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G71" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
-      </c>
-      <c r="H71" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72">
-        <v>71</v>
-      </c>
-      <c r="B72">
-        <v>71</v>
-      </c>
-      <c r="C72" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
-      </c>
-      <c r="D72" t="str">
-        <v>198410082024211016</v>
-      </c>
-      <c r="E72" t="str">
-        <v>-</v>
-      </c>
-      <c r="F72" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G72" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
-      </c>
-      <c r="H72" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73">
-        <v>72</v>
-      </c>
-      <c r="B73">
-        <v>72</v>
-      </c>
-      <c r="C73" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
-      </c>
-      <c r="D73" t="str">
-        <v>198606052024212013</v>
-      </c>
-      <c r="E73" t="str">
-        <v>-</v>
-      </c>
-      <c r="F73" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G73" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeqYfnPkvY4AdwC8V4UHvNEndqvqZuSZZj_2LqzOVCpFLaKXg/viewform</v>
-      </c>
-      <c r="H73" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74">
-        <v>73</v>
-      </c>
-      <c r="B74">
-        <v>73</v>
-      </c>
-      <c r="C74" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
-      </c>
-      <c r="D74" t="str">
-        <v>197411202025212006</v>
-      </c>
-      <c r="E74" t="str">
-        <v>-</v>
-      </c>
-      <c r="F74" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G74" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
-      </c>
-      <c r="H74" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75">
-        <v>74</v>
-      </c>
-      <c r="B75">
-        <v>74</v>
-      </c>
-      <c r="C75" t="str">
-        <v>SUYANTI, S.Kom.</v>
-      </c>
-      <c r="D75" t="str">
-        <v>198206012025212027</v>
-      </c>
-      <c r="E75" t="str">
-        <v>-</v>
-      </c>
-      <c r="F75" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G75" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf9LjiU4ww9Pt_xAA8_SHzsqfA3_tENCX11_lJEl64I8BOmrw/viewform</v>
-      </c>
-      <c r="H75" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76">
-        <v>75</v>
-      </c>
-      <c r="B76">
-        <v>75</v>
-      </c>
-      <c r="C76" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
-      </c>
-      <c r="D76" t="str">
-        <v>-</v>
-      </c>
-      <c r="E76" t="str">
-        <v>-</v>
-      </c>
-      <c r="F76" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G76" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdSOrQUklEFC17Wn9lGEgECqp4VP7B7A76ywjj7aydH8lBisA/viewform</v>
-      </c>
-      <c r="H76" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77">
-        <v>76</v>
-      </c>
-      <c r="B77">
-        <v>76</v>
-      </c>
-      <c r="C77" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
-      </c>
-      <c r="D77" t="str">
-        <v>-</v>
-      </c>
-      <c r="E77" t="str">
-        <v>-</v>
-      </c>
-      <c r="F77" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G77" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
-      </c>
-      <c r="H77" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78">
-        <v>77</v>
-      </c>
-      <c r="B78">
-        <v>77</v>
-      </c>
-      <c r="C78" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
-      </c>
-      <c r="D78" t="str">
-        <v>-</v>
-      </c>
-      <c r="E78" t="str">
-        <v>-</v>
-      </c>
-      <c r="F78" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G78" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe-iUqyVQtHbDMTfC_7ufj97I7ZUaQqm6A5AEb35wPuyyYjtw/viewform</v>
-      </c>
-      <c r="H78" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79">
-        <v>78</v>
-      </c>
-      <c r="B79">
-        <v>78</v>
-      </c>
-      <c r="C79" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
-      </c>
-      <c r="D79" t="str">
-        <v>-</v>
-      </c>
-      <c r="E79" t="str">
-        <v>-</v>
-      </c>
-      <c r="F79" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G79" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
-      </c>
-      <c r="H79" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80">
-        <v>79</v>
-      </c>
-      <c r="B80">
-        <v>79</v>
-      </c>
-      <c r="C80" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
-      </c>
-      <c r="D80" t="str">
-        <v>-</v>
-      </c>
-      <c r="E80" t="str">
-        <v>-</v>
-      </c>
-      <c r="F80" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G80" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
-      </c>
-      <c r="H80" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81">
-        <v>80</v>
-      </c>
-      <c r="B81">
-        <v>80</v>
-      </c>
-      <c r="C81" t="str">
-        <v>BENY WIJAYANTO, SS</v>
-      </c>
-      <c r="D81" t="str">
-        <v>-</v>
-      </c>
-      <c r="E81" t="str">
-        <v>-</v>
-      </c>
-      <c r="F81" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G81" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdoJpvoEo84fRoDbBiej0XGRlAW9_Ws8hrrM4HYvg1UuY08-A/viewform</v>
-      </c>
-      <c r="H81" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82">
-        <v>81</v>
-      </c>
-      <c r="B82">
-        <v>81</v>
-      </c>
-      <c r="C82" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
-      </c>
-      <c r="D82" t="str">
-        <v>-</v>
-      </c>
-      <c r="E82" t="str">
-        <v>-</v>
-      </c>
-      <c r="F82" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G82" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdvb6XVfWMHXObfg9Qt1qHVFJG91UMNtxkOVmOl8rIiMWyflw/viewform</v>
-      </c>
-      <c r="H82" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83">
-        <v>82</v>
-      </c>
-      <c r="B83">
-        <v>82</v>
-      </c>
-      <c r="C83" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
-      </c>
-      <c r="D83" t="str">
-        <v>-</v>
-      </c>
-      <c r="E83" t="str">
-        <v>-</v>
-      </c>
-      <c r="F83" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G83" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfIKb0_RA5kQm53YRXY6XxgtyTJnWLyMt8rbszzAxQM5OVfcw/viewform</v>
-      </c>
-      <c r="H83" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84">
-        <v>83</v>
-      </c>
-      <c r="B84">
-        <v>83</v>
-      </c>
-      <c r="C84" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
-      </c>
-      <c r="D84" t="str">
-        <v>-</v>
-      </c>
-      <c r="E84" t="str">
-        <v>-</v>
-      </c>
-      <c r="F84" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G84" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdVc_vPbnRafJ0MFj_iMwBjMvcx-SWamCBstx-Zx0eEWJWpow/viewform</v>
-      </c>
-      <c r="H84" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85">
-        <v>84</v>
-      </c>
-      <c r="B85">
-        <v>84</v>
-      </c>
-      <c r="C85" t="str">
-        <v>SAMUJI, S.Ag</v>
-      </c>
-      <c r="D85" t="str">
-        <v>-</v>
-      </c>
-      <c r="E85" t="str">
-        <v>-</v>
-      </c>
-      <c r="F85" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G85" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeH_z8k1zjOPd5-ALKEBIwAwnlGEYxrGSwIvU53bPzn4pVj5w/viewform</v>
-      </c>
-      <c r="H85" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86">
-        <v>85</v>
-      </c>
-      <c r="B86">
-        <v>85</v>
-      </c>
-      <c r="C86" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
-      </c>
-      <c r="D86" t="str">
-        <v>-</v>
-      </c>
-      <c r="E86" t="str">
-        <v>-</v>
-      </c>
-      <c r="F86" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G86" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdvQigaXQYmjPnCMU-VOYwFW7tL_wdiEQWFrrEHjwgPUriWVQ/viewform</v>
-      </c>
-      <c r="H86" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87">
-        <v>86</v>
-      </c>
-      <c r="B87">
-        <v>86</v>
-      </c>
-      <c r="C87" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
-      </c>
-      <c r="D87" t="str">
-        <v>-</v>
-      </c>
-      <c r="E87" t="str">
-        <v>-</v>
-      </c>
-      <c r="F87" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G87" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
-      </c>
-      <c r="H87" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88">
-        <v>87</v>
-      </c>
-      <c r="B88">
-        <v>87</v>
-      </c>
-      <c r="C88" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
-      </c>
-      <c r="D88" t="str">
-        <v>-</v>
-      </c>
-      <c r="E88" t="str">
-        <v>-</v>
-      </c>
-      <c r="F88" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G88" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScO5dWuDM9bbQPPRFU7wj2KYpndQWl6MjW4aeBRmp2gd1zsIg/viewform</v>
-      </c>
-      <c r="H88" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89">
-        <v>88</v>
-      </c>
-      <c r="B89">
-        <v>88</v>
-      </c>
-      <c r="C89" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
-      </c>
-      <c r="D89" t="str">
-        <v>-</v>
-      </c>
-      <c r="E89" t="str">
-        <v>-</v>
-      </c>
-      <c r="F89" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G89" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSetc4dTjz3vYbJvKTJp6Fev2T1Omw8up-uaiqGjN911bM5VhQ/viewform</v>
-      </c>
-      <c r="H89" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90">
-        <v>89</v>
-      </c>
-      <c r="B90">
-        <v>89</v>
-      </c>
-      <c r="C90" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
-      </c>
-      <c r="D90" t="str">
-        <v>-</v>
-      </c>
-      <c r="E90" t="str">
-        <v>-</v>
-      </c>
-      <c r="F90" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G90" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSegF6rlZWgN9LSLJ-b_0D-Q5rIwzgMKjDZb7njyjkb9m175Cw/viewform</v>
-      </c>
-      <c r="H90" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91">
-        <v>90</v>
-      </c>
-      <c r="B91">
-        <v>90</v>
-      </c>
-      <c r="C91" t="str">
-        <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
-      </c>
-      <c r="D91" t="str">
-        <v>-</v>
-      </c>
-      <c r="E91" t="str">
-        <v>-</v>
-      </c>
-      <c r="F91" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G91" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
-      </c>
-      <c r="H91" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92">
-        <v>91</v>
-      </c>
-      <c r="B92">
-        <v>91</v>
-      </c>
-      <c r="C92" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
-      </c>
-      <c r="D92" t="str">
-        <v>-</v>
-      </c>
-      <c r="E92" t="str">
-        <v>-</v>
-      </c>
-      <c r="F92" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G92" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc8hB1Jne1cZcXsMyyah9zkwsD-5XKk5o91E4fXfHBFtfeheg/viewform</v>
-      </c>
-      <c r="H92" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93">
-        <v>92</v>
-      </c>
-      <c r="B93">
-        <v>92</v>
-      </c>
-      <c r="C93" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="D93" t="str">
-        <v>-</v>
-      </c>
-      <c r="E93" t="str">
-        <v>-</v>
-      </c>
-      <c r="F93" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G93" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe9TyB66OIRNYnCfIgvtMfcDfVMgbJpD-JByezy7I4Gp20-Bw/viewform</v>
-      </c>
-      <c r="H93" t="str">
-        <v>✅ Valid &amp; Siap Autofill</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H93"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H41"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I95"/>
+  <dimension ref="A1:I93"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -2990,13 +3165,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G4" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSez4gjTar2bPbopGm6ErVaBlugek0rGtLocS5azfCCp0MDSIA/viewform</v>
+        <v>https://forms.gle/ekQJWbDbi72DSNHX9</v>
       </c>
       <c r="H4" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I4" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="5">
@@ -3077,13 +3252,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G7" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfb21fBd9nBHkgM2MBTbSNxfeTgWiXbFL43E9QIZX-zGLzq0g/viewform</v>
+        <v>https://forms.gle/FzjMqjr2bhYB4mFGA</v>
       </c>
       <c r="H7" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I7" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="8">
@@ -3135,13 +3310,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G9" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe-IzLFr71Gdhgd06mjpg2ToTRv1yEa_u8WYc9JsSpikG-NuA/viewform</v>
+        <v>https://forms.gle/hpaJmjc4TSuY21187</v>
       </c>
       <c r="H9" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I9" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="10">
@@ -3164,13 +3339,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G10" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf3zl2VpfYKhir9CPBloLYg_xU95VEOzo28tGm9RxY8hWf_8Q/viewform</v>
+        <v>https://forms.gle/zCXw2UY7hgtbguuc6</v>
       </c>
       <c r="H10" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I10" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="11">
@@ -3193,13 +3368,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G11" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdEgJQrGVluy9utuyyeyZ7psIgxX5H9-OTYUG63if-14TLXNg/viewform</v>
+        <v>https://forms.gle/8SMDhw8YpsNPPHPK7</v>
       </c>
       <c r="H11" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I11" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="12">
@@ -3222,13 +3397,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G12" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeYIRHhpNjh1FmGBMMlPQPwu6jnRfYLe__qCNtcIES7ZefQvQ/viewform</v>
+        <v>https://forms.gle/sZ2Rff4sL9N4FTrh9</v>
       </c>
       <c r="H12" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I12" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="13">
@@ -3367,13 +3542,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G17" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYaU-G7gAyHPvwtYTw67xI_BcR43imBjiP3RB58jOjnU1XeQ/viewform</v>
+        <v>https://forms.gle/ghNaoJYp7o2SbkjS8</v>
       </c>
       <c r="H17" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I17" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="18">
@@ -3396,13 +3571,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G18" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSd2bLbWa9Pca9QT7JTzZAnSSDZOakUabHJxB_JnNT3CQEv4gA/viewform</v>
+        <v>https://forms.gle/bPxWzjgFDES2StGo6</v>
       </c>
       <c r="H18" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I18" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="19">
@@ -3454,13 +3629,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G20" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSd4Etrlv7kK9gUfKVu1OwwyBhjLAn4-l3PArWhzLxF13MmmVw/viewform</v>
+        <v>https://forms.gle/aaS7YNQQ97713C18A</v>
       </c>
       <c r="H20" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I20" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="21">
@@ -3483,13 +3658,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G21" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScZ2l8R4TTNeJdfXVZvYAgc3WGgT9QtEVz0-ANUsebuRgsWsQ/viewform</v>
+        <v>https://forms.gle/6YPzECievjrGJZBnA</v>
       </c>
       <c r="H21" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I21" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="22">
@@ -3512,13 +3687,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G22" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdcvHzA1p4OhUC9iXA97o8okqRsjziPMeWoPw6g-Nvt7Pr9jg/viewform</v>
+        <v>https://forms.gle/2mog9vghqCw6TSTw7</v>
       </c>
       <c r="H22" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I22" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="23">
@@ -3599,13 +3774,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G25" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdoHRTHs-yCXOAaQukleNcx5jWI79dOK6qbeeCW4p45bJ9CLg/viewform</v>
+        <v>https://forms.gle/DSDoMKgI8XxbcPr78</v>
       </c>
       <c r="H25" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I25" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="26">
@@ -3628,13 +3803,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G26" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSftHQdc5-VZ5uwLLimFvRnkwycT7Ys50sjgRzMN-ALHGSjCqA/viewform</v>
+        <v>https://forms.gle/jVwhLYXebas1GSZQJ6</v>
       </c>
       <c r="H26" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I26" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="27">
@@ -3686,13 +3861,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G28" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNEYg6DAPuUemLNfKalqh5_nN6m2oxlOxSvPG1Fu55a4gqNA/viewform</v>
+        <v>https://forms.gle/r3mekFxufrTcJjgRA</v>
       </c>
       <c r="H28" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I28" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="29">
@@ -3802,13 +3977,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G32" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdRlmK9kl1qIAOcGpf1Uu18upIQ0GWK8VkTv12k_6AEAERRMQ/viewform</v>
+        <v>https://forms.gle/PSXtPwi7yQN3Mfi8</v>
       </c>
       <c r="H32" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I32" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="33">
@@ -3860,13 +4035,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G34" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdPW1l4LaclpGdRqS2jqaCtnP9mivQff9TM2a9if71auoCj6g/viewform</v>
+        <v>https://forms.gle/ESlazXu6aQ3PklsD9</v>
       </c>
       <c r="H34" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I34" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="35">
@@ -3889,13 +4064,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G35" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSejtfmzSD3f24E8Z4AXVPgC0RTs8brRuZ_KCxV9-lmsq4C5iQ/viewform</v>
+        <v>https://forms.gle/KwfitQjMYbtsnr4UZV6</v>
       </c>
       <c r="H35" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I35" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="36">
@@ -3918,13 +4093,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G36" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdaT-LhGEwSzPtm9G3LL6KRs-gFmbNF2uiIykR7J7HDmdC2uQ/viewform</v>
+        <v>https://forms.gle/DStwfQQGe3W3gc73A</v>
       </c>
       <c r="H36" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I36" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="37">
@@ -3947,13 +4122,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G37" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFjcTg73409mYsq9RTVwH8IBBBz5ya0_y6K1t74WjfpPWMhA/viewform</v>
+        <v>https://forms.gle/8Z33XXUnWmhZCY9S9</v>
       </c>
       <c r="H37" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I37" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="38">
@@ -4005,13 +4180,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G39" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScUo8DXP3Tp38IveX-Bq5eu4aD3aJBRVAjTA8896rGx1WUsNQ/viewform</v>
+        <v>https://forms.gle/iGQNqJij1huPUYbk8</v>
       </c>
       <c r="H39" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I39" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="40">
@@ -4034,13 +4209,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G40" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScKk6RYj6qkwSYwir5SH2zma20b5qhM4boLx8UqeQ19DUTIfA/viewform</v>
+        <v>https://forms.gle/RvBNnww2vjNe3gNo76</v>
       </c>
       <c r="H40" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I40" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="41">
@@ -4063,13 +4238,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G41" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSczNF2YAQXf9165kZ-FthvzailwmMrM-uSTecJzWHq0JCEldQ/viewform</v>
+        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
       </c>
       <c r="H41" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I41" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="42">
@@ -4121,13 +4296,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G43" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4Z31ED-5m9YP8u3CbOt0PWt94nwzJafZSig17a3DoqRlpCQ/viewform</v>
+        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
       </c>
       <c r="H43" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I43" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="44">
@@ -4324,13 +4499,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G50" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdUwe7or4Y0G1-MxBUlVlO5CHIQU7My-9_OxXNA87sJhdXBZA/viewform</v>
+        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
       </c>
       <c r="H50" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I50" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="51">
@@ -4353,13 +4528,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G51" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe4vBzUIUsBJNN39klf82XO2jf2iJXqigXNdhNMkSI7-lcsEw/viewform</v>
+        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
       </c>
       <c r="H51" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I51" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="52">
@@ -4382,13 +4557,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G52" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFgOYb82K7kj70lOwDL28zNyaVYlK3CX9WHttQtR-KGtb2Mg/viewform</v>
+        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
       </c>
       <c r="H52" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I52" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="53">
@@ -4469,13 +4644,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G55" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
+        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
       </c>
       <c r="H55" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I55" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="56">
@@ -4556,13 +4731,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G58" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSety3ZkhI7AVI8v-VQRPaTax5rflclagowfHbFtFrNjSSZNHg/viewform</v>
+        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
       </c>
       <c r="H58" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I58" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="59">
@@ -4585,13 +4760,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G59" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScLoRQkJKESig6rf-hq4Hq-9UsA2rpsBuDhVX6113r1OrYeLw/viewform</v>
+        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
       </c>
       <c r="H59" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I59" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="60">
@@ -4643,13 +4818,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G61" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeBM6FY62A84yCrWK-O8XZ_ehP9cDsy6qNu0MHDEXeCZlsATA/viewform</v>
+        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
       </c>
       <c r="H61" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I61" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="62">
@@ -4672,13 +4847,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G62" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGR9KnW2FGcWAVjUfLzEpLkENkH6O1XpstPv9041fsBK4r7A/viewform</v>
+        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
       </c>
       <c r="H62" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I62" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="63">
@@ -4730,13 +4905,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G64" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4F9PoN3h1R3EmQmS-KTPCmUB2ghq3K7N1e00Ni4NE30hESw/viewform</v>
+        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
       </c>
       <c r="H64" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I64" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="65">
@@ -4759,13 +4934,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G65" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSee6t_4PgxzeHNbhtwqZROlfNE9Iz6Sf5QJvGMjzkmAGvhcAw/viewform</v>
+        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
       </c>
       <c r="H65" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I65" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="66">
@@ -4817,13 +4992,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G67" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf_FdCdD6ohlhQX_f3H7SVBGc4nrC2Ui3-rcrQZRPNnltfamQ/viewform</v>
+        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
       </c>
       <c r="H67" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I67" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="68">
@@ -4846,13 +5021,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G68" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfnkOblKHmHEQZv7mSD1vVCZo9F05r9j_4cB8Gf13YpClrBEA/viewform</v>
+        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
       </c>
       <c r="H68" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I68" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="69">
@@ -4875,13 +5050,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G69" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdWSaS-TIna_zsswr8VBL4h5etsBLiiX8g9DDJoMFMbqcqRaQ/viewform</v>
+        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
       </c>
       <c r="H69" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I69" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="70">
@@ -4904,13 +5079,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G70" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdEXPOLI2_EBQt6mzHWAdm2mEw2qMyBnYwO7RHZF7l_PG5XoQ/viewform</v>
+        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
       </c>
       <c r="H70" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I70" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="71">
@@ -4991,13 +5166,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G73" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeqYfnPkvY4AdwC8V4UHvNEndqvqZuSZZj_2LqzOVCpFLaKXg/viewform</v>
+        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
       </c>
       <c r="H73" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I73" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="74">
@@ -5049,13 +5224,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G75" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf9LjiU4ww9Pt_xAA8_SHzsqfA3_tENCX11_lJEl64I8BOmrw/viewform</v>
+        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
       </c>
       <c r="H75" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I75" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="76">
@@ -5078,13 +5253,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G76" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdSOrQUklEFC17Wn9lGEgECqp4VP7B7A76ywjj7aydH8lBisA/viewform</v>
+        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
       </c>
       <c r="H76" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I76" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="77">
@@ -5136,13 +5311,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G78" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe-iUqyVQtHbDMTfC_7ufj97I7ZUaQqm6A5AEb35wPuyyYjtw/viewform</v>
+        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
       </c>
       <c r="H78" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I78" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="79">
@@ -5223,13 +5398,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G81" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdoJpvoEo84fRoDbBiej0XGRlAW9_Ws8hrrM4HYvg1UuY08-A/viewform</v>
+        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
       </c>
       <c r="H81" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I81" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="82">
@@ -5252,13 +5427,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G82" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdvb6XVfWMHXObfg9Qt1qHVFJG91UMNtxkOVmOl8rIiMWyflw/viewform</v>
+        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
       </c>
       <c r="H82" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I82" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="83">
@@ -5281,13 +5456,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G83" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfIKb0_RA5kQm53YRXY6XxgtyTJnWLyMt8rbszzAxQM5OVfcw/viewform</v>
+        <v>https://forms.gle/Auiix31BCC39d3827</v>
       </c>
       <c r="H83" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I83" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="84">
@@ -5310,13 +5485,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G84" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdVc_vPbnRafJ0MFj_iMwBjMvcx-SWamCBstx-Zx0eEWJWpow/viewform</v>
+        <v>https://forms.gle/9ox7839w57zhmph37</v>
       </c>
       <c r="H84" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I84" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="85">
@@ -5339,13 +5514,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G85" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeH_z8k1zjOPd5-ALKEBIwAwnlGEYxrGSwIvU53bPzn4pVj5w/viewform</v>
+        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
       </c>
       <c r="H85" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I85" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="86">
@@ -5368,13 +5543,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G86" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdvQigaXQYmjPnCMU-VOYwFW7tL_wdiEQWFrrEHjwgPUriWVQ/viewform</v>
+        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
       </c>
       <c r="H86" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I86" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="87">
@@ -5426,13 +5601,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G88" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScO5dWuDM9bbQPPRFU7wj2KYpndQWl6MjW4aeBRmp2gd1zsIg/viewform</v>
+        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
       </c>
       <c r="H88" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I88" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="89">
@@ -5455,13 +5630,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G89" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSetc4dTjz3vYbJvKTJp6Fev2T1Omw8up-uaiqGjN911bM5VhQ/viewform</v>
+        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
       </c>
       <c r="H89" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I89" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="90">
@@ -5484,13 +5659,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G90" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSegF6rlZWgN9LSLJ-b_0D-Q5rIwzgMKjDZb7njyjkb9m175Cw/viewform</v>
+        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
       </c>
       <c r="H90" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I90" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="91">
@@ -5542,13 +5717,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G92" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc8hB1Jne1cZcXsMyyah9zkwsD-5XKk5o91E4fXfHBFtfeheg/viewform</v>
+        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
       </c>
       <c r="H92" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I92" t="str">
-        <v>✅ Langsung Siap Autofill</v>
+        <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
     <row r="93">
@@ -5571,76 +5746,18 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G93" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe9TyB66OIRNYnCfIgvtMfcDfVMgbJpD-JByezy7I4Gp20-Bw/viewform</v>
+        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
       </c>
       <c r="H93" t="str">
-        <v>Long URL (Canonical)</v>
+        <v>Shortlink (forms.gle)</v>
       </c>
       <c r="I93" t="str">
-        <v>✅ Langsung Siap Autofill</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94">
-        <v>93</v>
-      </c>
-      <c r="B94">
-        <v>999</v>
-      </c>
-      <c r="C94" t="str">
-        <v>ARI KUNTADI, S.Pd</v>
-      </c>
-      <c r="D94" t="str">
-        <v>196712112008011004</v>
-      </c>
-      <c r="E94" t="str">
-        <v>-</v>
-      </c>
-      <c r="F94" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G94" t="str">
-        <v>-</v>
-      </c>
-      <c r="H94" t="str">
-        <v>Shortlink (forms.gle)</v>
-      </c>
-      <c r="I94" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95">
-        <v>94</v>
-      </c>
-      <c r="B95">
-        <v>999</v>
-      </c>
-      <c r="C95" t="str">
-        <v>DWI FENDI DADANG ADRIANTO, S.PD., M.T</v>
-      </c>
-      <c r="D95" t="str">
-        <v>197105162000031005</v>
-      </c>
-      <c r="E95" t="str">
-        <v>-</v>
-      </c>
-      <c r="F95" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G95" t="str">
-        <v>-</v>
-      </c>
-      <c r="H95" t="str">
-        <v>Shortlink (forms.gle)</v>
-      </c>
-      <c r="I95" t="str">
         <v>🟡 Menggunakan Fallback Form Induk</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I95"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I93"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: standardize entire application and audit tools to FORM-AutoForm project
</commit_message>
<xml_diff>
--- a/daftar_guru_status_link_google_form.xlsx
+++ b/daftar_guru_status_link_google_form.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="52 Guru Perlu Update" sheetId="1" r:id="rId1"/>
-    <sheet name="40 Guru Link Valid" sheetId="2" r:id="rId2"/>
+    <sheet name="0 Guru Perlu Update" sheetId="1" r:id="rId1"/>
+    <sheet name="92 Guru Link Valid" sheetId="2" r:id="rId2"/>
     <sheet name="Master 92 Guru Lengkap" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:A2"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -414,1551 +414,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>No</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Order</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Nama Guru</v>
-      </c>
-      <c r="D1" t="str">
-        <v>NIP</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Kelas Binaan</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Peran</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Shortlink Lama</v>
-      </c>
-      <c r="H1" t="str">
         <v>Status</v>
       </c>
-      <c r="I1" t="str">
-        <v>Link Baru (docs.google.com/forms/d/e/.../viewform)</v>
-      </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>3</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Drs. MOEHAIMIN</v>
-      </c>
-      <c r="D2" t="str">
-        <v>196709041997031005</v>
-      </c>
-      <c r="E2" t="str">
-        <v>X TEI 2</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G2" t="str">
-        <v>https://forms.gle/ekQJWbDbi72DSNHX9</v>
-      </c>
-      <c r="H2" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>6</v>
-      </c>
-      <c r="C3" t="str">
-        <v>MUNASRI, S.Pd.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>197003282008012013</v>
-      </c>
-      <c r="E3" t="str">
-        <v>X TPM 1</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G3" t="str">
-        <v>https://forms.gle/FzjMqjr2bhYB4mFGA</v>
-      </c>
-      <c r="H3" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>8</v>
-      </c>
-      <c r="C4" t="str">
-        <v>DWI RETNO TUGAS ERNAWATI, S.Pd</v>
-      </c>
-      <c r="D4" t="str">
-        <v>196702142008012009</v>
-      </c>
-      <c r="E4" t="str">
-        <v>X TKR1</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G4" t="str">
-        <v>https://forms.gle/hpaJmjc4TSuY21187</v>
-      </c>
-      <c r="H4" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>9</v>
-      </c>
-      <c r="C5" t="str">
-        <v>KASIATIN, S.Pd</v>
-      </c>
-      <c r="D5" t="str">
-        <v>196908112007012019</v>
-      </c>
-      <c r="E5" t="str">
-        <v>X TKR2</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G5" t="str">
-        <v>https://forms.gle/zCXw2UY7hgtbguuc6</v>
-      </c>
-      <c r="H5" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>10</v>
-      </c>
-      <c r="C6" t="str">
-        <v>SUHARTO DWI SUHERNOWO, ST</v>
-      </c>
-      <c r="D6" t="str">
-        <v>197803262009011007</v>
-      </c>
-      <c r="E6" t="str">
-        <v>X TBKR</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G6" t="str">
-        <v>https://forms.gle/8SMDhw8YpsNPPHPK7</v>
-      </c>
-      <c r="H6" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I6" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>11</v>
-      </c>
-      <c r="C7" t="str">
-        <v>ARSYL NOVA ARIRI, ST, M.Pd.</v>
-      </c>
-      <c r="D7" t="str">
-        <v>197811142009012007</v>
-      </c>
-      <c r="E7" t="str">
-        <v>X TSM 1</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G7" t="str">
-        <v>https://forms.gle/sZ2Rff4sL9N4FTrh9</v>
-      </c>
-      <c r="H7" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>16</v>
-      </c>
-      <c r="C8" t="str">
-        <v>WAWAN SISWANTO, SS</v>
-      </c>
-      <c r="D8" t="str">
-        <v>196904012007011025</v>
-      </c>
-      <c r="E8" t="str">
-        <v>XI TAV</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G8" t="str">
-        <v>https://forms.gle/ghNaoJYp7o2SbkjS8</v>
-      </c>
-      <c r="H8" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>17</v>
-      </c>
-      <c r="C9" t="str">
-        <v>R.A. RATNA KARTIKAWATI, S.Pd</v>
-      </c>
-      <c r="D9" t="str">
-        <v>196905132008012023</v>
-      </c>
-      <c r="E9" t="str">
-        <v>XI TEI 1</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G9" t="str">
-        <v>https://forms.gle/bPxWzjgFDES2StGo6</v>
-      </c>
-      <c r="H9" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I9" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>19</v>
-      </c>
-      <c r="C10" t="str">
-        <v>NURUL HUDA, ST, M.Si.</v>
-      </c>
-      <c r="D10" t="str">
-        <v>197102162008011009</v>
-      </c>
-      <c r="E10" t="str">
-        <v>XI TPL 1</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G10" t="str">
-        <v>https://forms.gle/aaS7YNQQ97713C18A</v>
-      </c>
-      <c r="H10" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I10" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>20</v>
-      </c>
-      <c r="C11" t="str">
-        <v>NUR 'AFIIFAH, M.Pd.</v>
-      </c>
-      <c r="D11" t="str">
-        <v>197208052007012020</v>
-      </c>
-      <c r="E11" t="str">
-        <v>XI TPL 2</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G11" t="str">
-        <v>https://forms.gle/6YPzECievjrGJZBnA</v>
-      </c>
-      <c r="H11" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I11" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>21</v>
-      </c>
-      <c r="C12" t="str">
-        <v>TRIBUDI HARTONO, S.Pd</v>
-      </c>
-      <c r="D12" t="str">
-        <v>197511052003121004</v>
-      </c>
-      <c r="E12" t="str">
-        <v>XI TPM 1</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G12" t="str">
-        <v>https://forms.gle/2mog9vghqCw6TSTw7</v>
-      </c>
-      <c r="H12" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I12" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>24</v>
-      </c>
-      <c r="C13" t="str">
-        <v>SAMSUL HADI, M.Pd.</v>
-      </c>
-      <c r="D13" t="str">
-        <v>197509262008011011</v>
-      </c>
-      <c r="E13" t="str">
-        <v>XI TKR2</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G13" t="str">
-        <v>https://forms.gle/DSDoMKgI8XxbcPr78</v>
-      </c>
-      <c r="H13" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I13" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>25</v>
-      </c>
-      <c r="C14" t="str">
-        <v>HISBULLOH HUDA, M.Pd.</v>
-      </c>
-      <c r="D14" t="str">
-        <v>197602072010011006</v>
-      </c>
-      <c r="E14" t="str">
-        <v>XI TBKR</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G14" t="str">
-        <v>https://forms.gle/jVwhLYXebas1GSZQJ6</v>
-      </c>
-      <c r="H14" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I14" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>27</v>
-      </c>
-      <c r="C15" t="str">
-        <v>AGUS HARIYANTO, ST. M.Pd</v>
-      </c>
-      <c r="D15" t="str">
-        <v>198010032010011010</v>
-      </c>
-      <c r="E15" t="str">
-        <v>XI TSM 2</v>
-      </c>
-      <c r="F15" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G15" t="str">
-        <v>https://forms.gle/r3mekFxufrTcJjgRA</v>
-      </c>
-      <c r="H15" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I15" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16">
-        <v>31</v>
-      </c>
-      <c r="C16" t="str">
-        <v>SIGIT EKO PRAMONO, S.Pd</v>
-      </c>
-      <c r="D16" t="str">
-        <v>198301122009011006</v>
-      </c>
-      <c r="E16" t="str">
-        <v>XII TAV</v>
-      </c>
-      <c r="F16" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G16" t="str">
-        <v>https://forms.gle/PSXtPwi7yQN3Mfi8</v>
-      </c>
-      <c r="H16" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I16" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17">
-        <v>33</v>
-      </c>
-      <c r="C17" t="str">
-        <v>MOHAMAD ARIEF PRIYO UTOMO, S.Pd</v>
-      </c>
-      <c r="D17" t="str">
-        <v>198209292010011011</v>
-      </c>
-      <c r="E17" t="str">
-        <v>XII TPL 1</v>
-      </c>
-      <c r="F17" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G17" t="str">
-        <v>https://forms.gle/ESlazXu6aQ3PklsD9</v>
-      </c>
-      <c r="H17" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I17" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18">
-        <v>34</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Dr. RIRIN DIYANNITA SASANTI, M.Pd.</v>
-      </c>
-      <c r="D18" t="str">
-        <v>198212022014062003</v>
-      </c>
-      <c r="E18" t="str">
-        <v>XII TPL 2</v>
-      </c>
-      <c r="F18" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G18" t="str">
-        <v>https://forms.gle/KwfitQjMYbtsnr4UZV6</v>
-      </c>
-      <c r="H18" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I18" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19">
-        <v>35</v>
-      </c>
-      <c r="C19" t="str">
-        <v>SULIADI, S.Pd</v>
-      </c>
-      <c r="D19" t="str">
-        <v>198403262010011008</v>
-      </c>
-      <c r="E19" t="str">
-        <v>XII TPM 1</v>
-      </c>
-      <c r="F19" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G19" t="str">
-        <v>https://forms.gle/DStwfQQGe3W3gc73A</v>
-      </c>
-      <c r="H19" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I19" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20">
-        <v>36</v>
-      </c>
-      <c r="C20" t="str">
-        <v>TUTIK QOMARIYAH, S.Si</v>
-      </c>
-      <c r="D20" t="str">
-        <v>198504032010012014</v>
-      </c>
-      <c r="E20" t="str">
-        <v>XII TPM 2</v>
-      </c>
-      <c r="F20" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G20" t="str">
-        <v>https://forms.gle/8Z33XXUnWmhZCY9S9</v>
-      </c>
-      <c r="H20" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I20" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21">
-        <v>38</v>
-      </c>
-      <c r="C21" t="str">
-        <v>FIRMAN ARDIANSYAH, S.Pd.</v>
-      </c>
-      <c r="D21" t="str">
-        <v>198706172011011010</v>
-      </c>
-      <c r="E21" t="str">
-        <v>XII TKR2</v>
-      </c>
-      <c r="F21" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G21" t="str">
-        <v>https://forms.gle/iGQNqJij1huPUYbk8</v>
-      </c>
-      <c r="H21" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I21" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22">
-        <v>39</v>
-      </c>
-      <c r="C22" t="str">
-        <v>AZIZ CAHYA PRADANA, S.Pd.</v>
-      </c>
-      <c r="D22" t="str">
-        <v>199103072019031014</v>
-      </c>
-      <c r="E22" t="str">
-        <v>XII TBKR</v>
-      </c>
-      <c r="F22" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G22" t="str">
-        <v>https://forms.gle/RvBNnww2vjNe3gNo76</v>
-      </c>
-      <c r="H22" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I22" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23">
-        <v>40</v>
-      </c>
-      <c r="C23" t="str">
-        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
-      </c>
-      <c r="D23" t="str">
-        <v>199311072019031004</v>
-      </c>
-      <c r="E23" t="str">
-        <v>XII TSM 1</v>
-      </c>
-      <c r="F23" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G23" t="str">
-        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
-      </c>
-      <c r="H23" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I23" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24">
-        <v>42</v>
-      </c>
-      <c r="C24" t="str">
-        <v>EFRIDA ISBANDRIYAH, S.T.</v>
-      </c>
-      <c r="D24" t="str">
-        <v>199511062019032010</v>
-      </c>
-      <c r="E24" t="str">
-        <v>XII DKV 1</v>
-      </c>
-      <c r="F24" t="str">
-        <v>Walikelas</v>
-      </c>
-      <c r="G24" t="str">
-        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
-      </c>
-      <c r="H24" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I24" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25">
-        <v>49</v>
-      </c>
-      <c r="C25" t="str">
-        <v>ETIK SULISTYOWATI, S.Pd.</v>
-      </c>
-      <c r="D25" t="str">
-        <v>198304282022212026</v>
-      </c>
-      <c r="E25" t="str">
-        <v>-</v>
-      </c>
-      <c r="F25" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G25" t="str">
-        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
-      </c>
-      <c r="H25" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I25" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26">
-        <v>50</v>
-      </c>
-      <c r="C26" t="str">
-        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
-      </c>
-      <c r="D26" t="str">
-        <v>198404192022211018</v>
-      </c>
-      <c r="E26" t="str">
-        <v>-</v>
-      </c>
-      <c r="F26" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G26" t="str">
-        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
-      </c>
-      <c r="H26" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I26" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27">
-        <v>51</v>
-      </c>
-      <c r="C27" t="str">
-        <v>YAYUK NURNANINGSIH, S.Pd</v>
-      </c>
-      <c r="D27" t="str">
-        <v>198607052022212052</v>
-      </c>
-      <c r="E27" t="str">
-        <v>-</v>
-      </c>
-      <c r="F27" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G27" t="str">
-        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
-      </c>
-      <c r="H27" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I27" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28">
-        <v>54</v>
-      </c>
-      <c r="C28" t="str">
-        <v>KHOIRUZEN, ST</v>
-      </c>
-      <c r="D28" t="str">
-        <v>197107222023211002</v>
-      </c>
-      <c r="E28" t="str">
-        <v>-</v>
-      </c>
-      <c r="F28" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G28" t="str">
-        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
-      </c>
-      <c r="H28" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I28" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29">
-        <v>28</v>
-      </c>
-      <c r="B29">
-        <v>57</v>
-      </c>
-      <c r="C29" t="str">
-        <v>DARIS UMAMI, S.Pd.</v>
-      </c>
-      <c r="D29" t="str">
-        <v>198205042023212026</v>
-      </c>
-      <c r="E29" t="str">
-        <v>-</v>
-      </c>
-      <c r="F29" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G29" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
-      </c>
-      <c r="H29" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I29" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30">
-        <v>29</v>
-      </c>
-      <c r="B30">
-        <v>58</v>
-      </c>
-      <c r="C30" t="str">
-        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
-      </c>
-      <c r="D30" t="str">
-        <v>198808072023211018</v>
-      </c>
-      <c r="E30" t="str">
-        <v>-</v>
-      </c>
-      <c r="F30" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G30" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
-      </c>
-      <c r="H30" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I30" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31">
-        <v>30</v>
-      </c>
-      <c r="B31">
-        <v>60</v>
-      </c>
-      <c r="C31" t="str">
-        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
-      </c>
-      <c r="D31" t="str">
-        <v>199606142023212026</v>
-      </c>
-      <c r="E31" t="str">
-        <v>-</v>
-      </c>
-      <c r="F31" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G31" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
-      </c>
-      <c r="H31" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I31" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32">
-        <v>31</v>
-      </c>
-      <c r="B32">
-        <v>61</v>
-      </c>
-      <c r="C32" t="str">
-        <v>SUDARMONO, ST</v>
-      </c>
-      <c r="D32" t="str">
-        <v>197206202024211005</v>
-      </c>
-      <c r="E32" t="str">
-        <v>-</v>
-      </c>
-      <c r="F32" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G32" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
-      </c>
-      <c r="H32" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I32" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33">
-        <v>32</v>
-      </c>
-      <c r="B33">
-        <v>63</v>
-      </c>
-      <c r="C33" t="str">
-        <v>ANDRI YUDHI PRASETYO, ST</v>
-      </c>
-      <c r="D33" t="str">
-        <v>197907232024211002</v>
-      </c>
-      <c r="E33" t="str">
-        <v>-</v>
-      </c>
-      <c r="F33" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G33" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
-      </c>
-      <c r="H33" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I33" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34">
-        <v>33</v>
-      </c>
-      <c r="B34">
-        <v>64</v>
-      </c>
-      <c r="C34" t="str">
-        <v>MIANTO, S.Kom.</v>
-      </c>
-      <c r="D34" t="str">
-        <v>198005222024211005</v>
-      </c>
-      <c r="E34" t="str">
-        <v>-</v>
-      </c>
-      <c r="F34" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G34" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
-      </c>
-      <c r="H34" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I34" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35">
-        <v>34</v>
-      </c>
-      <c r="B35">
-        <v>66</v>
-      </c>
-      <c r="C35" t="str">
-        <v>MAMIEK ZUHRIYAH. S.Hum</v>
-      </c>
-      <c r="D35" t="str">
-        <v>198112142024212008</v>
-      </c>
-      <c r="E35" t="str">
-        <v>-</v>
-      </c>
-      <c r="F35" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G35" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
-      </c>
-      <c r="H35" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I35" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36">
-        <v>35</v>
-      </c>
-      <c r="B36">
-        <v>67</v>
-      </c>
-      <c r="C36" t="str">
-        <v>UMI RU'YATIN, S.Pd</v>
-      </c>
-      <c r="D36" t="str">
-        <v>198201062024212001</v>
-      </c>
-      <c r="E36" t="str">
-        <v>-</v>
-      </c>
-      <c r="F36" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G36" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
-      </c>
-      <c r="H36" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I36" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37">
-        <v>36</v>
-      </c>
-      <c r="B37">
-        <v>68</v>
-      </c>
-      <c r="C37" t="str">
-        <v>YEFI WULANDARI, SE</v>
-      </c>
-      <c r="D37" t="str">
-        <v>198204272024212014</v>
-      </c>
-      <c r="E37" t="str">
-        <v>-</v>
-      </c>
-      <c r="F37" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G37" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
-      </c>
-      <c r="H37" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I37" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38">
-        <v>37</v>
-      </c>
-      <c r="B38">
-        <v>69</v>
-      </c>
-      <c r="C38" t="str">
-        <v>SARI NURHIDAYATI, S.Pd.</v>
-      </c>
-      <c r="D38" t="str">
-        <v>198209202024212008</v>
-      </c>
-      <c r="E38" t="str">
-        <v>-</v>
-      </c>
-      <c r="F38" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G38" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
-      </c>
-      <c r="H38" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I38" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39">
-        <v>38</v>
-      </c>
-      <c r="B39">
-        <v>72</v>
-      </c>
-      <c r="C39" t="str">
-        <v>YUNITA DWI WIRANTI, S.Pd</v>
-      </c>
-      <c r="D39" t="str">
-        <v>198606052024212013</v>
-      </c>
-      <c r="E39" t="str">
-        <v>-</v>
-      </c>
-      <c r="F39" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G39" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
-      </c>
-      <c r="H39" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I39" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40">
-        <v>39</v>
-      </c>
-      <c r="B40">
-        <v>74</v>
-      </c>
-      <c r="C40" t="str">
-        <v>SUYANTI, S.Kom.</v>
-      </c>
-      <c r="D40" t="str">
-        <v>198206012025212027</v>
-      </c>
-      <c r="E40" t="str">
-        <v>-</v>
-      </c>
-      <c r="F40" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G40" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
-      </c>
-      <c r="H40" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I40" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41">
-        <v>40</v>
-      </c>
-      <c r="B41">
-        <v>75</v>
-      </c>
-      <c r="C41" t="str">
-        <v>DELIA NURUL AFIFAH, S.Pd</v>
-      </c>
-      <c r="D41" t="str">
-        <v>-</v>
-      </c>
-      <c r="E41" t="str">
-        <v>-</v>
-      </c>
-      <c r="F41" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G41" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
-      </c>
-      <c r="H41" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I41" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42">
-        <v>41</v>
-      </c>
-      <c r="B42">
-        <v>77</v>
-      </c>
-      <c r="C42" t="str">
-        <v>EVY KUSHARDIANY, S.Pd</v>
-      </c>
-      <c r="D42" t="str">
-        <v>-</v>
-      </c>
-      <c r="E42" t="str">
-        <v>-</v>
-      </c>
-      <c r="F42" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G42" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
-      </c>
-      <c r="H42" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I42" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43">
-        <v>42</v>
-      </c>
-      <c r="B43">
-        <v>80</v>
-      </c>
-      <c r="C43" t="str">
-        <v>BENY WIJAYANTO, SS</v>
-      </c>
-      <c r="D43" t="str">
-        <v>-</v>
-      </c>
-      <c r="E43" t="str">
-        <v>-</v>
-      </c>
-      <c r="F43" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G43" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
-      </c>
-      <c r="H43" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I43" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44">
-        <v>43</v>
-      </c>
-      <c r="B44">
-        <v>81</v>
-      </c>
-      <c r="C44" t="str">
-        <v>NURUL JAMILAH, S.Hum.</v>
-      </c>
-      <c r="D44" t="str">
-        <v>-</v>
-      </c>
-      <c r="E44" t="str">
-        <v>-</v>
-      </c>
-      <c r="F44" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G44" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
-      </c>
-      <c r="H44" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I44" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45">
-        <v>44</v>
-      </c>
-      <c r="B45">
-        <v>82</v>
-      </c>
-      <c r="C45" t="str">
-        <v>ENDANG MULYANI, S.Pd.</v>
-      </c>
-      <c r="D45" t="str">
-        <v>-</v>
-      </c>
-      <c r="E45" t="str">
-        <v>-</v>
-      </c>
-      <c r="F45" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G45" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
-      </c>
-      <c r="H45" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I45" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46">
-        <v>45</v>
-      </c>
-      <c r="B46">
-        <v>83</v>
-      </c>
-      <c r="C46" t="str">
-        <v>AGUS IRIANTO, S.Pd</v>
-      </c>
-      <c r="D46" t="str">
-        <v>-</v>
-      </c>
-      <c r="E46" t="str">
-        <v>-</v>
-      </c>
-      <c r="F46" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G46" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
-      </c>
-      <c r="H46" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I46" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47">
-        <v>46</v>
-      </c>
-      <c r="B47">
-        <v>84</v>
-      </c>
-      <c r="C47" t="str">
-        <v>SAMUJI, S.Ag</v>
-      </c>
-      <c r="D47" t="str">
-        <v>-</v>
-      </c>
-      <c r="E47" t="str">
-        <v>-</v>
-      </c>
-      <c r="F47" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G47" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
-      </c>
-      <c r="H47" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I47" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48">
-        <v>47</v>
-      </c>
-      <c r="B48">
-        <v>85</v>
-      </c>
-      <c r="C48" t="str">
-        <v>IKA UMAYA MARDIANA, S.Pd</v>
-      </c>
-      <c r="D48" t="str">
-        <v>-</v>
-      </c>
-      <c r="E48" t="str">
-        <v>-</v>
-      </c>
-      <c r="F48" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G48" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
-      </c>
-      <c r="H48" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I48" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49">
-        <v>48</v>
-      </c>
-      <c r="B49">
-        <v>87</v>
-      </c>
-      <c r="C49" t="str">
-        <v>AIDA QONITATILLAH, S.Pd</v>
-      </c>
-      <c r="D49" t="str">
-        <v>-</v>
-      </c>
-      <c r="E49" t="str">
-        <v>-</v>
-      </c>
-      <c r="F49" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G49" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
-      </c>
-      <c r="H49" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I49" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50">
-        <v>49</v>
-      </c>
-      <c r="B50">
-        <v>88</v>
-      </c>
-      <c r="C50" t="str">
-        <v>YULI ANDRIYANI,  S.Pd</v>
-      </c>
-      <c r="D50" t="str">
-        <v>-</v>
-      </c>
-      <c r="E50" t="str">
-        <v>-</v>
-      </c>
-      <c r="F50" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G50" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
-      </c>
-      <c r="H50" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I50" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51">
-        <v>50</v>
-      </c>
-      <c r="B51">
-        <v>89</v>
-      </c>
-      <c r="C51" t="str">
-        <v>VITA EKA RAHAYU, S.Pd</v>
-      </c>
-      <c r="D51" t="str">
-        <v>-</v>
-      </c>
-      <c r="E51" t="str">
-        <v>-</v>
-      </c>
-      <c r="F51" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G51" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
-      </c>
-      <c r="H51" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I51" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52">
-        <v>51</v>
-      </c>
-      <c r="B52">
-        <v>91</v>
-      </c>
-      <c r="C52" t="str">
-        <v>HERI SUGIANTORO, S.Ag</v>
-      </c>
-      <c r="D52" t="str">
-        <v>-</v>
-      </c>
-      <c r="E52" t="str">
-        <v>-</v>
-      </c>
-      <c r="F52" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G52" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
-      </c>
-      <c r="H52" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I52" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53">
-        <v>52</v>
-      </c>
-      <c r="B53">
-        <v>92</v>
-      </c>
-      <c r="C53" t="str">
-        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
-      </c>
-      <c r="D53" t="str">
-        <v>-</v>
-      </c>
-      <c r="E53" t="str">
-        <v>-</v>
-      </c>
-      <c r="F53" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G53" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
-      </c>
-      <c r="H53" t="str">
-        <v>⚠️ Perlu Update URL Panjang</v>
-      </c>
-      <c r="I53" t="str">
-        <v/>
+      <c r="A2" t="str">
+        <v>Semua guru telah valid 100%!</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H93"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -2053,22 +526,22 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" t="str">
-        <v>DHURROTUL FARIDAH, S.Pd</v>
+        <v>Drs. MOEHAIMIN</v>
       </c>
       <c r="D4" t="str">
-        <v>196707142006042005</v>
+        <v>196709041997031005</v>
       </c>
       <c r="E4" t="str">
-        <v>X TPL 1</v>
+        <v>X TEI 2</v>
       </c>
       <c r="F4" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G4" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeMVWzzDZ53AHLlhGUhchbGtjSPh774mpA2M0nanLr8yfuENQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSez4gjTar2bPbopGm6ErVaBlugek0rGtLocS5azfCCp0MDSIA/viewform</v>
       </c>
       <c r="H4" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2079,22 +552,22 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5" t="str">
-        <v>SRI WINARTI, S.Pd</v>
+        <v>DHURROTUL FARIDAH, S.Pd</v>
       </c>
       <c r="D5" t="str">
-        <v>197307112007012008</v>
+        <v>196707142006042005</v>
       </c>
       <c r="E5" t="str">
-        <v>X TPL 2</v>
+        <v>X TPL 1</v>
       </c>
       <c r="F5" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G5" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeDax_Aw_bF0ozmHf2395mK0_9K9QaIgPxKL3Msw8FyZrsKJw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeMVWzzDZ53AHLlhGUhchbGtjSPh774mpA2M0nanLr8yfuENQ/viewform</v>
       </c>
       <c r="H5" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2105,22 +578,22 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C6" t="str">
-        <v>NUR HAYATI, S.Psi, M.Pd.</v>
+        <v>SRI WINARTI, S.Pd</v>
       </c>
       <c r="D6" t="str">
-        <v>197310152009012003</v>
+        <v>197307112007012008</v>
       </c>
       <c r="E6" t="str">
-        <v>X TPM 2</v>
+        <v>X TPL 2</v>
       </c>
       <c r="F6" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G6" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeD8S_m6otgqVphxM7Ux4fGC0wrPh7aPQIKMKg_uaW5tKl42w/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeDax_Aw_bF0ozmHf2395mK0_9K9QaIgPxKL3Msw8FyZrsKJw/viewform</v>
       </c>
       <c r="H6" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2131,22 +604,22 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C7" t="str">
-        <v>LAILA FITRIYA, S.Pd.I</v>
+        <v>MUNASRI, S.Pd.</v>
       </c>
       <c r="D7" t="str">
-        <v>198506172009012006</v>
+        <v>197003282008012013</v>
       </c>
       <c r="E7" t="str">
-        <v>X TSM 2</v>
+        <v>X TPM 1</v>
       </c>
       <c r="F7" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G7" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfLY_MCLONnsdcq8EWaQayXJZ8_9cAWE7IYKvdeEhm2S0GL9A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfb21fBd9nBHkgM2MBTbSNxfeTgWiXbFL43E9QIZX-zGLzq0g/viewform</v>
       </c>
       <c r="H7" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2157,22 +630,22 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C8" t="str">
-        <v>EKA PRAMITASARI, S.Pd. M.Pd.</v>
+        <v>NUR HAYATI, S.Psi, M.Pd.</v>
       </c>
       <c r="D8" t="str">
-        <v>198710302010012005</v>
+        <v>197310152009012003</v>
       </c>
       <c r="E8" t="str">
-        <v>X DKV 1</v>
+        <v>X TPM 2</v>
       </c>
       <c r="F8" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G8" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFNOjWRONIbFscUAVy_gPYaD8c1ehSpS2dTykzwJAn_RUDGw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeD8S_m6otgqVphxM7Ux4fGC0wrPh7aPQIKMKg_uaW5tKl42w/viewform</v>
       </c>
       <c r="H8" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2183,22 +656,22 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C9" t="str">
-        <v>MISBAHUR ROSYIDIN, S.Pd.</v>
+        <v>DWI RETNO TUGAS ERNAWATI, S.Pd</v>
       </c>
       <c r="D9" t="str">
-        <v>196802112008011008</v>
+        <v>196702142008012009</v>
       </c>
       <c r="E9" t="str">
-        <v>X DKV 2</v>
+        <v>X TKR1</v>
       </c>
       <c r="F9" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G9" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe7MHsr1k2S6apY2TP7L_VulJ7MaQqcKaEsASfOrFV2WfDKSw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe-IzLFr71Gdhgd06mjpg2ToTRv1yEa_u8WYc9JsSpikG-NuA/viewform</v>
       </c>
       <c r="H9" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2209,22 +682,22 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C10" t="str">
-        <v>Dra. DYAH CHUSNUL CHOTIMAH</v>
+        <v>KASIATIN, S.Pd</v>
       </c>
       <c r="D10" t="str">
-        <v>196802142007012016</v>
+        <v>196908112007012019</v>
       </c>
       <c r="E10" t="str">
-        <v>X DKV 3</v>
+        <v>X TKR2</v>
       </c>
       <c r="F10" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G10" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScl7wa5Pd4jitd3sxqnpqk8tlBpTw-Bx1jl50JwfjGXK_v6ZQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf3zl2VpfYKhir9CPBloLYg_xU95VEOzo28tGm9RxY8hWf_8Q/viewform</v>
       </c>
       <c r="H10" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2235,22 +708,22 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C11" t="str">
-        <v>HERI SUBYANTORO, ST, M.Pd.</v>
+        <v>SUHARTO DWI SUHERNOWO, ST</v>
       </c>
       <c r="D11" t="str">
-        <v>196910102008011021</v>
+        <v>197803262009011007</v>
       </c>
       <c r="E11" t="str">
-        <v>XI TEI 2</v>
+        <v>X TBKR</v>
       </c>
       <c r="F11" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G11" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdHmC5tO01PGYfeU-it6vioHYot6MO4Enq9Nbw1oA8DLgGJog/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdEgJQrGVluy9utuyyeyZ7psIgxX5H9-OTYUG63if-14TLXNg/viewform</v>
       </c>
       <c r="H11" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2261,22 +734,22 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="C12" t="str">
-        <v>DEDY HENDRIANA, S.Pd. M.Pd.</v>
+        <v>ARSYL NOVA ARIRI, ST, M.Pd.</v>
       </c>
       <c r="D12" t="str">
-        <v>197904072010011002</v>
+        <v>197811142009012007</v>
       </c>
       <c r="E12" t="str">
-        <v>XI TPM 2</v>
+        <v>X TSM 1</v>
       </c>
       <c r="F12" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G12" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSecBLlEDfTwutpIfoRhoxlk9TykVgqtywzFBczl8dG7w3nLgg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeYIRHhpNjh1FmGBMMlPQPwu6jnRfYLe__qCNtcIES7ZefQvQ/viewform</v>
       </c>
       <c r="H12" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2287,22 +760,22 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C13" t="str">
-        <v>AGUS HIDAYAT, S.Pd</v>
+        <v>LAILA FITRIYA, S.Pd.I</v>
       </c>
       <c r="D13" t="str">
-        <v>196907272007011018</v>
+        <v>198506172009012006</v>
       </c>
       <c r="E13" t="str">
-        <v>XI TKR1</v>
+        <v>X TSM 2</v>
       </c>
       <c r="F13" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G13" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4cLrLtqJrSQCZlTZvjVDTqCqwr0Ezvo9jj1xlEEVIA1TgLQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfLY_MCLONnsdcq8EWaQayXJZ8_9cAWE7IYKvdeEhm2S0GL9A/viewform</v>
       </c>
       <c r="H13" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2313,22 +786,22 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="C14" t="str">
-        <v>DWI SANTOSO, S.Pd</v>
+        <v>EKA PRAMITASARI, S.Pd. M.Pd.</v>
       </c>
       <c r="D14" t="str">
-        <v>197908082006041019</v>
+        <v>198710302010012005</v>
       </c>
       <c r="E14" t="str">
-        <v>XI TSM 1</v>
+        <v>X DKV 1</v>
       </c>
       <c r="F14" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G14" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc3pPlG2fg8z9mrKutplhHQxr-oLEDr0OrG2tbckE403avEiw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFNOjWRONIbFscUAVy_gPYaD8c1ehSpS2dTykzwJAn_RUDGw/viewform</v>
       </c>
       <c r="H14" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2339,22 +812,22 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="C15" t="str">
-        <v>ZAINUL ARIFIN, M.Pd.</v>
+        <v>MISBAHUR ROSYIDIN, S.Pd.</v>
       </c>
       <c r="D15" t="str">
-        <v>198210112010011009</v>
+        <v>196802112008011008</v>
       </c>
       <c r="E15" t="str">
-        <v>XI DKV 1</v>
+        <v>X DKV 2</v>
       </c>
       <c r="F15" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G15" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc1knrp09uNEhFpIHg2HnTVcw1HE0-aoR7bacYb4cXIsHAleQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe7MHsr1k2S6apY2TP7L_VulJ7MaQqcKaEsASfOrFV2WfDKSw/viewform</v>
       </c>
       <c r="H15" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2365,22 +838,22 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="C16" t="str">
-        <v>BAMBANG SUJATMIKO, S.Pd</v>
+        <v>Dra. DYAH CHUSNUL CHOTIMAH</v>
       </c>
       <c r="D16" t="str">
-        <v>198211222006041009</v>
+        <v>196802142007012016</v>
       </c>
       <c r="E16" t="str">
-        <v>XI DKV 2</v>
+        <v>X DKV 3</v>
       </c>
       <c r="F16" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G16" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYyOzS9TUnTH79m-niYDGHWqxmhbtWyxFehMM6Td06hqBh1A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScl7wa5Pd4jitd3sxqnpqk8tlBpTw-Bx1jl50JwfjGXK_v6ZQ/viewform</v>
       </c>
       <c r="H16" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2391,22 +864,22 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C17" t="str">
-        <v>HARTONO, S.Pd</v>
+        <v>WAWAN SISWANTO, SS</v>
       </c>
       <c r="D17" t="str">
-        <v>198205122009011009</v>
+        <v>196904012007011025</v>
       </c>
       <c r="E17" t="str">
-        <v>XI DKV 3</v>
+        <v>XI TAV</v>
       </c>
       <c r="F17" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G17" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSczcB1-HoNbq4XLNVL6d22ps_sHXrr_yAMrTdi-SXUI9dyDiA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYaU-G7gAyHPvwtYTw67xI_BcR43imBjiP3RB58jOjnU1XeQ/viewform</v>
       </c>
       <c r="H17" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2417,22 +890,22 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="C18" t="str">
-        <v>AGUNG RAKHMANDA, S.Kom.</v>
+        <v>R.A. RATNA KARTIKAWATI, S.Pd</v>
       </c>
       <c r="D18" t="str">
-        <v>198303272009031002</v>
+        <v>196905132008012023</v>
       </c>
       <c r="E18" t="str">
-        <v>XII TEI 1</v>
+        <v>XI TEI 1</v>
       </c>
       <c r="F18" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G18" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe3WNA-vHAA16POkCpcvBUl2Kc57HtjVXCkAQEm_mMB69NPow/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSd2bLbWa9Pca9QT7JTzZAnSSDZOakUabHJxB_JnNT3CQEv4gA/viewform</v>
       </c>
       <c r="H18" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2443,22 +916,22 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="C19" t="str">
-        <v>IMAM SUFERI, ST.</v>
+        <v>HERI SUBYANTORO, ST, M.Pd.</v>
       </c>
       <c r="D19" t="str">
-        <v>197712302008011013</v>
+        <v>196910102008011021</v>
       </c>
       <c r="E19" t="str">
-        <v>XII TKR1</v>
+        <v>XI TEI 2</v>
       </c>
       <c r="F19" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G19" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSe8sSOVeefXvVkHVMUzrTdYO8RrfqdFwT5AQRWWlJ3ZzJAluQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdHmC5tO01PGYfeU-it6vioHYot6MO4Enq9Nbw1oA8DLgGJog/viewform</v>
       </c>
       <c r="H19" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2469,22 +942,22 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="C20" t="str">
-        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
+        <v>NURUL HUDA, ST, M.Si.</v>
       </c>
       <c r="D20" t="str">
-        <v>199410092019032012</v>
+        <v>197102162008011009</v>
       </c>
       <c r="E20" t="str">
-        <v>XII TSM 2</v>
+        <v>XI TPL 1</v>
       </c>
       <c r="F20" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G20" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSd4Etrlv7kK9gUfKVu1OwwyBhjLAn4-l3PArWhzLxF13MmmVw/viewform</v>
       </c>
       <c r="H20" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2495,22 +968,22 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="C21" t="str">
-        <v>SOTYA BAYUNTARA, S.Pd.</v>
+        <v>NUR 'AFIIFAH, M.Pd.</v>
       </c>
       <c r="D21" t="str">
-        <v>196906252022211004</v>
+        <v>197208052007012020</v>
       </c>
       <c r="E21" t="str">
-        <v>XII DKV 2</v>
+        <v>XI TPL 2</v>
       </c>
       <c r="F21" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G21" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScZ2l8R4TTNeJdfXVZvYAgc3WGgT9QtEVz0-ANUsebuRgsWsQ/viewform</v>
       </c>
       <c r="H21" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2521,22 +994,22 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="C22" t="str">
-        <v>SRIGATI, SE</v>
+        <v>TRIBUDI HARTONO, S.Pd</v>
       </c>
       <c r="D22" t="str">
-        <v>197505052022212013</v>
+        <v>197511052003121004</v>
       </c>
       <c r="E22" t="str">
-        <v>XII DKV 3</v>
+        <v>XI TPM 1</v>
       </c>
       <c r="F22" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G22" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdcvHzA1p4OhUC9iXA97o8okqRsjziPMeWoPw6g-Nvt7Pr9jg/viewform</v>
       </c>
       <c r="H22" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2547,22 +1020,22 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="C23" t="str">
-        <v>HARI PURWANTO, ST</v>
+        <v>DEDY HENDRIANA, S.Pd. M.Pd.</v>
       </c>
       <c r="D23" t="str">
-        <v>197711242022211006</v>
+        <v>197904072010011002</v>
       </c>
       <c r="E23" t="str">
-        <v>-</v>
+        <v>XI TPM 2</v>
       </c>
       <c r="F23" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G23" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSecBLlEDfTwutpIfoRhoxlk9TykVgqtywzFBczl8dG7w3nLgg/viewform</v>
       </c>
       <c r="H23" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2573,22 +1046,22 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C24" t="str">
-        <v>ESTI WIDHIARNI, S.T</v>
+        <v>AGUS HIDAYAT, S.Pd</v>
       </c>
       <c r="D24" t="str">
-        <v>197906032022212022</v>
+        <v>196907272007011018</v>
       </c>
       <c r="E24" t="str">
-        <v>-</v>
+        <v>XI TKR1</v>
       </c>
       <c r="F24" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G24" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4cLrLtqJrSQCZlTZvjVDTqCqwr0Ezvo9jj1xlEEVIA1TgLQ/viewform</v>
       </c>
       <c r="H24" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2599,22 +1072,22 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="C25" t="str">
-        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
+        <v>SAMSUL HADI, M.Pd.</v>
       </c>
       <c r="D25" t="str">
-        <v>198109092022211004</v>
+        <v>197509262008011011</v>
       </c>
       <c r="E25" t="str">
-        <v>XII TEI 2</v>
+        <v>XI TKR2</v>
       </c>
       <c r="F25" t="str">
         <v>Walikelas</v>
       </c>
       <c r="G25" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdoHRTHs-yCXOAaQukleNcx5jWI79dOK6qbeeCW4p45bJ9CLg/viewform</v>
       </c>
       <c r="H25" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2625,22 +1098,22 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="C26" t="str">
-        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
+        <v>HISBULLOH HUDA, M.Pd.</v>
       </c>
       <c r="D26" t="str">
-        <v>198212102022211017</v>
+        <v>197602072010011006</v>
       </c>
       <c r="E26" t="str">
-        <v>-</v>
+        <v>XI TBKR</v>
       </c>
       <c r="F26" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G26" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSftHQdc5-VZ5uwLLimFvRnkwycT7Ys50sjgRzMN-ALHGSjCqA/viewform</v>
       </c>
       <c r="H26" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2651,22 +1124,22 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="C27" t="str">
-        <v>KHOIRUL AMIN, S.Pd</v>
+        <v>DWI SANTOSO, S.Pd</v>
       </c>
       <c r="D27" t="str">
-        <v>198701192022211009</v>
+        <v>197908082006041019</v>
       </c>
       <c r="E27" t="str">
-        <v>-</v>
+        <v>XI TSM 1</v>
       </c>
       <c r="F27" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G27" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc3pPlG2fg8z9mrKutplhHQxr-oLEDr0OrG2tbckE403avEiw/viewform</v>
       </c>
       <c r="H27" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2677,22 +1150,22 @@
         <v>27</v>
       </c>
       <c r="B28">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="C28" t="str">
-        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
+        <v>AGUS HARIYANTO, ST. M.Pd</v>
       </c>
       <c r="D28" t="str">
-        <v>198712072022211015</v>
+        <v>198010032010011010</v>
       </c>
       <c r="E28" t="str">
-        <v>-</v>
+        <v>XI TSM 2</v>
       </c>
       <c r="F28" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G28" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNEYg6DAPuUemLNfKalqh5_nN6m2oxlOxSvPG1Fu55a4gqNA/viewform</v>
       </c>
       <c r="H28" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2703,22 +1176,22 @@
         <v>28</v>
       </c>
       <c r="B29">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="C29" t="str">
-        <v>HEPPY LUCKITO, SST</v>
+        <v>ZAINUL ARIFIN, M.Pd.</v>
       </c>
       <c r="D29" t="str">
-        <v>198110272023211008</v>
+        <v>198210112010011009</v>
       </c>
       <c r="E29" t="str">
-        <v>-</v>
+        <v>XI DKV 1</v>
       </c>
       <c r="F29" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G29" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc1knrp09uNEhFpIHg2HnTVcw1HE0-aoR7bacYb4cXIsHAleQ/viewform</v>
       </c>
       <c r="H29" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2729,22 +1202,22 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="C30" t="str">
-        <v>SRI PURWANINGSIH, S.Pd</v>
+        <v>BAMBANG SUJATMIKO, S.Pd</v>
       </c>
       <c r="D30" t="str">
-        <v>198203022023212020</v>
+        <v>198211222006041009</v>
       </c>
       <c r="E30" t="str">
-        <v>-</v>
+        <v>XI DKV 2</v>
       </c>
       <c r="F30" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G30" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYyOzS9TUnTH79m-niYDGHWqxmhbtWyxFehMM6Td06hqBh1A/viewform</v>
       </c>
       <c r="H30" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2755,22 +1228,22 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="C31" t="str">
-        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+        <v>HARTONO, S.Pd</v>
       </c>
       <c r="D31" t="str">
-        <v>199410282023211012</v>
+        <v>198205122009011009</v>
       </c>
       <c r="E31" t="str">
-        <v>-</v>
+        <v>XI DKV 3</v>
       </c>
       <c r="F31" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G31" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSczcB1-HoNbq4XLNVL6d22ps_sHXrr_yAMrTdi-SXUI9dyDiA/viewform</v>
       </c>
       <c r="H31" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2781,22 +1254,22 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="C32" t="str">
-        <v>ROHMAN, S.T.</v>
+        <v>SIGIT EKO PRAMONO, S.Pd</v>
       </c>
       <c r="D32" t="str">
-        <v>197509042024211002</v>
+        <v>198301122009011006</v>
       </c>
       <c r="E32" t="str">
-        <v>-</v>
+        <v>XII TAV</v>
       </c>
       <c r="F32" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G32" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdRlmK9kl1qIAOcGpf1Uu18upIQ0GWK8VkTv12k_6AEAERRMQ/viewform</v>
       </c>
       <c r="H32" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2807,22 +1280,22 @@
         <v>32</v>
       </c>
       <c r="B33">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="C33" t="str">
-        <v>HARIS ALI MUHYIDIN, S.T</v>
+        <v>AGUNG RAKHMANDA, S.Kom.</v>
       </c>
       <c r="D33" t="str">
-        <v>198103052024211008</v>
+        <v>198303272009031002</v>
       </c>
       <c r="E33" t="str">
-        <v>-</v>
+        <v>XII TEI 1</v>
       </c>
       <c r="F33" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G33" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe3WNA-vHAA16POkCpcvBUl2Kc57HtjVXCkAQEm_mMB69NPow/viewform</v>
       </c>
       <c r="H33" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2833,22 +1306,22 @@
         <v>33</v>
       </c>
       <c r="B34">
-        <v>70</v>
+        <v>33</v>
       </c>
       <c r="C34" t="str">
-        <v>SUWOYO, S.Kom</v>
+        <v>MOHAMAD ARIEF PRIYO UTOMO, S.Pd</v>
       </c>
       <c r="D34" t="str">
-        <v>198403072024211011</v>
+        <v>198209292010011011</v>
       </c>
       <c r="E34" t="str">
-        <v>-</v>
+        <v>XII TPL 1</v>
       </c>
       <c r="F34" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G34" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdPW1l4LaclpGdRqS2jqaCtnP9mivQff9TM2a9if71auoCj6g/viewform</v>
       </c>
       <c r="H34" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2859,22 +1332,22 @@
         <v>34</v>
       </c>
       <c r="B35">
-        <v>71</v>
+        <v>34</v>
       </c>
       <c r="C35" t="str">
-        <v>AAN SUSANTO, S.Pd.</v>
+        <v>Dr. RIRIN DIYANNITA SASANTI, M.Pd.</v>
       </c>
       <c r="D35" t="str">
-        <v>198410082024211016</v>
+        <v>198212022014062003</v>
       </c>
       <c r="E35" t="str">
-        <v>-</v>
+        <v>XII TPL 2</v>
       </c>
       <c r="F35" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G35" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSejtfmzSD3f24E8Z4AXVPgC0RTs8brRuZ_KCxV9-lmsq4C5iQ/viewform</v>
       </c>
       <c r="H35" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2885,22 +1358,22 @@
         <v>35</v>
       </c>
       <c r="B36">
-        <v>73</v>
+        <v>35</v>
       </c>
       <c r="C36" t="str">
-        <v>NUR FAUZIYAH, S.Ag.</v>
+        <v>SULIADI, S.Pd</v>
       </c>
       <c r="D36" t="str">
-        <v>197411202025212006</v>
+        <v>198403262010011008</v>
       </c>
       <c r="E36" t="str">
-        <v>-</v>
+        <v>XII TPM 1</v>
       </c>
       <c r="F36" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G36" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdaT-LhGEwSzPtm9G3LL6KRs-gFmbNF2uiIykR7J7HDmdC2uQ/viewform</v>
       </c>
       <c r="H36" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2911,22 +1384,22 @@
         <v>36</v>
       </c>
       <c r="B37">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="C37" t="str">
-        <v>CAHYA ISKANDAR, S.T</v>
+        <v>TUTIK QOMARIYAH, S.Si</v>
       </c>
       <c r="D37" t="str">
-        <v>-</v>
+        <v>198504032010012014</v>
       </c>
       <c r="E37" t="str">
-        <v>-</v>
+        <v>XII TPM 2</v>
       </c>
       <c r="F37" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G37" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFjcTg73409mYsq9RTVwH8IBBBz5ya0_y6K1t74WjfpPWMhA/viewform</v>
       </c>
       <c r="H37" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2937,22 +1410,22 @@
         <v>37</v>
       </c>
       <c r="B38">
-        <v>78</v>
+        <v>37</v>
       </c>
       <c r="C38" t="str">
-        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+        <v>IMAM SUFERI, ST.</v>
       </c>
       <c r="D38" t="str">
-        <v>-</v>
+        <v>197712302008011013</v>
       </c>
       <c r="E38" t="str">
-        <v>-</v>
+        <v>XII TKR1</v>
       </c>
       <c r="F38" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G38" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe8sSOVeefXvVkHVMUzrTdYO8RrfqdFwT5AQRWWlJ3ZzJAluQ/viewform</v>
       </c>
       <c r="H38" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2963,22 +1436,22 @@
         <v>38</v>
       </c>
       <c r="B39">
-        <v>79</v>
+        <v>38</v>
       </c>
       <c r="C39" t="str">
-        <v>YUNIAR DWI LISTYANTO, ST</v>
+        <v>FIRMAN ARDIANSYAH, S.Pd.</v>
       </c>
       <c r="D39" t="str">
-        <v>-</v>
+        <v>198706172011011010</v>
       </c>
       <c r="E39" t="str">
-        <v>-</v>
+        <v>XII TKR2</v>
       </c>
       <c r="F39" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G39" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScUo8DXP3Tp38IveX-Bq5eu4aD3aJBRVAjTA8896rGx1WUsNQ/viewform</v>
       </c>
       <c r="H39" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -2989,22 +1462,22 @@
         <v>39</v>
       </c>
       <c r="B40">
-        <v>86</v>
+        <v>39</v>
       </c>
       <c r="C40" t="str">
-        <v>NUR KHOLIFAH, S.Pd.</v>
+        <v>AZIZ CAHYA PRADANA, S.Pd.</v>
       </c>
       <c r="D40" t="str">
-        <v>-</v>
+        <v>199103072019031014</v>
       </c>
       <c r="E40" t="str">
-        <v>-</v>
+        <v>XII TBKR</v>
       </c>
       <c r="F40" t="str">
-        <v>Guru Pengajar</v>
+        <v>Walikelas</v>
       </c>
       <c r="G40" t="str">
-        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScKk6RYj6qkwSYwir5SH2zma20b5qhM4boLx8UqeQ19DUTIfA/viewform</v>
       </c>
       <c r="H40" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
@@ -3015,30 +1488,1382 @@
         <v>40</v>
       </c>
       <c r="B41">
+        <v>40</v>
+      </c>
+      <c r="C41" t="str">
+        <v>WAHYU ROFIUL AMIN, S.Pd.</v>
+      </c>
+      <c r="D41" t="str">
+        <v>199311072019031004</v>
+      </c>
+      <c r="E41" t="str">
+        <v>XII TSM 1</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G41" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSczNF2YAQXf9165kZ-FthvzailwmMrM-uSTecJzWHq0JCEldQ/viewform</v>
+      </c>
+      <c r="H41" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>41</v>
+      </c>
+      <c r="C42" t="str">
+        <v>ROHMA EKA INDRI AHADIAH, S.Pd, Gr</v>
+      </c>
+      <c r="D42" t="str">
+        <v>199410092019032012</v>
+      </c>
+      <c r="E42" t="str">
+        <v>XII TSM 2</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G42" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScK_Fn5phDHlhyiBBBWJCXbly98uhXuUeDJI8SvpUkG7rVDOA/viewform</v>
+      </c>
+      <c r="H42" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>42</v>
+      </c>
+      <c r="C43" t="str">
+        <v>EFRIDA ISBANDRIYAH, S.T.</v>
+      </c>
+      <c r="D43" t="str">
+        <v>199511062019032010</v>
+      </c>
+      <c r="E43" t="str">
+        <v>XII DKV 1</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G43" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4Z31ED-5m9YP8u3CbOt0PWt94nwzJafZSig17a3DoqRlpCQ/viewform</v>
+      </c>
+      <c r="H43" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>43</v>
+      </c>
+      <c r="C44" t="str">
+        <v>SOTYA BAYUNTARA, S.Pd.</v>
+      </c>
+      <c r="D44" t="str">
+        <v>196906252022211004</v>
+      </c>
+      <c r="E44" t="str">
+        <v>XII DKV 2</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G44" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdwaCYi61FdUUCDjn3mXAV6GKexgFlYoZgo-vf_JhnDJWZFyQ/viewform</v>
+      </c>
+      <c r="H44" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>44</v>
+      </c>
+      <c r="C45" t="str">
+        <v>SRIGATI, SE</v>
+      </c>
+      <c r="D45" t="str">
+        <v>197505052022212013</v>
+      </c>
+      <c r="E45" t="str">
+        <v>XII DKV 3</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G45" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFWBI_dGdSFaSy9f7QnJpSPQD8ArZ5DWF08v2sXfUtCf9vNg/viewform</v>
+      </c>
+      <c r="H45" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>45</v>
+      </c>
+      <c r="C46" t="str">
+        <v>HARI PURWANTO, ST</v>
+      </c>
+      <c r="D46" t="str">
+        <v>197711242022211006</v>
+      </c>
+      <c r="E46" t="str">
+        <v>-</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G46" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0YfQN7C3oqM_e_gkF-IHzItqHHrH06SNEgwoteprcY9u3Fw/viewform</v>
+      </c>
+      <c r="H46" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>46</v>
+      </c>
+      <c r="C47" t="str">
+        <v>ESTI WIDHIARNI, S.T</v>
+      </c>
+      <c r="D47" t="str">
+        <v>197906032022212022</v>
+      </c>
+      <c r="E47" t="str">
+        <v>-</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G47" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScjOVIF4Br99MIEOWVROsGlzRdhA3fblU_WANEmzYffGpUlxw/viewform</v>
+      </c>
+      <c r="H47" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>47</v>
+      </c>
+      <c r="C48" t="str">
+        <v>MUCHAMAD ISKAK FATONI, S.Pd.</v>
+      </c>
+      <c r="D48" t="str">
+        <v>198109092022211004</v>
+      </c>
+      <c r="E48" t="str">
+        <v>XII TEI 2</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Walikelas</v>
+      </c>
+      <c r="G48" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfjyDwlnrARMtXAIKoDfFKeXOmdboY3BzLrniikGApFQctXqQ/viewform</v>
+      </c>
+      <c r="H48" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <v>48</v>
+      </c>
+      <c r="C49" t="str">
+        <v>EKO FAJAR KURNIAWAN, S.Pd</v>
+      </c>
+      <c r="D49" t="str">
+        <v>198212102022211017</v>
+      </c>
+      <c r="E49" t="str">
+        <v>-</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G49" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc0NlfwB6ZuoqiE6ScJiGrPeB-Qam31S7PDjICgFf5MPdIkiw/viewform</v>
+      </c>
+      <c r="H49" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <v>49</v>
+      </c>
+      <c r="C50" t="str">
+        <v>ETIK SULISTYOWATI, S.Pd.</v>
+      </c>
+      <c r="D50" t="str">
+        <v>198304282022212026</v>
+      </c>
+      <c r="E50" t="str">
+        <v>-</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G50" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdUwe7or4Y0G1-MxBUlVlO5CHIQU7My-9_OxXNA87sJhdXBZA/viewform</v>
+      </c>
+      <c r="H50" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>50</v>
+      </c>
+      <c r="C51" t="str">
+        <v>NOVAN EKO SETYAWAN, S.Kom.</v>
+      </c>
+      <c r="D51" t="str">
+        <v>198404192022211018</v>
+      </c>
+      <c r="E51" t="str">
+        <v>-</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G51" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe4vBzUIUsBJNN39klf82XO2jf2iJXqigXNdhNMkSI7-lcsEw/viewform</v>
+      </c>
+      <c r="H51" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52">
+        <v>51</v>
+      </c>
+      <c r="C52" t="str">
+        <v>YAYUK NURNANINGSIH, S.Pd</v>
+      </c>
+      <c r="D52" t="str">
+        <v>198607052022212052</v>
+      </c>
+      <c r="E52" t="str">
+        <v>-</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G52" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFgOYb82K7kj70lOwDL28zNyaVYlK3CX9WHttQtR-KGtb2Mg/viewform</v>
+      </c>
+      <c r="H52" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53">
+        <v>52</v>
+      </c>
+      <c r="C53" t="str">
+        <v>KHOIRUL AMIN, S.Pd</v>
+      </c>
+      <c r="D53" t="str">
+        <v>198701192022211009</v>
+      </c>
+      <c r="E53" t="str">
+        <v>-</v>
+      </c>
+      <c r="F53" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G53" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfm6LdDpeLyDCvK_EBRBQAFn2KZzRu1O2RcuNEeS-rXHm5ARQ/viewform</v>
+      </c>
+      <c r="H53" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54">
+        <v>53</v>
+      </c>
+      <c r="C54" t="str">
+        <v>REZA ZULKARNAIN ARIFIN, S.Pd.</v>
+      </c>
+      <c r="D54" t="str">
+        <v>198712072022211015</v>
+      </c>
+      <c r="E54" t="str">
+        <v>-</v>
+      </c>
+      <c r="F54" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G54" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdCbU4OVvmv8Y1juU-PWfd0aLqXc9SPgcVze8F8GqeYZXpYEw/viewform</v>
+      </c>
+      <c r="H54" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55">
+        <v>54</v>
+      </c>
+      <c r="C55" t="str">
+        <v>KHOIRUZEN, ST</v>
+      </c>
+      <c r="D55" t="str">
+        <v>197107222023211002</v>
+      </c>
+      <c r="E55" t="str">
+        <v>-</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G55" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
+      </c>
+      <c r="H55" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56">
+        <v>55</v>
+      </c>
+      <c r="C56" t="str">
+        <v>HEPPY LUCKITO, SST</v>
+      </c>
+      <c r="D56" t="str">
+        <v>198110272023211008</v>
+      </c>
+      <c r="E56" t="str">
+        <v>-</v>
+      </c>
+      <c r="F56" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G56" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfKzYb7Tb1GQICmf-UOYUp99-MdQogm7IRxd3BN88zTRcftmA/viewform</v>
+      </c>
+      <c r="H56" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57">
+        <v>56</v>
+      </c>
+      <c r="C57" t="str">
+        <v>SRI PURWANINGSIH, S.Pd</v>
+      </c>
+      <c r="D57" t="str">
+        <v>198203022023212020</v>
+      </c>
+      <c r="E57" t="str">
+        <v>-</v>
+      </c>
+      <c r="F57" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G57" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSciUprlTkbnMdDIkcOoeZN_KuWUcVafGVknPqPgIZNqrfjo-A/viewform</v>
+      </c>
+      <c r="H57" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58">
+        <v>57</v>
+      </c>
+      <c r="C58" t="str">
+        <v>DARIS UMAMI, S.Pd.</v>
+      </c>
+      <c r="D58" t="str">
+        <v>198205042023212026</v>
+      </c>
+      <c r="E58" t="str">
+        <v>-</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G58" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSety3ZkhI7AVI8v-VQRPaTax5rflclagowfHbFtFrNjSSZNHg/viewform</v>
+      </c>
+      <c r="H58" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59">
+        <v>58</v>
+      </c>
+      <c r="C59" t="str">
+        <v>AKHMAD ROFI SAFUAT, S.Pd.</v>
+      </c>
+      <c r="D59" t="str">
+        <v>198808072023211018</v>
+      </c>
+      <c r="E59" t="str">
+        <v>-</v>
+      </c>
+      <c r="F59" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G59" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScLoRQkJKESig6rf-hq4Hq-9UsA2rpsBuDhVX6113r1OrYeLw/viewform</v>
+      </c>
+      <c r="H59" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60">
+        <v>59</v>
+      </c>
+      <c r="C60" t="str">
+        <v>SIDHARTHA BUDI SUMEDHA, S.Pd</v>
+      </c>
+      <c r="D60" t="str">
+        <v>199410282023211012</v>
+      </c>
+      <c r="E60" t="str">
+        <v>-</v>
+      </c>
+      <c r="F60" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G60" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeyOibEzsSXoKuudKE99ynaPyji9xnu894iTgezdD34JzKmJg/viewform</v>
+      </c>
+      <c r="H60" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61">
+        <v>60</v>
+      </c>
+      <c r="C61" t="str">
+        <v>ASYITAH  ALMUFIDAH, S.Pd</v>
+      </c>
+      <c r="D61" t="str">
+        <v>199606142023212026</v>
+      </c>
+      <c r="E61" t="str">
+        <v>-</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G61" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeBM6FY62A84yCrWK-O8XZ_ehP9cDsy6qNu0MHDEXeCZlsATA/viewform</v>
+      </c>
+      <c r="H61" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62">
+        <v>61</v>
+      </c>
+      <c r="C62" t="str">
+        <v>SUDARMONO, ST</v>
+      </c>
+      <c r="D62" t="str">
+        <v>197206202024211005</v>
+      </c>
+      <c r="E62" t="str">
+        <v>-</v>
+      </c>
+      <c r="F62" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G62" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGR9KnW2FGcWAVjUfLzEpLkENkH6O1XpstPv9041fsBK4r7A/viewform</v>
+      </c>
+      <c r="H62" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63">
+        <v>62</v>
+      </c>
+      <c r="C63" t="str">
+        <v>ROHMAN, S.T.</v>
+      </c>
+      <c r="D63" t="str">
+        <v>197509042024211002</v>
+      </c>
+      <c r="E63" t="str">
+        <v>-</v>
+      </c>
+      <c r="F63" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G63" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScGZ84pyS-MstOKQkNP2TD0SMihbvT1G-Gm-XPV_V8SfOGKuQ/viewform</v>
+      </c>
+      <c r="H63" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64">
+        <v>63</v>
+      </c>
+      <c r="C64" t="str">
+        <v>ANDRI YUDHI PRASETYO, ST</v>
+      </c>
+      <c r="D64" t="str">
+        <v>197907232024211002</v>
+      </c>
+      <c r="E64" t="str">
+        <v>-</v>
+      </c>
+      <c r="F64" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G64" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4F9PoN3h1R3EmQmS-KTPCmUB2ghq3K7N1e00Ni4NE30hESw/viewform</v>
+      </c>
+      <c r="H64" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65">
+        <v>64</v>
+      </c>
+      <c r="C65" t="str">
+        <v>MIANTO, S.Kom.</v>
+      </c>
+      <c r="D65" t="str">
+        <v>198005222024211005</v>
+      </c>
+      <c r="E65" t="str">
+        <v>-</v>
+      </c>
+      <c r="F65" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G65" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSee6t_4PgxzeHNbhtwqZROlfNE9Iz6Sf5QJvGMjzkmAGvhcAw/viewform</v>
+      </c>
+      <c r="H65" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66">
+        <v>65</v>
+      </c>
+      <c r="C66" t="str">
+        <v>HARIS ALI MUHYIDIN, S.T</v>
+      </c>
+      <c r="D66" t="str">
+        <v>198103052024211008</v>
+      </c>
+      <c r="E66" t="str">
+        <v>-</v>
+      </c>
+      <c r="F66" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G66" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSePrT6SB-ho1Qu-8X9Msnl2pHSrhkeXp3sh_m5NJQBt1K2-LA/viewform</v>
+      </c>
+      <c r="H66" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67">
+        <v>66</v>
+      </c>
+      <c r="C67" t="str">
+        <v>MAMIEK ZUHRIYAH. S.Hum</v>
+      </c>
+      <c r="D67" t="str">
+        <v>198112142024212008</v>
+      </c>
+      <c r="E67" t="str">
+        <v>-</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G67" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf_FdCdD6ohlhQX_f3H7SVBGc4nrC2Ui3-rcrQZRPNnltfamQ/viewform</v>
+      </c>
+      <c r="H67" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68">
+        <v>67</v>
+      </c>
+      <c r="C68" t="str">
+        <v>UMI RU'YATIN, S.Pd</v>
+      </c>
+      <c r="D68" t="str">
+        <v>198201062024212001</v>
+      </c>
+      <c r="E68" t="str">
+        <v>-</v>
+      </c>
+      <c r="F68" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G68" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfnkOblKHmHEQZv7mSD1vVCZo9F05r9j_4cB8Gf13YpClrBEA/viewform</v>
+      </c>
+      <c r="H68" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69">
+        <v>68</v>
+      </c>
+      <c r="C69" t="str">
+        <v>YEFI WULANDARI, SE</v>
+      </c>
+      <c r="D69" t="str">
+        <v>198204272024212014</v>
+      </c>
+      <c r="E69" t="str">
+        <v>-</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G69" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdWSaS-TIna_zsswr8VBL4h5etsBLiiX8g9DDJoMFMbqcqRaQ/viewform</v>
+      </c>
+      <c r="H69" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70">
+        <v>69</v>
+      </c>
+      <c r="C70" t="str">
+        <v>SARI NURHIDAYATI, S.Pd.</v>
+      </c>
+      <c r="D70" t="str">
+        <v>198209202024212008</v>
+      </c>
+      <c r="E70" t="str">
+        <v>-</v>
+      </c>
+      <c r="F70" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G70" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdEXPOLI2_EBQt6mzHWAdm2mEw2qMyBnYwO7RHZF7l_PG5XoQ/viewform</v>
+      </c>
+      <c r="H70" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71">
+        <v>70</v>
+      </c>
+      <c r="C71" t="str">
+        <v>SUWOYO, S.Kom</v>
+      </c>
+      <c r="D71" t="str">
+        <v>198403072024211011</v>
+      </c>
+      <c r="E71" t="str">
+        <v>-</v>
+      </c>
+      <c r="F71" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G71" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdu7xAgcP3EduN8K2GQ4TgkUqHBOYkmDQCI07RKwj8csn0P3A/viewform</v>
+      </c>
+      <c r="H71" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72">
+        <v>71</v>
+      </c>
+      <c r="C72" t="str">
+        <v>AAN SUSANTO, S.Pd.</v>
+      </c>
+      <c r="D72" t="str">
+        <v>198410082024211016</v>
+      </c>
+      <c r="E72" t="str">
+        <v>-</v>
+      </c>
+      <c r="F72" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G72" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNvGrFaOMlKRAFM-pU2Ri99i0wMsYyrBzlaPhRWrx3v3F_rw/viewform</v>
+      </c>
+      <c r="H72" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73">
+        <v>72</v>
+      </c>
+      <c r="C73" t="str">
+        <v>YUNITA DWI WIRANTI, S.Pd</v>
+      </c>
+      <c r="D73" t="str">
+        <v>198606052024212013</v>
+      </c>
+      <c r="E73" t="str">
+        <v>-</v>
+      </c>
+      <c r="F73" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G73" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeqYfnPkvY4AdwC8V4UHvNEndqvqZuSZZj_2LqzOVCpFLaKXg/viewform</v>
+      </c>
+      <c r="H73" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74">
+        <v>73</v>
+      </c>
+      <c r="C74" t="str">
+        <v>NUR FAUZIYAH, S.Ag.</v>
+      </c>
+      <c r="D74" t="str">
+        <v>197411202025212006</v>
+      </c>
+      <c r="E74" t="str">
+        <v>-</v>
+      </c>
+      <c r="F74" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G74" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfv3nzKCScYWg6AFek-3gvT8RkTVVgcld3sF3LPxXMO0ST9fA/viewform</v>
+      </c>
+      <c r="H74" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75">
+        <v>74</v>
+      </c>
+      <c r="C75" t="str">
+        <v>SUYANTI, S.Kom.</v>
+      </c>
+      <c r="D75" t="str">
+        <v>198206012025212027</v>
+      </c>
+      <c r="E75" t="str">
+        <v>-</v>
+      </c>
+      <c r="F75" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G75" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf9LjiU4ww9Pt_xAA8_SHzsqfA3_tENCX11_lJEl64I8BOmrw/viewform</v>
+      </c>
+      <c r="H75" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76">
+        <v>75</v>
+      </c>
+      <c r="C76" t="str">
+        <v>DELIA NURUL AFIFAH, S.Pd</v>
+      </c>
+      <c r="D76" t="str">
+        <v>-</v>
+      </c>
+      <c r="E76" t="str">
+        <v>-</v>
+      </c>
+      <c r="F76" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G76" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdSOrQUklEFC17Wn9lGEgECqp4VP7B7A76ywjj7aydH8lBisA/viewform</v>
+      </c>
+      <c r="H76" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77">
+        <v>76</v>
+      </c>
+      <c r="C77" t="str">
+        <v>CAHYA ISKANDAR, S.T</v>
+      </c>
+      <c r="D77" t="str">
+        <v>-</v>
+      </c>
+      <c r="E77" t="str">
+        <v>-</v>
+      </c>
+      <c r="F77" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G77" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdI0DpURY4PnMrrxOZrTgYpoNM0Oi8z0kdkriti50-5Jcc8AA/viewform</v>
+      </c>
+      <c r="H77" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78">
+        <v>77</v>
+      </c>
+      <c r="C78" t="str">
+        <v>EVY KUSHARDIANY, S.Pd</v>
+      </c>
+      <c r="D78" t="str">
+        <v>-</v>
+      </c>
+      <c r="E78" t="str">
+        <v>-</v>
+      </c>
+      <c r="F78" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G78" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe-iUqyVQtHbDMTfC_7ufj97I7ZUaQqm6A5AEb35wPuyyYjtw/viewform</v>
+      </c>
+      <c r="H78" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79">
+        <v>78</v>
+      </c>
+      <c r="C79" t="str">
+        <v>HUDAN RHARA ANGGRIADI, S.Pd</v>
+      </c>
+      <c r="D79" t="str">
+        <v>-</v>
+      </c>
+      <c r="E79" t="str">
+        <v>-</v>
+      </c>
+      <c r="F79" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G79" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGiZq5Z_NRQ4BnCeDf3KwvRCPJp5pdbJ6d-IWHzLuQ_JTzLw/viewform</v>
+      </c>
+      <c r="H79" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80">
+        <v>79</v>
+      </c>
+      <c r="C80" t="str">
+        <v>YUNIAR DWI LISTYANTO, ST</v>
+      </c>
+      <c r="D80" t="str">
+        <v>-</v>
+      </c>
+      <c r="E80" t="str">
+        <v>-</v>
+      </c>
+      <c r="F80" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G80" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfObp6dU2YLs8UnHrzFalutFKBR7jcQHfriWJ_eL89rfsp4yA/viewform</v>
+      </c>
+      <c r="H80" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81">
+        <v>80</v>
+      </c>
+      <c r="C81" t="str">
+        <v>BENY WIJAYANTO, SS</v>
+      </c>
+      <c r="D81" t="str">
+        <v>-</v>
+      </c>
+      <c r="E81" t="str">
+        <v>-</v>
+      </c>
+      <c r="F81" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G81" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdoJpvoEo84fRoDbBiej0XGRlAW9_Ws8hrrM4HYvg1UuY08-A/viewform</v>
+      </c>
+      <c r="H81" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82">
+        <v>81</v>
+      </c>
+      <c r="C82" t="str">
+        <v>NURUL JAMILAH, S.Hum.</v>
+      </c>
+      <c r="D82" t="str">
+        <v>-</v>
+      </c>
+      <c r="E82" t="str">
+        <v>-</v>
+      </c>
+      <c r="F82" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G82" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdvb6XVfWMHXObfg9Qt1qHVFJG91UMNtxkOVmOl8rIiMWyflw/viewform</v>
+      </c>
+      <c r="H82" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83">
+        <v>82</v>
+      </c>
+      <c r="C83" t="str">
+        <v>ENDANG MULYANI, S.Pd.</v>
+      </c>
+      <c r="D83" t="str">
+        <v>-</v>
+      </c>
+      <c r="E83" t="str">
+        <v>-</v>
+      </c>
+      <c r="F83" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G83" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfIKb0_RA5kQm53YRXY6XxgtyTJnWLyMt8rbszzAxQM5OVfcw/viewform</v>
+      </c>
+      <c r="H83" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84">
+        <v>83</v>
+      </c>
+      <c r="C84" t="str">
+        <v>AGUS IRIANTO, S.Pd</v>
+      </c>
+      <c r="D84" t="str">
+        <v>-</v>
+      </c>
+      <c r="E84" t="str">
+        <v>-</v>
+      </c>
+      <c r="F84" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G84" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdVc_vPbnRafJ0MFj_iMwBjMvcx-SWamCBstx-Zx0eEWJWpow/viewform</v>
+      </c>
+      <c r="H84" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85">
+        <v>84</v>
+      </c>
+      <c r="C85" t="str">
+        <v>SAMUJI, S.Ag</v>
+      </c>
+      <c r="D85" t="str">
+        <v>-</v>
+      </c>
+      <c r="E85" t="str">
+        <v>-</v>
+      </c>
+      <c r="F85" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G85" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeH_z8k1zjOPd5-ALKEBIwAwnlGEYxrGSwIvU53bPzn4pVj5w/viewform</v>
+      </c>
+      <c r="H85" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86">
+        <v>85</v>
+      </c>
+      <c r="C86" t="str">
+        <v>IKA UMAYA MARDIANA, S.Pd</v>
+      </c>
+      <c r="D86" t="str">
+        <v>-</v>
+      </c>
+      <c r="E86" t="str">
+        <v>-</v>
+      </c>
+      <c r="F86" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G86" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdvQigaXQYmjPnCMU-VOYwFW7tL_wdiEQWFrrEHjwgPUriWVQ/viewform</v>
+      </c>
+      <c r="H86" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87">
+        <v>86</v>
+      </c>
+      <c r="C87" t="str">
+        <v>NUR KHOLIFAH, S.Pd.</v>
+      </c>
+      <c r="D87" t="str">
+        <v>-</v>
+      </c>
+      <c r="E87" t="str">
+        <v>-</v>
+      </c>
+      <c r="F87" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G87" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfbc-fqTUiN-W3eGoJx6clkQZ0gJmQ33llKL0DkrWqSw_-cXA/viewform</v>
+      </c>
+      <c r="H87" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88">
+        <v>87</v>
+      </c>
+      <c r="C88" t="str">
+        <v>AIDA QONITATILLAH, S.Pd</v>
+      </c>
+      <c r="D88" t="str">
+        <v>-</v>
+      </c>
+      <c r="E88" t="str">
+        <v>-</v>
+      </c>
+      <c r="F88" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G88" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScO5dWuDM9bbQPPRFU7wj2KYpndQWl6MjW4aeBRmp2gd1zsIg/viewform</v>
+      </c>
+      <c r="H88" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89">
+        <v>88</v>
+      </c>
+      <c r="C89" t="str">
+        <v>YULI ANDRIYANI,  S.Pd</v>
+      </c>
+      <c r="D89" t="str">
+        <v>-</v>
+      </c>
+      <c r="E89" t="str">
+        <v>-</v>
+      </c>
+      <c r="F89" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G89" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSetc4dTjz3vYbJvKTJp6Fev2T1Omw8up-uaiqGjN911bM5VhQ/viewform</v>
+      </c>
+      <c r="H89" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90">
+        <v>89</v>
+      </c>
+      <c r="C90" t="str">
+        <v>VITA EKA RAHAYU, S.Pd</v>
+      </c>
+      <c r="D90" t="str">
+        <v>-</v>
+      </c>
+      <c r="E90" t="str">
+        <v>-</v>
+      </c>
+      <c r="F90" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G90" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSegF6rlZWgN9LSLJ-b_0D-Q5rIwzgMKjDZb7njyjkb9m175Cw/viewform</v>
+      </c>
+      <c r="H90" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91">
         <v>90</v>
       </c>
-      <c r="C41" t="str">
+      <c r="B91">
+        <v>90</v>
+      </c>
+      <c r="C91" t="str">
         <v>AKHMAD VICKRI HIDAYATULLAH, S.Pd</v>
       </c>
-      <c r="D41" t="str">
-        <v>-</v>
-      </c>
-      <c r="E41" t="str">
-        <v>-</v>
-      </c>
-      <c r="F41" t="str">
-        <v>Guru Pengajar</v>
-      </c>
-      <c r="G41" t="str">
+      <c r="D91" t="str">
+        <v>-</v>
+      </c>
+      <c r="E91" t="str">
+        <v>-</v>
+      </c>
+      <c r="F91" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G91" t="str">
         <v>https://docs.google.com/forms/d/e/1FAIpQLScsaQccrJrLWyFuELeJUY_dlYER0px-lNCoStikizRhMTHllQ/viewform</v>
       </c>
-      <c r="H41" t="str">
+      <c r="H91" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92">
+        <v>91</v>
+      </c>
+      <c r="C92" t="str">
+        <v>HERI SUGIANTORO, S.Ag</v>
+      </c>
+      <c r="D92" t="str">
+        <v>-</v>
+      </c>
+      <c r="E92" t="str">
+        <v>-</v>
+      </c>
+      <c r="F92" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G92" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc8hB1Jne1cZcXsMyyah9zkwsD-5XKk5o91E4fXfHBFtfeheg/viewform</v>
+      </c>
+      <c r="H92" t="str">
+        <v>✅ Valid &amp; Siap Autofill</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93">
+        <v>92</v>
+      </c>
+      <c r="C93" t="str">
+        <v>AKBAR ILHAM BAGASKARA PRATAMA, S.T</v>
+      </c>
+      <c r="D93" t="str">
+        <v>-</v>
+      </c>
+      <c r="E93" t="str">
+        <v>-</v>
+      </c>
+      <c r="F93" t="str">
+        <v>Guru Pengajar</v>
+      </c>
+      <c r="G93" t="str">
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe9TyB66OIRNYnCfIgvtMfcDfVMgbJpD-JByezy7I4Gp20-Bw/viewform</v>
+      </c>
+      <c r="H93" t="str">
         <v>✅ Valid &amp; Siap Autofill</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H93"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3165,13 +2990,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G4" t="str">
-        <v>https://forms.gle/ekQJWbDbi72DSNHX9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSez4gjTar2bPbopGm6ErVaBlugek0rGtLocS5azfCCp0MDSIA/viewform</v>
       </c>
       <c r="H4" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I4" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="5">
@@ -3252,13 +3077,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G7" t="str">
-        <v>https://forms.gle/FzjMqjr2bhYB4mFGA</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfb21fBd9nBHkgM2MBTbSNxfeTgWiXbFL43E9QIZX-zGLzq0g/viewform</v>
       </c>
       <c r="H7" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I7" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="8">
@@ -3310,13 +3135,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G9" t="str">
-        <v>https://forms.gle/hpaJmjc4TSuY21187</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe-IzLFr71Gdhgd06mjpg2ToTRv1yEa_u8WYc9JsSpikG-NuA/viewform</v>
       </c>
       <c r="H9" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I9" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="10">
@@ -3339,13 +3164,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G10" t="str">
-        <v>https://forms.gle/zCXw2UY7hgtbguuc6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf3zl2VpfYKhir9CPBloLYg_xU95VEOzo28tGm9RxY8hWf_8Q/viewform</v>
       </c>
       <c r="H10" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I10" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="11">
@@ -3368,13 +3193,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G11" t="str">
-        <v>https://forms.gle/8SMDhw8YpsNPPHPK7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdEgJQrGVluy9utuyyeyZ7psIgxX5H9-OTYUG63if-14TLXNg/viewform</v>
       </c>
       <c r="H11" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I11" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="12">
@@ -3397,13 +3222,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G12" t="str">
-        <v>https://forms.gle/sZ2Rff4sL9N4FTrh9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeYIRHhpNjh1FmGBMMlPQPwu6jnRfYLe__qCNtcIES7ZefQvQ/viewform</v>
       </c>
       <c r="H12" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I12" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="13">
@@ -3542,13 +3367,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G17" t="str">
-        <v>https://forms.gle/ghNaoJYp7o2SbkjS8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdYaU-G7gAyHPvwtYTw67xI_BcR43imBjiP3RB58jOjnU1XeQ/viewform</v>
       </c>
       <c r="H17" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I17" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="18">
@@ -3571,13 +3396,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G18" t="str">
-        <v>https://forms.gle/bPxWzjgFDES2StGo6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSd2bLbWa9Pca9QT7JTzZAnSSDZOakUabHJxB_JnNT3CQEv4gA/viewform</v>
       </c>
       <c r="H18" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I18" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="19">
@@ -3629,13 +3454,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G20" t="str">
-        <v>https://forms.gle/aaS7YNQQ97713C18A</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSd4Etrlv7kK9gUfKVu1OwwyBhjLAn4-l3PArWhzLxF13MmmVw/viewform</v>
       </c>
       <c r="H20" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I20" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="21">
@@ -3658,13 +3483,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G21" t="str">
-        <v>https://forms.gle/6YPzECievjrGJZBnA</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScZ2l8R4TTNeJdfXVZvYAgc3WGgT9QtEVz0-ANUsebuRgsWsQ/viewform</v>
       </c>
       <c r="H21" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I21" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="22">
@@ -3687,13 +3512,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G22" t="str">
-        <v>https://forms.gle/2mog9vghqCw6TSTw7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdcvHzA1p4OhUC9iXA97o8okqRsjziPMeWoPw6g-Nvt7Pr9jg/viewform</v>
       </c>
       <c r="H22" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I22" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="23">
@@ -3774,13 +3599,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G25" t="str">
-        <v>https://forms.gle/DSDoMKgI8XxbcPr78</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdoHRTHs-yCXOAaQukleNcx5jWI79dOK6qbeeCW4p45bJ9CLg/viewform</v>
       </c>
       <c r="H25" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I25" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="26">
@@ -3803,13 +3628,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G26" t="str">
-        <v>https://forms.gle/jVwhLYXebas1GSZQJ6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSftHQdc5-VZ5uwLLimFvRnkwycT7Ys50sjgRzMN-ALHGSjCqA/viewform</v>
       </c>
       <c r="H26" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I26" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="27">
@@ -3861,13 +3686,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G28" t="str">
-        <v>https://forms.gle/r3mekFxufrTcJjgRA</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfNEYg6DAPuUemLNfKalqh5_nN6m2oxlOxSvPG1Fu55a4gqNA/viewform</v>
       </c>
       <c r="H28" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I28" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="29">
@@ -3977,13 +3802,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G32" t="str">
-        <v>https://forms.gle/PSXtPwi7yQN3Mfi8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdRlmK9kl1qIAOcGpf1Uu18upIQ0GWK8VkTv12k_6AEAERRMQ/viewform</v>
       </c>
       <c r="H32" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I32" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="33">
@@ -4035,13 +3860,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G34" t="str">
-        <v>https://forms.gle/ESlazXu6aQ3PklsD9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdPW1l4LaclpGdRqS2jqaCtnP9mivQff9TM2a9if71auoCj6g/viewform</v>
       </c>
       <c r="H34" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I34" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="35">
@@ -4064,13 +3889,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G35" t="str">
-        <v>https://forms.gle/KwfitQjMYbtsnr4UZV6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSejtfmzSD3f24E8Z4AXVPgC0RTs8brRuZ_KCxV9-lmsq4C5iQ/viewform</v>
       </c>
       <c r="H35" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I35" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="36">
@@ -4093,13 +3918,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G36" t="str">
-        <v>https://forms.gle/DStwfQQGe3W3gc73A</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdaT-LhGEwSzPtm9G3LL6KRs-gFmbNF2uiIykR7J7HDmdC2uQ/viewform</v>
       </c>
       <c r="H36" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I36" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="37">
@@ -4122,13 +3947,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G37" t="str">
-        <v>https://forms.gle/8Z33XXUnWmhZCY9S9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdFjcTg73409mYsq9RTVwH8IBBBz5ya0_y6K1t74WjfpPWMhA/viewform</v>
       </c>
       <c r="H37" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I37" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="38">
@@ -4180,13 +4005,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G39" t="str">
-        <v>https://forms.gle/iGQNqJij1huPUYbk8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScUo8DXP3Tp38IveX-Bq5eu4aD3aJBRVAjTA8896rGx1WUsNQ/viewform</v>
       </c>
       <c r="H39" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I39" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="40">
@@ -4209,13 +4034,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G40" t="str">
-        <v>https://forms.gle/RvBNnww2vjNe3gNo76</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScKk6RYj6qkwSYwir5SH2zma20b5qhM4boLx8UqeQ19DUTIfA/viewform</v>
       </c>
       <c r="H40" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I40" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="41">
@@ -4238,13 +4063,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G41" t="str">
-        <v>https://forms.gle/eSTVKcrx2NqqFGR28</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSczNF2YAQXf9165kZ-FthvzailwmMrM-uSTecJzWHq0JCEldQ/viewform</v>
       </c>
       <c r="H41" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I41" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="42">
@@ -4296,13 +4121,13 @@
         <v>Walikelas</v>
       </c>
       <c r="G43" t="str">
-        <v>https://forms.gle/wtPkKSjFyF5RRwop8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4Z31ED-5m9YP8u3CbOt0PWt94nwzJafZSig17a3DoqRlpCQ/viewform</v>
       </c>
       <c r="H43" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I43" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="44">
@@ -4499,13 +4324,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G50" t="str">
-        <v>https://forms.gle/U9F3SKAciwAgqt8S6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdUwe7or4Y0G1-MxBUlVlO5CHIQU7My-9_OxXNA87sJhdXBZA/viewform</v>
       </c>
       <c r="H50" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I50" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="51">
@@ -4528,13 +4353,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G51" t="str">
-        <v>https://forms.gle/5ukkAKPa1f6AFkZc7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe4vBzUIUsBJNN39klf82XO2jf2iJXqigXNdhNMkSI7-lcsEw/viewform</v>
       </c>
       <c r="H51" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I51" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="52">
@@ -4557,13 +4382,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G52" t="str">
-        <v>https://forms.gle/55GCWMt4rvFq8Tpl9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfFgOYb82K7kj70lOwDL28zNyaVYlK3CX9WHttQtR-KGtb2Mg/viewform</v>
       </c>
       <c r="H52" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I52" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="53">
@@ -4644,13 +4469,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G55" t="str">
-        <v>https://forms.gle/ZNeYDpDbGFZanGsy9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSch1k6AMaxaF6RHrG1J7kyOQfurlM7pv6Zfg2K8H3X94whrPA/viewform</v>
       </c>
       <c r="H55" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I55" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="56">
@@ -4731,13 +4556,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G58" t="str">
-        <v>https://forms.gle/JSRwHajfSJNBKxr9</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSety3ZkhI7AVI8v-VQRPaTax5rflclagowfHbFtFrNjSSZNHg/viewform</v>
       </c>
       <c r="H58" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I58" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="59">
@@ -4760,13 +4585,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G59" t="str">
-        <v>https://forms.gle/wDAYP8evmdZCEvHr7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScLoRQkJKESig6rf-hq4Hq-9UsA2rpsBuDhVX6113r1OrYeLw/viewform</v>
       </c>
       <c r="H59" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I59" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="60">
@@ -4818,13 +4643,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G61" t="str">
-        <v>https://forms.gle/byFX3UbYfSVMGRUx5</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeBM6FY62A84yCrWK-O8XZ_ehP9cDsy6qNu0MHDEXeCZlsATA/viewform</v>
       </c>
       <c r="H61" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I61" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="62">
@@ -4847,13 +4672,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G62" t="str">
-        <v>https://forms.gle/1DCZSoKurcAwXyia8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdGR9KnW2FGcWAVjUfLzEpLkENkH6O1XpstPv9041fsBK4r7A/viewform</v>
       </c>
       <c r="H62" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I62" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="63">
@@ -4905,13 +4730,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G64" t="str">
-        <v>https://forms.gle/z5unoXhPisrFHYQe6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf4F9PoN3h1R3EmQmS-KTPCmUB2ghq3K7N1e00Ni4NE30hESw/viewform</v>
       </c>
       <c r="H64" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I64" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="65">
@@ -4934,13 +4759,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G65" t="str">
-        <v>https://forms.gle/St3Fvko6Q8Rk5P1N6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSee6t_4PgxzeHNbhtwqZROlfNE9Iz6Sf5QJvGMjzkmAGvhcAw/viewform</v>
       </c>
       <c r="H65" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I65" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="66">
@@ -4992,13 +4817,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G67" t="str">
-        <v>https://forms.gle/6SoaEmuGWvds11M57</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf_FdCdD6ohlhQX_f3H7SVBGc4nrC2Ui3-rcrQZRPNnltfamQ/viewform</v>
       </c>
       <c r="H67" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I67" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="68">
@@ -5021,13 +4846,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G68" t="str">
-        <v>https://forms.gle/f1Bak224cs2fbQWv6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfnkOblKHmHEQZv7mSD1vVCZo9F05r9j_4cB8Gf13YpClrBEA/viewform</v>
       </c>
       <c r="H68" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I68" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="69">
@@ -5050,13 +4875,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G69" t="str">
-        <v>https://forms.gle/uRdDxC8DuaGwexXS6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdWSaS-TIna_zsswr8VBL4h5etsBLiiX8g9DDJoMFMbqcqRaQ/viewform</v>
       </c>
       <c r="H69" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I69" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="70">
@@ -5079,13 +4904,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G70" t="str">
-        <v>https://forms.gle/RinuqtFA6SvqSL1k8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdEXPOLI2_EBQt6mzHWAdm2mEw2qMyBnYwO7RHZF7l_PG5XoQ/viewform</v>
       </c>
       <c r="H70" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I70" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="71">
@@ -5166,13 +4991,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G73" t="str">
-        <v>https://forms.gle/pcpQzaMSk9Stp7cg7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeqYfnPkvY4AdwC8V4UHvNEndqvqZuSZZj_2LqzOVCpFLaKXg/viewform</v>
       </c>
       <c r="H73" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I73" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="74">
@@ -5224,13 +5049,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G75" t="str">
-        <v>https://forms.gle/fgP9YYo9hxHuTtXj6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSf9LjiU4ww9Pt_xAA8_SHzsqfA3_tENCX11_lJEl64I8BOmrw/viewform</v>
       </c>
       <c r="H75" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I75" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="76">
@@ -5253,13 +5078,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G76" t="str">
-        <v>https://forms.gle/DyU5ZXtraYh9wYc29</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdSOrQUklEFC17Wn9lGEgECqp4VP7B7A76ywjj7aydH8lBisA/viewform</v>
       </c>
       <c r="H76" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I76" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="77">
@@ -5311,13 +5136,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G78" t="str">
-        <v>https://forms.gle/5VYu1RujWovmBBU3A</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe-iUqyVQtHbDMTfC_7ufj97I7ZUaQqm6A5AEb35wPuyyYjtw/viewform</v>
       </c>
       <c r="H78" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I78" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="79">
@@ -5398,13 +5223,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G81" t="str">
-        <v>https://forms.gle/2d2erB3kRKMkYt7U7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdoJpvoEo84fRoDbBiej0XGRlAW9_Ws8hrrM4HYvg1UuY08-A/viewform</v>
       </c>
       <c r="H81" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I81" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="82">
@@ -5427,13 +5252,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G82" t="str">
-        <v>https://forms.gle/wsT14LzF1YIGLA4f6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdvb6XVfWMHXObfg9Qt1qHVFJG91UMNtxkOVmOl8rIiMWyflw/viewform</v>
       </c>
       <c r="H82" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I82" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="83">
@@ -5456,13 +5281,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G83" t="str">
-        <v>https://forms.gle/Auiix31BCC39d3827</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSfIKb0_RA5kQm53YRXY6XxgtyTJnWLyMt8rbszzAxQM5OVfcw/viewform</v>
       </c>
       <c r="H83" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I83" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="84">
@@ -5485,13 +5310,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G84" t="str">
-        <v>https://forms.gle/9ox7839w57zhmph37</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdVc_vPbnRafJ0MFj_iMwBjMvcx-SWamCBstx-Zx0eEWJWpow/viewform</v>
       </c>
       <c r="H84" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I84" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="85">
@@ -5514,13 +5339,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G85" t="str">
-        <v>https://forms.gle/xaxakR9EjF5QRACyv8</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSeH_z8k1zjOPd5-ALKEBIwAwnlGEYxrGSwIvU53bPzn4pVj5w/viewform</v>
       </c>
       <c r="H85" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I85" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="86">
@@ -5543,13 +5368,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G86" t="str">
-        <v>https://forms.gle/FdBUf1m2wrFUJUXW7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSdvQigaXQYmjPnCMU-VOYwFW7tL_wdiEQWFrrEHjwgPUriWVQ/viewform</v>
       </c>
       <c r="H86" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I86" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="87">
@@ -5601,13 +5426,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G88" t="str">
-        <v>https://forms.gle/iTp6ejZeufb9GjdD6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLScO5dWuDM9bbQPPRFU7wj2KYpndQWl6MjW4aeBRmp2gd1zsIg/viewform</v>
       </c>
       <c r="H88" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I88" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="89">
@@ -5630,13 +5455,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G89" t="str">
-        <v>https://forms.gle/zNoEfcKBWk4cLrSw6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSetc4dTjz3vYbJvKTJp6Fev2T1Omw8up-uaiqGjN911bM5VhQ/viewform</v>
       </c>
       <c r="H89" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I89" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="90">
@@ -5659,13 +5484,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G90" t="str">
-        <v>https://forms.gle/w4dULz23fLn5t2FS6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSegF6rlZWgN9LSLJ-b_0D-Q5rIwzgMKjDZb7njyjkb9m175Cw/viewform</v>
       </c>
       <c r="H90" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I90" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="91">
@@ -5717,13 +5542,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G92" t="str">
-        <v>https://forms.gle/FP6TDKV278Clj95X7</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSc8hB1Jne1cZcXsMyyah9zkwsD-5XKk5o91E4fXfHBFtfeheg/viewform</v>
       </c>
       <c r="H92" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I92" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
     <row r="93">
@@ -5746,13 +5571,13 @@
         <v>Guru Pengajar</v>
       </c>
       <c r="G93" t="str">
-        <v>https://forms.gle/ECwx7SMeMMkf7RfN6</v>
+        <v>https://docs.google.com/forms/d/e/1FAIpQLSe9TyB66OIRNYnCfIgvtMfcDfVMgbJpD-JByezy7I4Gp20-Bw/viewform</v>
       </c>
       <c r="H93" t="str">
-        <v>Shortlink (forms.gle)</v>
+        <v>Long URL (Canonical)</v>
       </c>
       <c r="I93" t="str">
-        <v>🟡 Menggunakan Fallback Form Induk</v>
+        <v>✅ Langsung Siap Autofill</v>
       </c>
     </row>
   </sheetData>

</xml_diff>